<commit_message>
feat(grafico-planilha): inverte a ordem e as coordenadas de Obturado e Perdido mantendo as cores e o padrão C-O-P
</commit_message>
<xml_diff>
--- a/app/assets/planilhas/teethgram_en.xlsx
+++ b/app/assets/planilhas/teethgram_en.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DEV Workspace\projetos-profissionais\teethGram\app\assets\planilhas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\almei\dev\teethGram\app\assets\planilhas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34173F18-15A4-41A8-A2B5-721002CB9B30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{071AEE10-5C9E-46EF-807F-451296B52ACC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{AFFBEBE6-A6BC-498C-A820-BBF450B005CB}"/>
   </bookViews>
@@ -56,7 +56,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A6" authorId="0" shapeId="0" xr:uid="{A4DD2828-35E0-4A5F-9196-F4E1CED96808}">
+    <comment ref="A6" authorId="0" shapeId="0" xr:uid="{2E440F82-1ED1-4C0A-8C89-CAC623CBBD31}">
       <text>
         <r>
           <rPr>
@@ -70,7 +70,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A7" authorId="0" shapeId="0" xr:uid="{2E440F82-1ED1-4C0A-8C89-CAC623CBBD31}">
+    <comment ref="A7" authorId="0" shapeId="0" xr:uid="{A4DD2828-35E0-4A5F-9196-F4E1CED96808}">
       <text>
         <r>
           <rPr>
@@ -111,7 +111,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A13" authorId="0" shapeId="0" xr:uid="{7354F24A-D9B6-400C-9B5C-7188D1761EE6}">
+    <comment ref="A13" authorId="0" shapeId="0" xr:uid="{5C01E885-706E-4DD4-8899-0996FA7C1E83}">
       <text>
         <r>
           <rPr>
@@ -125,7 +125,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A14" authorId="0" shapeId="0" xr:uid="{5C01E885-706E-4DD4-8899-0996FA7C1E83}">
+    <comment ref="A14" authorId="0" shapeId="0" xr:uid="{7354F24A-D9B6-400C-9B5C-7188D1761EE6}">
       <text>
         <r>
           <rPr>
@@ -166,7 +166,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A22" authorId="0" shapeId="0" xr:uid="{AEDD797E-6029-49AB-B684-18BCF2D7ABA1}">
+    <comment ref="A22" authorId="0" shapeId="0" xr:uid="{8D07286F-8727-4357-9417-A22B0C5C0E9E}">
       <text>
         <r>
           <rPr>
@@ -180,7 +180,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A23" authorId="0" shapeId="0" xr:uid="{8D07286F-8727-4357-9417-A22B0C5C0E9E}">
+    <comment ref="A23" authorId="0" shapeId="0" xr:uid="{AEDD797E-6029-49AB-B684-18BCF2D7ABA1}">
       <text>
         <r>
           <rPr>
@@ -221,7 +221,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A29" authorId="0" shapeId="0" xr:uid="{65F162A7-3776-48D5-AF6F-F6BBAD7337E5}">
+    <comment ref="A29" authorId="0" shapeId="0" xr:uid="{EAE70C67-A158-42EA-81E3-7ED4E2D2B0F6}">
       <text>
         <r>
           <rPr>
@@ -235,7 +235,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A30" authorId="0" shapeId="0" xr:uid="{EAE70C67-A158-42EA-81E3-7ED4E2D2B0F6}">
+    <comment ref="A30" authorId="0" shapeId="0" xr:uid="{65F162A7-3776-48D5-AF6F-F6BBAD7337E5}">
       <text>
         <r>
           <rPr>
@@ -381,7 +381,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -418,6 +418,14 @@
       <color indexed="81"/>
       <name val="Segoe UI"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="15">
@@ -780,7 +788,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -870,6 +878,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1209,7 +1218,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91CAF953-5A63-4D25-9285-6A1D6422454A}">
-  <dimension ref="A1:AG34"/>
+  <dimension ref="A1:AG40"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.28515625" customWidth="1"/>
@@ -1431,78 +1440,78 @@
       <c r="AG5" s="14"/>
     </row>
     <row r="6" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A6" s="15" t="s">
+      <c r="A6" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" s="5"/>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
+      <c r="F6" s="5"/>
+      <c r="G6" s="5"/>
+      <c r="H6" s="5"/>
+      <c r="I6" s="5"/>
+      <c r="J6" s="5"/>
+      <c r="K6" s="5"/>
+      <c r="L6" s="5"/>
+      <c r="M6" s="5"/>
+      <c r="N6" s="5"/>
+      <c r="O6" s="5"/>
+      <c r="P6" s="5"/>
+      <c r="Q6" s="5"/>
+      <c r="R6" s="5"/>
+      <c r="S6" s="5"/>
+      <c r="T6" s="5"/>
+      <c r="U6" s="5"/>
+      <c r="V6" s="5"/>
+      <c r="W6" s="5"/>
+      <c r="X6" s="5"/>
+      <c r="Y6" s="5"/>
+      <c r="Z6" s="5"/>
+      <c r="AA6" s="5"/>
+      <c r="AB6" s="5"/>
+      <c r="AC6" s="5"/>
+      <c r="AD6" s="5"/>
+      <c r="AE6" s="5"/>
+      <c r="AF6" s="5"/>
+      <c r="AG6" s="18"/>
+    </row>
+    <row r="7" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A7" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
-      <c r="G6" s="1"/>
-      <c r="H6" s="1"/>
-      <c r="I6" s="1"/>
-      <c r="J6" s="1"/>
-      <c r="K6" s="1"/>
-      <c r="L6" s="1"/>
-      <c r="M6" s="1"/>
-      <c r="N6" s="1"/>
-      <c r="O6" s="1"/>
-      <c r="P6" s="1"/>
-      <c r="Q6" s="1"/>
-      <c r="R6" s="1"/>
-      <c r="S6" s="1"/>
-      <c r="T6" s="1"/>
-      <c r="U6" s="1"/>
-      <c r="V6" s="1"/>
-      <c r="W6" s="1"/>
-      <c r="X6" s="1"/>
-      <c r="Y6" s="1"/>
-      <c r="Z6" s="1"/>
-      <c r="AA6" s="1"/>
-      <c r="AB6" s="1"/>
-      <c r="AC6" s="1"/>
-      <c r="AD6" s="1"/>
-      <c r="AE6" s="1"/>
-      <c r="AF6" s="1"/>
-      <c r="AG6" s="16"/>
-    </row>
-    <row r="7" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A7" s="17" t="s">
-        <v>25</v>
-      </c>
-      <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="5"/>
-      <c r="J7" s="5"/>
-      <c r="K7" s="5"/>
-      <c r="L7" s="5"/>
-      <c r="M7" s="5"/>
-      <c r="N7" s="5"/>
-      <c r="O7" s="5"/>
-      <c r="P7" s="5"/>
-      <c r="Q7" s="5"/>
-      <c r="R7" s="5"/>
-      <c r="S7" s="5"/>
-      <c r="T7" s="5"/>
-      <c r="U7" s="5"/>
-      <c r="V7" s="5"/>
-      <c r="W7" s="5"/>
-      <c r="X7" s="5"/>
-      <c r="Y7" s="5"/>
-      <c r="Z7" s="5"/>
-      <c r="AA7" s="5"/>
-      <c r="AB7" s="5"/>
-      <c r="AC7" s="5"/>
-      <c r="AD7" s="5"/>
-      <c r="AE7" s="5"/>
-      <c r="AF7" s="5"/>
-      <c r="AG7" s="18"/>
+      <c r="B7" s="1"/>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1"/>
+      <c r="H7" s="1"/>
+      <c r="I7" s="1"/>
+      <c r="J7" s="1"/>
+      <c r="K7" s="1"/>
+      <c r="L7" s="1"/>
+      <c r="M7" s="1"/>
+      <c r="N7" s="1"/>
+      <c r="O7" s="1"/>
+      <c r="P7" s="1"/>
+      <c r="Q7" s="1"/>
+      <c r="R7" s="1"/>
+      <c r="S7" s="1"/>
+      <c r="T7" s="1"/>
+      <c r="U7" s="1"/>
+      <c r="V7" s="1"/>
+      <c r="W7" s="1"/>
+      <c r="X7" s="1"/>
+      <c r="Y7" s="1"/>
+      <c r="Z7" s="1"/>
+      <c r="AA7" s="1"/>
+      <c r="AB7" s="1"/>
+      <c r="AC7" s="1"/>
+      <c r="AD7" s="1"/>
+      <c r="AE7" s="1"/>
+      <c r="AF7" s="1"/>
+      <c r="AG7" s="16"/>
     </row>
     <row r="8" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A8" s="19" t="s">
@@ -1730,29 +1739,29 @@
       <c r="AG12" s="35"/>
     </row>
     <row r="13" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A13" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
-      <c r="F13" s="1"/>
-      <c r="G13" s="1"/>
-      <c r="H13" s="1"/>
-      <c r="I13" s="1"/>
-      <c r="J13" s="1"/>
-      <c r="K13" s="1"/>
-      <c r="L13" s="1"/>
-      <c r="M13" s="1"/>
-      <c r="N13" s="1"/>
-      <c r="O13" s="1"/>
-      <c r="P13" s="1"/>
-      <c r="Q13" s="1"/>
-      <c r="R13" s="1"/>
-      <c r="S13" s="1"/>
-      <c r="T13" s="1"/>
-      <c r="U13" s="1"/>
+      <c r="A13" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13" s="5"/>
+      <c r="C13" s="5"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="5"/>
+      <c r="G13" s="5"/>
+      <c r="H13" s="5"/>
+      <c r="I13" s="5"/>
+      <c r="J13" s="5"/>
+      <c r="K13" s="5"/>
+      <c r="L13" s="5"/>
+      <c r="M13" s="5"/>
+      <c r="N13" s="5"/>
+      <c r="O13" s="5"/>
+      <c r="P13" s="5"/>
+      <c r="Q13" s="5"/>
+      <c r="R13" s="5"/>
+      <c r="S13" s="5"/>
+      <c r="T13" s="5"/>
+      <c r="U13" s="5"/>
       <c r="V13" s="34"/>
       <c r="W13" s="34"/>
       <c r="X13" s="34"/>
@@ -1767,29 +1776,29 @@
       <c r="AG13" s="35"/>
     </row>
     <row r="14" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A14" s="17" t="s">
-        <v>29</v>
-      </c>
-      <c r="B14" s="5"/>
-      <c r="C14" s="5"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
-      <c r="F14" s="5"/>
-      <c r="G14" s="5"/>
-      <c r="H14" s="5"/>
-      <c r="I14" s="5"/>
-      <c r="J14" s="5"/>
-      <c r="K14" s="5"/>
-      <c r="L14" s="5"/>
-      <c r="M14" s="5"/>
-      <c r="N14" s="5"/>
-      <c r="O14" s="5"/>
-      <c r="P14" s="5"/>
-      <c r="Q14" s="5"/>
-      <c r="R14" s="5"/>
-      <c r="S14" s="5"/>
-      <c r="T14" s="5"/>
-      <c r="U14" s="5"/>
+      <c r="A14" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
+      <c r="G14" s="1"/>
+      <c r="H14" s="1"/>
+      <c r="I14" s="1"/>
+      <c r="J14" s="1"/>
+      <c r="K14" s="1"/>
+      <c r="L14" s="1"/>
+      <c r="M14" s="1"/>
+      <c r="N14" s="1"/>
+      <c r="O14" s="1"/>
+      <c r="P14" s="1"/>
+      <c r="Q14" s="1"/>
+      <c r="R14" s="1"/>
+      <c r="S14" s="1"/>
+      <c r="T14" s="1"/>
+      <c r="U14" s="1"/>
       <c r="V14" s="34"/>
       <c r="W14" s="34"/>
       <c r="X14" s="34"/>
@@ -2091,78 +2100,78 @@
       <c r="AG21" s="14"/>
     </row>
     <row r="22" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A22" s="15" t="s">
+      <c r="A22" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="B22" s="5"/>
+      <c r="C22" s="5"/>
+      <c r="D22" s="5"/>
+      <c r="E22" s="5"/>
+      <c r="F22" s="5"/>
+      <c r="G22" s="5"/>
+      <c r="H22" s="5"/>
+      <c r="I22" s="5"/>
+      <c r="J22" s="5"/>
+      <c r="K22" s="5"/>
+      <c r="L22" s="5"/>
+      <c r="M22" s="5"/>
+      <c r="N22" s="5"/>
+      <c r="O22" s="5"/>
+      <c r="P22" s="5"/>
+      <c r="Q22" s="5"/>
+      <c r="R22" s="5"/>
+      <c r="S22" s="5"/>
+      <c r="T22" s="5"/>
+      <c r="U22" s="5"/>
+      <c r="V22" s="5"/>
+      <c r="W22" s="5"/>
+      <c r="X22" s="5"/>
+      <c r="Y22" s="5"/>
+      <c r="Z22" s="5"/>
+      <c r="AA22" s="5"/>
+      <c r="AB22" s="5"/>
+      <c r="AC22" s="5"/>
+      <c r="AD22" s="5"/>
+      <c r="AE22" s="5"/>
+      <c r="AF22" s="5"/>
+      <c r="AG22" s="18"/>
+    </row>
+    <row r="23" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A23" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B22" s="1"/>
-      <c r="C22" s="1"/>
-      <c r="D22" s="1"/>
-      <c r="E22" s="1"/>
-      <c r="F22" s="1"/>
-      <c r="G22" s="1"/>
-      <c r="H22" s="1"/>
-      <c r="I22" s="1"/>
-      <c r="J22" s="1"/>
-      <c r="K22" s="1"/>
-      <c r="L22" s="1"/>
-      <c r="M22" s="1"/>
-      <c r="N22" s="1"/>
-      <c r="O22" s="1"/>
-      <c r="P22" s="1"/>
-      <c r="Q22" s="1"/>
-      <c r="R22" s="1"/>
-      <c r="S22" s="1"/>
-      <c r="T22" s="1"/>
-      <c r="U22" s="1"/>
-      <c r="V22" s="1"/>
-      <c r="W22" s="1"/>
-      <c r="X22" s="1"/>
-      <c r="Y22" s="1"/>
-      <c r="Z22" s="1"/>
-      <c r="AA22" s="1"/>
-      <c r="AB22" s="1"/>
-      <c r="AC22" s="1"/>
-      <c r="AD22" s="1"/>
-      <c r="AE22" s="1"/>
-      <c r="AF22" s="1"/>
-      <c r="AG22" s="16"/>
-    </row>
-    <row r="23" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A23" s="17" t="s">
-        <v>25</v>
-      </c>
-      <c r="B23" s="5"/>
-      <c r="C23" s="5"/>
-      <c r="D23" s="5"/>
-      <c r="E23" s="5"/>
-      <c r="F23" s="5"/>
-      <c r="G23" s="5"/>
-      <c r="H23" s="5"/>
-      <c r="I23" s="5"/>
-      <c r="J23" s="5"/>
-      <c r="K23" s="5"/>
-      <c r="L23" s="5"/>
-      <c r="M23" s="5"/>
-      <c r="N23" s="5"/>
-      <c r="O23" s="5"/>
-      <c r="P23" s="5"/>
-      <c r="Q23" s="5"/>
-      <c r="R23" s="5"/>
-      <c r="S23" s="5"/>
-      <c r="T23" s="5"/>
-      <c r="U23" s="5"/>
-      <c r="V23" s="5"/>
-      <c r="W23" s="5"/>
-      <c r="X23" s="5"/>
-      <c r="Y23" s="5"/>
-      <c r="Z23" s="5"/>
-      <c r="AA23" s="5"/>
-      <c r="AB23" s="5"/>
-      <c r="AC23" s="5"/>
-      <c r="AD23" s="5"/>
-      <c r="AE23" s="5"/>
-      <c r="AF23" s="5"/>
-      <c r="AG23" s="18"/>
+      <c r="B23" s="1"/>
+      <c r="C23" s="1"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="1"/>
+      <c r="F23" s="1"/>
+      <c r="G23" s="1"/>
+      <c r="H23" s="1"/>
+      <c r="I23" s="1"/>
+      <c r="J23" s="1"/>
+      <c r="K23" s="1"/>
+      <c r="L23" s="1"/>
+      <c r="M23" s="1"/>
+      <c r="N23" s="1"/>
+      <c r="O23" s="1"/>
+      <c r="P23" s="1"/>
+      <c r="Q23" s="1"/>
+      <c r="R23" s="1"/>
+      <c r="S23" s="1"/>
+      <c r="T23" s="1"/>
+      <c r="U23" s="1"/>
+      <c r="V23" s="1"/>
+      <c r="W23" s="1"/>
+      <c r="X23" s="1"/>
+      <c r="Y23" s="1"/>
+      <c r="Z23" s="1"/>
+      <c r="AA23" s="1"/>
+      <c r="AB23" s="1"/>
+      <c r="AC23" s="1"/>
+      <c r="AD23" s="1"/>
+      <c r="AE23" s="1"/>
+      <c r="AF23" s="1"/>
+      <c r="AG23" s="16"/>
     </row>
     <row r="24" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A24" s="19" t="s">
@@ -2390,29 +2399,29 @@
       <c r="AG28" s="35"/>
     </row>
     <row r="29" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A29" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="B29" s="1"/>
-      <c r="C29" s="1"/>
-      <c r="D29" s="1"/>
-      <c r="E29" s="1"/>
-      <c r="F29" s="1"/>
-      <c r="G29" s="1"/>
-      <c r="H29" s="1"/>
-      <c r="I29" s="1"/>
-      <c r="J29" s="1"/>
-      <c r="K29" s="1"/>
-      <c r="L29" s="1"/>
-      <c r="M29" s="1"/>
-      <c r="N29" s="1"/>
-      <c r="O29" s="1"/>
-      <c r="P29" s="1"/>
-      <c r="Q29" s="1"/>
-      <c r="R29" s="1"/>
-      <c r="S29" s="1"/>
-      <c r="T29" s="1"/>
-      <c r="U29" s="1"/>
+      <c r="A29" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="B29" s="5"/>
+      <c r="C29" s="5"/>
+      <c r="D29" s="5"/>
+      <c r="E29" s="5"/>
+      <c r="F29" s="5"/>
+      <c r="G29" s="5"/>
+      <c r="H29" s="5"/>
+      <c r="I29" s="5"/>
+      <c r="J29" s="5"/>
+      <c r="K29" s="5"/>
+      <c r="L29" s="5"/>
+      <c r="M29" s="5"/>
+      <c r="N29" s="5"/>
+      <c r="O29" s="5"/>
+      <c r="P29" s="5"/>
+      <c r="Q29" s="5"/>
+      <c r="R29" s="5"/>
+      <c r="S29" s="5"/>
+      <c r="T29" s="5"/>
+      <c r="U29" s="5"/>
       <c r="V29" s="34"/>
       <c r="W29" s="34"/>
       <c r="X29" s="34"/>
@@ -2427,29 +2436,29 @@
       <c r="AG29" s="35"/>
     </row>
     <row r="30" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A30" s="17" t="s">
-        <v>29</v>
-      </c>
-      <c r="B30" s="5"/>
-      <c r="C30" s="5"/>
-      <c r="D30" s="5"/>
-      <c r="E30" s="5"/>
-      <c r="F30" s="5"/>
-      <c r="G30" s="5"/>
-      <c r="H30" s="5"/>
-      <c r="I30" s="5"/>
-      <c r="J30" s="5"/>
-      <c r="K30" s="5"/>
-      <c r="L30" s="5"/>
-      <c r="M30" s="5"/>
-      <c r="N30" s="5"/>
-      <c r="O30" s="5"/>
-      <c r="P30" s="5"/>
-      <c r="Q30" s="5"/>
-      <c r="R30" s="5"/>
-      <c r="S30" s="5"/>
-      <c r="T30" s="5"/>
-      <c r="U30" s="5"/>
+      <c r="A30" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="B30" s="1"/>
+      <c r="C30" s="1"/>
+      <c r="D30" s="1"/>
+      <c r="E30" s="1"/>
+      <c r="F30" s="1"/>
+      <c r="G30" s="1"/>
+      <c r="H30" s="1"/>
+      <c r="I30" s="1"/>
+      <c r="J30" s="1"/>
+      <c r="K30" s="1"/>
+      <c r="L30" s="1"/>
+      <c r="M30" s="1"/>
+      <c r="N30" s="1"/>
+      <c r="O30" s="1"/>
+      <c r="P30" s="1"/>
+      <c r="Q30" s="1"/>
+      <c r="R30" s="1"/>
+      <c r="S30" s="1"/>
+      <c r="T30" s="1"/>
+      <c r="U30" s="1"/>
       <c r="V30" s="34"/>
       <c r="W30" s="34"/>
       <c r="X30" s="34"/>
@@ -2575,6 +2584,9 @@
     <row r="34" spans="1:33" x14ac:dyDescent="0.25">
       <c r="N34" s="41"/>
     </row>
+    <row r="40" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="C40" s="51"/>
+    </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A1:XFD1"/>

</xml_diff>

<commit_message>
feat(grafico-planilha): inverte a ordem e as coordenadas de Obturado e Perdido mantendo as cores e o padrão C-O-P (#25)
</commit_message>
<xml_diff>
--- a/app/assets/planilhas/teethgram_en.xlsx
+++ b/app/assets/planilhas/teethgram_en.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DEV Workspace\projetos-profissionais\teethGram\app\assets\planilhas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\almei\dev\teethGram\app\assets\planilhas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34173F18-15A4-41A8-A2B5-721002CB9B30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{071AEE10-5C9E-46EF-807F-451296B52ACC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{AFFBEBE6-A6BC-498C-A820-BBF450B005CB}"/>
   </bookViews>
@@ -56,7 +56,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A6" authorId="0" shapeId="0" xr:uid="{A4DD2828-35E0-4A5F-9196-F4E1CED96808}">
+    <comment ref="A6" authorId="0" shapeId="0" xr:uid="{2E440F82-1ED1-4C0A-8C89-CAC623CBBD31}">
       <text>
         <r>
           <rPr>
@@ -70,7 +70,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A7" authorId="0" shapeId="0" xr:uid="{2E440F82-1ED1-4C0A-8C89-CAC623CBBD31}">
+    <comment ref="A7" authorId="0" shapeId="0" xr:uid="{A4DD2828-35E0-4A5F-9196-F4E1CED96808}">
       <text>
         <r>
           <rPr>
@@ -111,7 +111,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A13" authorId="0" shapeId="0" xr:uid="{7354F24A-D9B6-400C-9B5C-7188D1761EE6}">
+    <comment ref="A13" authorId="0" shapeId="0" xr:uid="{5C01E885-706E-4DD4-8899-0996FA7C1E83}">
       <text>
         <r>
           <rPr>
@@ -125,7 +125,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A14" authorId="0" shapeId="0" xr:uid="{5C01E885-706E-4DD4-8899-0996FA7C1E83}">
+    <comment ref="A14" authorId="0" shapeId="0" xr:uid="{7354F24A-D9B6-400C-9B5C-7188D1761EE6}">
       <text>
         <r>
           <rPr>
@@ -166,7 +166,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A22" authorId="0" shapeId="0" xr:uid="{AEDD797E-6029-49AB-B684-18BCF2D7ABA1}">
+    <comment ref="A22" authorId="0" shapeId="0" xr:uid="{8D07286F-8727-4357-9417-A22B0C5C0E9E}">
       <text>
         <r>
           <rPr>
@@ -180,7 +180,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A23" authorId="0" shapeId="0" xr:uid="{8D07286F-8727-4357-9417-A22B0C5C0E9E}">
+    <comment ref="A23" authorId="0" shapeId="0" xr:uid="{AEDD797E-6029-49AB-B684-18BCF2D7ABA1}">
       <text>
         <r>
           <rPr>
@@ -221,7 +221,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A29" authorId="0" shapeId="0" xr:uid="{65F162A7-3776-48D5-AF6F-F6BBAD7337E5}">
+    <comment ref="A29" authorId="0" shapeId="0" xr:uid="{EAE70C67-A158-42EA-81E3-7ED4E2D2B0F6}">
       <text>
         <r>
           <rPr>
@@ -235,7 +235,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A30" authorId="0" shapeId="0" xr:uid="{EAE70C67-A158-42EA-81E3-7ED4E2D2B0F6}">
+    <comment ref="A30" authorId="0" shapeId="0" xr:uid="{65F162A7-3776-48D5-AF6F-F6BBAD7337E5}">
       <text>
         <r>
           <rPr>
@@ -381,7 +381,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -418,6 +418,14 @@
       <color indexed="81"/>
       <name val="Segoe UI"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="15">
@@ -780,7 +788,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -870,6 +878,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1209,7 +1218,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91CAF953-5A63-4D25-9285-6A1D6422454A}">
-  <dimension ref="A1:AG34"/>
+  <dimension ref="A1:AG40"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.28515625" customWidth="1"/>
@@ -1431,78 +1440,78 @@
       <c r="AG5" s="14"/>
     </row>
     <row r="6" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A6" s="15" t="s">
+      <c r="A6" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" s="5"/>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
+      <c r="F6" s="5"/>
+      <c r="G6" s="5"/>
+      <c r="H6" s="5"/>
+      <c r="I6" s="5"/>
+      <c r="J6" s="5"/>
+      <c r="K6" s="5"/>
+      <c r="L6" s="5"/>
+      <c r="M6" s="5"/>
+      <c r="N6" s="5"/>
+      <c r="O6" s="5"/>
+      <c r="P6" s="5"/>
+      <c r="Q6" s="5"/>
+      <c r="R6" s="5"/>
+      <c r="S6" s="5"/>
+      <c r="T6" s="5"/>
+      <c r="U6" s="5"/>
+      <c r="V6" s="5"/>
+      <c r="W6" s="5"/>
+      <c r="X6" s="5"/>
+      <c r="Y6" s="5"/>
+      <c r="Z6" s="5"/>
+      <c r="AA6" s="5"/>
+      <c r="AB6" s="5"/>
+      <c r="AC6" s="5"/>
+      <c r="AD6" s="5"/>
+      <c r="AE6" s="5"/>
+      <c r="AF6" s="5"/>
+      <c r="AG6" s="18"/>
+    </row>
+    <row r="7" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A7" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
-      <c r="G6" s="1"/>
-      <c r="H6" s="1"/>
-      <c r="I6" s="1"/>
-      <c r="J6" s="1"/>
-      <c r="K6" s="1"/>
-      <c r="L6" s="1"/>
-      <c r="M6" s="1"/>
-      <c r="N6" s="1"/>
-      <c r="O6" s="1"/>
-      <c r="P6" s="1"/>
-      <c r="Q6" s="1"/>
-      <c r="R6" s="1"/>
-      <c r="S6" s="1"/>
-      <c r="T6" s="1"/>
-      <c r="U6" s="1"/>
-      <c r="V6" s="1"/>
-      <c r="W6" s="1"/>
-      <c r="X6" s="1"/>
-      <c r="Y6" s="1"/>
-      <c r="Z6" s="1"/>
-      <c r="AA6" s="1"/>
-      <c r="AB6" s="1"/>
-      <c r="AC6" s="1"/>
-      <c r="AD6" s="1"/>
-      <c r="AE6" s="1"/>
-      <c r="AF6" s="1"/>
-      <c r="AG6" s="16"/>
-    </row>
-    <row r="7" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A7" s="17" t="s">
-        <v>25</v>
-      </c>
-      <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="5"/>
-      <c r="J7" s="5"/>
-      <c r="K7" s="5"/>
-      <c r="L7" s="5"/>
-      <c r="M7" s="5"/>
-      <c r="N7" s="5"/>
-      <c r="O7" s="5"/>
-      <c r="P7" s="5"/>
-      <c r="Q7" s="5"/>
-      <c r="R7" s="5"/>
-      <c r="S7" s="5"/>
-      <c r="T7" s="5"/>
-      <c r="U7" s="5"/>
-      <c r="V7" s="5"/>
-      <c r="W7" s="5"/>
-      <c r="X7" s="5"/>
-      <c r="Y7" s="5"/>
-      <c r="Z7" s="5"/>
-      <c r="AA7" s="5"/>
-      <c r="AB7" s="5"/>
-      <c r="AC7" s="5"/>
-      <c r="AD7" s="5"/>
-      <c r="AE7" s="5"/>
-      <c r="AF7" s="5"/>
-      <c r="AG7" s="18"/>
+      <c r="B7" s="1"/>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1"/>
+      <c r="H7" s="1"/>
+      <c r="I7" s="1"/>
+      <c r="J7" s="1"/>
+      <c r="K7" s="1"/>
+      <c r="L7" s="1"/>
+      <c r="M7" s="1"/>
+      <c r="N7" s="1"/>
+      <c r="O7" s="1"/>
+      <c r="P7" s="1"/>
+      <c r="Q7" s="1"/>
+      <c r="R7" s="1"/>
+      <c r="S7" s="1"/>
+      <c r="T7" s="1"/>
+      <c r="U7" s="1"/>
+      <c r="V7" s="1"/>
+      <c r="W7" s="1"/>
+      <c r="X7" s="1"/>
+      <c r="Y7" s="1"/>
+      <c r="Z7" s="1"/>
+      <c r="AA7" s="1"/>
+      <c r="AB7" s="1"/>
+      <c r="AC7" s="1"/>
+      <c r="AD7" s="1"/>
+      <c r="AE7" s="1"/>
+      <c r="AF7" s="1"/>
+      <c r="AG7" s="16"/>
     </row>
     <row r="8" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A8" s="19" t="s">
@@ -1730,29 +1739,29 @@
       <c r="AG12" s="35"/>
     </row>
     <row r="13" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A13" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
-      <c r="F13" s="1"/>
-      <c r="G13" s="1"/>
-      <c r="H13" s="1"/>
-      <c r="I13" s="1"/>
-      <c r="J13" s="1"/>
-      <c r="K13" s="1"/>
-      <c r="L13" s="1"/>
-      <c r="M13" s="1"/>
-      <c r="N13" s="1"/>
-      <c r="O13" s="1"/>
-      <c r="P13" s="1"/>
-      <c r="Q13" s="1"/>
-      <c r="R13" s="1"/>
-      <c r="S13" s="1"/>
-      <c r="T13" s="1"/>
-      <c r="U13" s="1"/>
+      <c r="A13" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13" s="5"/>
+      <c r="C13" s="5"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="5"/>
+      <c r="G13" s="5"/>
+      <c r="H13" s="5"/>
+      <c r="I13" s="5"/>
+      <c r="J13" s="5"/>
+      <c r="K13" s="5"/>
+      <c r="L13" s="5"/>
+      <c r="M13" s="5"/>
+      <c r="N13" s="5"/>
+      <c r="O13" s="5"/>
+      <c r="P13" s="5"/>
+      <c r="Q13" s="5"/>
+      <c r="R13" s="5"/>
+      <c r="S13" s="5"/>
+      <c r="T13" s="5"/>
+      <c r="U13" s="5"/>
       <c r="V13" s="34"/>
       <c r="W13" s="34"/>
       <c r="X13" s="34"/>
@@ -1767,29 +1776,29 @@
       <c r="AG13" s="35"/>
     </row>
     <row r="14" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A14" s="17" t="s">
-        <v>29</v>
-      </c>
-      <c r="B14" s="5"/>
-      <c r="C14" s="5"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
-      <c r="F14" s="5"/>
-      <c r="G14" s="5"/>
-      <c r="H14" s="5"/>
-      <c r="I14" s="5"/>
-      <c r="J14" s="5"/>
-      <c r="K14" s="5"/>
-      <c r="L14" s="5"/>
-      <c r="M14" s="5"/>
-      <c r="N14" s="5"/>
-      <c r="O14" s="5"/>
-      <c r="P14" s="5"/>
-      <c r="Q14" s="5"/>
-      <c r="R14" s="5"/>
-      <c r="S14" s="5"/>
-      <c r="T14" s="5"/>
-      <c r="U14" s="5"/>
+      <c r="A14" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
+      <c r="G14" s="1"/>
+      <c r="H14" s="1"/>
+      <c r="I14" s="1"/>
+      <c r="J14" s="1"/>
+      <c r="K14" s="1"/>
+      <c r="L14" s="1"/>
+      <c r="M14" s="1"/>
+      <c r="N14" s="1"/>
+      <c r="O14" s="1"/>
+      <c r="P14" s="1"/>
+      <c r="Q14" s="1"/>
+      <c r="R14" s="1"/>
+      <c r="S14" s="1"/>
+      <c r="T14" s="1"/>
+      <c r="U14" s="1"/>
       <c r="V14" s="34"/>
       <c r="W14" s="34"/>
       <c r="X14" s="34"/>
@@ -2091,78 +2100,78 @@
       <c r="AG21" s="14"/>
     </row>
     <row r="22" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A22" s="15" t="s">
+      <c r="A22" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="B22" s="5"/>
+      <c r="C22" s="5"/>
+      <c r="D22" s="5"/>
+      <c r="E22" s="5"/>
+      <c r="F22" s="5"/>
+      <c r="G22" s="5"/>
+      <c r="H22" s="5"/>
+      <c r="I22" s="5"/>
+      <c r="J22" s="5"/>
+      <c r="K22" s="5"/>
+      <c r="L22" s="5"/>
+      <c r="M22" s="5"/>
+      <c r="N22" s="5"/>
+      <c r="O22" s="5"/>
+      <c r="P22" s="5"/>
+      <c r="Q22" s="5"/>
+      <c r="R22" s="5"/>
+      <c r="S22" s="5"/>
+      <c r="T22" s="5"/>
+      <c r="U22" s="5"/>
+      <c r="V22" s="5"/>
+      <c r="W22" s="5"/>
+      <c r="X22" s="5"/>
+      <c r="Y22" s="5"/>
+      <c r="Z22" s="5"/>
+      <c r="AA22" s="5"/>
+      <c r="AB22" s="5"/>
+      <c r="AC22" s="5"/>
+      <c r="AD22" s="5"/>
+      <c r="AE22" s="5"/>
+      <c r="AF22" s="5"/>
+      <c r="AG22" s="18"/>
+    </row>
+    <row r="23" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A23" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B22" s="1"/>
-      <c r="C22" s="1"/>
-      <c r="D22" s="1"/>
-      <c r="E22" s="1"/>
-      <c r="F22" s="1"/>
-      <c r="G22" s="1"/>
-      <c r="H22" s="1"/>
-      <c r="I22" s="1"/>
-      <c r="J22" s="1"/>
-      <c r="K22" s="1"/>
-      <c r="L22" s="1"/>
-      <c r="M22" s="1"/>
-      <c r="N22" s="1"/>
-      <c r="O22" s="1"/>
-      <c r="P22" s="1"/>
-      <c r="Q22" s="1"/>
-      <c r="R22" s="1"/>
-      <c r="S22" s="1"/>
-      <c r="T22" s="1"/>
-      <c r="U22" s="1"/>
-      <c r="V22" s="1"/>
-      <c r="W22" s="1"/>
-      <c r="X22" s="1"/>
-      <c r="Y22" s="1"/>
-      <c r="Z22" s="1"/>
-      <c r="AA22" s="1"/>
-      <c r="AB22" s="1"/>
-      <c r="AC22" s="1"/>
-      <c r="AD22" s="1"/>
-      <c r="AE22" s="1"/>
-      <c r="AF22" s="1"/>
-      <c r="AG22" s="16"/>
-    </row>
-    <row r="23" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A23" s="17" t="s">
-        <v>25</v>
-      </c>
-      <c r="B23" s="5"/>
-      <c r="C23" s="5"/>
-      <c r="D23" s="5"/>
-      <c r="E23" s="5"/>
-      <c r="F23" s="5"/>
-      <c r="G23" s="5"/>
-      <c r="H23" s="5"/>
-      <c r="I23" s="5"/>
-      <c r="J23" s="5"/>
-      <c r="K23" s="5"/>
-      <c r="L23" s="5"/>
-      <c r="M23" s="5"/>
-      <c r="N23" s="5"/>
-      <c r="O23" s="5"/>
-      <c r="P23" s="5"/>
-      <c r="Q23" s="5"/>
-      <c r="R23" s="5"/>
-      <c r="S23" s="5"/>
-      <c r="T23" s="5"/>
-      <c r="U23" s="5"/>
-      <c r="V23" s="5"/>
-      <c r="W23" s="5"/>
-      <c r="X23" s="5"/>
-      <c r="Y23" s="5"/>
-      <c r="Z23" s="5"/>
-      <c r="AA23" s="5"/>
-      <c r="AB23" s="5"/>
-      <c r="AC23" s="5"/>
-      <c r="AD23" s="5"/>
-      <c r="AE23" s="5"/>
-      <c r="AF23" s="5"/>
-      <c r="AG23" s="18"/>
+      <c r="B23" s="1"/>
+      <c r="C23" s="1"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="1"/>
+      <c r="F23" s="1"/>
+      <c r="G23" s="1"/>
+      <c r="H23" s="1"/>
+      <c r="I23" s="1"/>
+      <c r="J23" s="1"/>
+      <c r="K23" s="1"/>
+      <c r="L23" s="1"/>
+      <c r="M23" s="1"/>
+      <c r="N23" s="1"/>
+      <c r="O23" s="1"/>
+      <c r="P23" s="1"/>
+      <c r="Q23" s="1"/>
+      <c r="R23" s="1"/>
+      <c r="S23" s="1"/>
+      <c r="T23" s="1"/>
+      <c r="U23" s="1"/>
+      <c r="V23" s="1"/>
+      <c r="W23" s="1"/>
+      <c r="X23" s="1"/>
+      <c r="Y23" s="1"/>
+      <c r="Z23" s="1"/>
+      <c r="AA23" s="1"/>
+      <c r="AB23" s="1"/>
+      <c r="AC23" s="1"/>
+      <c r="AD23" s="1"/>
+      <c r="AE23" s="1"/>
+      <c r="AF23" s="1"/>
+      <c r="AG23" s="16"/>
     </row>
     <row r="24" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A24" s="19" t="s">
@@ -2390,29 +2399,29 @@
       <c r="AG28" s="35"/>
     </row>
     <row r="29" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A29" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="B29" s="1"/>
-      <c r="C29" s="1"/>
-      <c r="D29" s="1"/>
-      <c r="E29" s="1"/>
-      <c r="F29" s="1"/>
-      <c r="G29" s="1"/>
-      <c r="H29" s="1"/>
-      <c r="I29" s="1"/>
-      <c r="J29" s="1"/>
-      <c r="K29" s="1"/>
-      <c r="L29" s="1"/>
-      <c r="M29" s="1"/>
-      <c r="N29" s="1"/>
-      <c r="O29" s="1"/>
-      <c r="P29" s="1"/>
-      <c r="Q29" s="1"/>
-      <c r="R29" s="1"/>
-      <c r="S29" s="1"/>
-      <c r="T29" s="1"/>
-      <c r="U29" s="1"/>
+      <c r="A29" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="B29" s="5"/>
+      <c r="C29" s="5"/>
+      <c r="D29" s="5"/>
+      <c r="E29" s="5"/>
+      <c r="F29" s="5"/>
+      <c r="G29" s="5"/>
+      <c r="H29" s="5"/>
+      <c r="I29" s="5"/>
+      <c r="J29" s="5"/>
+      <c r="K29" s="5"/>
+      <c r="L29" s="5"/>
+      <c r="M29" s="5"/>
+      <c r="N29" s="5"/>
+      <c r="O29" s="5"/>
+      <c r="P29" s="5"/>
+      <c r="Q29" s="5"/>
+      <c r="R29" s="5"/>
+      <c r="S29" s="5"/>
+      <c r="T29" s="5"/>
+      <c r="U29" s="5"/>
       <c r="V29" s="34"/>
       <c r="W29" s="34"/>
       <c r="X29" s="34"/>
@@ -2427,29 +2436,29 @@
       <c r="AG29" s="35"/>
     </row>
     <row r="30" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A30" s="17" t="s">
-        <v>29</v>
-      </c>
-      <c r="B30" s="5"/>
-      <c r="C30" s="5"/>
-      <c r="D30" s="5"/>
-      <c r="E30" s="5"/>
-      <c r="F30" s="5"/>
-      <c r="G30" s="5"/>
-      <c r="H30" s="5"/>
-      <c r="I30" s="5"/>
-      <c r="J30" s="5"/>
-      <c r="K30" s="5"/>
-      <c r="L30" s="5"/>
-      <c r="M30" s="5"/>
-      <c r="N30" s="5"/>
-      <c r="O30" s="5"/>
-      <c r="P30" s="5"/>
-      <c r="Q30" s="5"/>
-      <c r="R30" s="5"/>
-      <c r="S30" s="5"/>
-      <c r="T30" s="5"/>
-      <c r="U30" s="5"/>
+      <c r="A30" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="B30" s="1"/>
+      <c r="C30" s="1"/>
+      <c r="D30" s="1"/>
+      <c r="E30" s="1"/>
+      <c r="F30" s="1"/>
+      <c r="G30" s="1"/>
+      <c r="H30" s="1"/>
+      <c r="I30" s="1"/>
+      <c r="J30" s="1"/>
+      <c r="K30" s="1"/>
+      <c r="L30" s="1"/>
+      <c r="M30" s="1"/>
+      <c r="N30" s="1"/>
+      <c r="O30" s="1"/>
+      <c r="P30" s="1"/>
+      <c r="Q30" s="1"/>
+      <c r="R30" s="1"/>
+      <c r="S30" s="1"/>
+      <c r="T30" s="1"/>
+      <c r="U30" s="1"/>
       <c r="V30" s="34"/>
       <c r="W30" s="34"/>
       <c r="X30" s="34"/>
@@ -2575,6 +2584,9 @@
     <row r="34" spans="1:33" x14ac:dyDescent="0.25">
       <c r="N34" s="41"/>
     </row>
+    <row r="40" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="C40" s="51"/>
+    </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A1:XFD1"/>

</xml_diff>

<commit_message>
feat: adiciona suporte ao modelo de 4 componentes (C/O) no processamento, formulários e canvas
</commit_message>
<xml_diff>
--- a/app/assets/planilhas/teethgram_en.xlsx
+++ b/app/assets/planilhas/teethgram_en.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\almei\dev\teethGram\app\assets\planilhas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{071AEE10-5C9E-46EF-807F-451296B52ACC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{AFFBEBE6-A6BC-498C-A820-BBF450B005CB}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,12 +36,12 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Acer</author>
   </authors>
   <commentList>
-    <comment ref="A5" authorId="0" shapeId="0" xr:uid="{644B7FCF-627E-4E62-A53E-F918F34EE001}">
+    <comment ref="A5" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -56,7 +55,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A6" authorId="0" shapeId="0" xr:uid="{2E440F82-1ED1-4C0A-8C89-CAC623CBBD31}">
+    <comment ref="A7" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -70,7 +69,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A7" authorId="0" shapeId="0" xr:uid="{A4DD2828-35E0-4A5F-9196-F4E1CED96808}">
+    <comment ref="A8" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -84,7 +83,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A8" authorId="0" shapeId="0" xr:uid="{E48B4EB0-D078-4A8C-A169-0ACA2332C515}">
+    <comment ref="A9" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -97,7 +96,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A12" authorId="0" shapeId="0" xr:uid="{4B1F7472-8288-4D18-AEBA-DFFCDEA8A3E2}">
+    <comment ref="A13" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -111,7 +110,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A13" authorId="0" shapeId="0" xr:uid="{5C01E885-706E-4DD4-8899-0996FA7C1E83}">
+    <comment ref="A15" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -125,7 +124,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A14" authorId="0" shapeId="0" xr:uid="{7354F24A-D9B6-400C-9B5C-7188D1761EE6}">
+    <comment ref="A16" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -139,7 +138,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A15" authorId="0" shapeId="0" xr:uid="{E1DBFD74-70CF-4967-8538-81E0FB5B8008}">
+    <comment ref="A17" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -152,7 +151,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A21" authorId="0" shapeId="0" xr:uid="{530DA091-E276-46FF-837E-F2FF425C6DF7}">
+    <comment ref="A23" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -166,7 +165,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A22" authorId="0" shapeId="0" xr:uid="{8D07286F-8727-4357-9417-A22B0C5C0E9E}">
+    <comment ref="A25" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -180,7 +179,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A23" authorId="0" shapeId="0" xr:uid="{AEDD797E-6029-49AB-B684-18BCF2D7ABA1}">
+    <comment ref="A26" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -194,7 +193,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A24" authorId="0" shapeId="0" xr:uid="{0BDDB6FB-1367-41B0-9ECD-1612D5B326D3}">
+    <comment ref="A27" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -207,7 +206,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A28" authorId="0" shapeId="0" xr:uid="{E586BBD3-A76F-47AB-9B09-03CA944C390E}">
+    <comment ref="A31" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -221,7 +220,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A29" authorId="0" shapeId="0" xr:uid="{EAE70C67-A158-42EA-81E3-7ED4E2D2B0F6}">
+    <comment ref="A33" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -235,7 +234,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A30" authorId="0" shapeId="0" xr:uid="{65F162A7-3776-48D5-AF6F-F6BBAD7337E5}">
+    <comment ref="A34" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -249,7 +248,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A31" authorId="0" shapeId="0" xr:uid="{838042A5-64E2-424B-8E3B-22D465E70084}">
+    <comment ref="A35" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -267,7 +266,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="38">
   <si>
     <t>A</t>
   </si>
@@ -375,13 +374,19 @@
   </si>
   <si>
     <t>Fill in the total number of participants affected per dental unit for each component (d, m, f) or for the total (dmft).</t>
+  </si>
+  <si>
+    <t>Decayed/Filled (D/F)</t>
+  </si>
+  <si>
+    <t>decayed/filled (d/f)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -788,7 +793,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -851,6 +856,7 @@
     <xf numFmtId="0" fontId="1" fillId="14" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="14" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -878,7 +884,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1217,15 +1225,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91CAF953-5A63-4D25-9285-6A1D6422454A}">
-  <dimension ref="A1:AG40"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:AG46"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="20.28515625" customWidth="1"/>
+    <col min="1" max="1" width="20.25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" s="42" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="1:33" s="2" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:33" s="43" customFormat="1" ht="15" customHeight="1" thickBot="1"/>
+    <row r="2" spans="1:33" s="2" customFormat="1" ht="15" customHeight="1" thickBot="1">
       <c r="A2" s="9" t="s">
         <v>20</v>
       </c>
@@ -1262,46 +1270,46 @@
       <c r="AF2" s="36"/>
       <c r="AG2" s="37"/>
     </row>
-    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:33">
       <c r="A3" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="45" t="s">
+      <c r="B3" s="46" t="s">
         <v>34</v>
       </c>
-      <c r="C3" s="46"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="46"/>
-      <c r="F3" s="46"/>
-      <c r="G3" s="46"/>
-      <c r="H3" s="46"/>
-      <c r="I3" s="46"/>
-      <c r="J3" s="46"/>
-      <c r="K3" s="46"/>
-      <c r="L3" s="46"/>
-      <c r="M3" s="46"/>
-      <c r="N3" s="46"/>
-      <c r="O3" s="46"/>
-      <c r="P3" s="46"/>
-      <c r="Q3" s="46"/>
-      <c r="R3" s="46"/>
-      <c r="S3" s="46"/>
-      <c r="T3" s="46"/>
-      <c r="U3" s="46"/>
-      <c r="V3" s="46"/>
-      <c r="W3" s="46"/>
-      <c r="X3" s="46"/>
-      <c r="Y3" s="46"/>
-      <c r="Z3" s="46"/>
-      <c r="AA3" s="46"/>
-      <c r="AB3" s="46"/>
-      <c r="AC3" s="46"/>
-      <c r="AD3" s="46"/>
-      <c r="AE3" s="46"/>
-      <c r="AF3" s="46"/>
-      <c r="AG3" s="47"/>
-    </row>
-    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="C3" s="47"/>
+      <c r="D3" s="47"/>
+      <c r="E3" s="47"/>
+      <c r="F3" s="47"/>
+      <c r="G3" s="47"/>
+      <c r="H3" s="47"/>
+      <c r="I3" s="47"/>
+      <c r="J3" s="47"/>
+      <c r="K3" s="47"/>
+      <c r="L3" s="47"/>
+      <c r="M3" s="47"/>
+      <c r="N3" s="47"/>
+      <c r="O3" s="47"/>
+      <c r="P3" s="47"/>
+      <c r="Q3" s="47"/>
+      <c r="R3" s="47"/>
+      <c r="S3" s="47"/>
+      <c r="T3" s="47"/>
+      <c r="U3" s="47"/>
+      <c r="V3" s="47"/>
+      <c r="W3" s="47"/>
+      <c r="X3" s="47"/>
+      <c r="Y3" s="47"/>
+      <c r="Z3" s="47"/>
+      <c r="AA3" s="47"/>
+      <c r="AB3" s="47"/>
+      <c r="AC3" s="47"/>
+      <c r="AD3" s="47"/>
+      <c r="AE3" s="47"/>
+      <c r="AF3" s="47"/>
+      <c r="AG3" s="48"/>
+    </row>
+    <row r="4" spans="1:33" ht="15">
       <c r="A4" s="11" t="s">
         <v>22</v>
       </c>
@@ -1402,7 +1410,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:33" ht="15">
       <c r="A5" s="13" t="s">
         <v>23</v>
       </c>
@@ -1439,329 +1447,329 @@
       <c r="AF5" s="6"/>
       <c r="AG5" s="14"/>
     </row>
-    <row r="6" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A6" s="17" t="s">
+    <row r="6" spans="1:33" ht="15">
+      <c r="A6" s="52" t="s">
+        <v>36</v>
+      </c>
+      <c r="B6" s="53"/>
+      <c r="C6" s="53"/>
+      <c r="D6" s="53"/>
+      <c r="E6" s="53"/>
+      <c r="F6" s="53"/>
+      <c r="G6" s="53"/>
+      <c r="H6" s="53"/>
+      <c r="I6" s="53"/>
+      <c r="J6" s="53"/>
+      <c r="K6" s="53"/>
+      <c r="L6" s="53"/>
+      <c r="M6" s="53"/>
+      <c r="N6" s="53"/>
+      <c r="O6" s="53"/>
+      <c r="P6" s="53"/>
+      <c r="Q6" s="53"/>
+      <c r="R6" s="53"/>
+      <c r="S6" s="53"/>
+      <c r="T6" s="53"/>
+      <c r="U6" s="53"/>
+      <c r="V6" s="53"/>
+      <c r="W6" s="53"/>
+      <c r="X6" s="53"/>
+      <c r="Y6" s="53"/>
+      <c r="Z6" s="53"/>
+      <c r="AA6" s="53"/>
+      <c r="AB6" s="53"/>
+      <c r="AC6" s="53"/>
+      <c r="AD6" s="53"/>
+      <c r="AE6" s="53"/>
+      <c r="AF6" s="53"/>
+      <c r="AG6" s="54"/>
+    </row>
+    <row r="7" spans="1:33" ht="15">
+      <c r="A7" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5"/>
-      <c r="H6" s="5"/>
-      <c r="I6" s="5"/>
-      <c r="J6" s="5"/>
-      <c r="K6" s="5"/>
-      <c r="L6" s="5"/>
-      <c r="M6" s="5"/>
-      <c r="N6" s="5"/>
-      <c r="O6" s="5"/>
-      <c r="P6" s="5"/>
-      <c r="Q6" s="5"/>
-      <c r="R6" s="5"/>
-      <c r="S6" s="5"/>
-      <c r="T6" s="5"/>
-      <c r="U6" s="5"/>
-      <c r="V6" s="5"/>
-      <c r="W6" s="5"/>
-      <c r="X6" s="5"/>
-      <c r="Y6" s="5"/>
-      <c r="Z6" s="5"/>
-      <c r="AA6" s="5"/>
-      <c r="AB6" s="5"/>
-      <c r="AC6" s="5"/>
-      <c r="AD6" s="5"/>
-      <c r="AE6" s="5"/>
-      <c r="AF6" s="5"/>
-      <c r="AG6" s="18"/>
-    </row>
-    <row r="7" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A7" s="15" t="s">
+      <c r="B7" s="5"/>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5"/>
+      <c r="F7" s="5"/>
+      <c r="G7" s="5"/>
+      <c r="H7" s="5"/>
+      <c r="I7" s="5"/>
+      <c r="J7" s="5"/>
+      <c r="K7" s="5"/>
+      <c r="L7" s="5"/>
+      <c r="M7" s="5"/>
+      <c r="N7" s="5"/>
+      <c r="O7" s="5"/>
+      <c r="P7" s="5"/>
+      <c r="Q7" s="5"/>
+      <c r="R7" s="5"/>
+      <c r="S7" s="5"/>
+      <c r="T7" s="5"/>
+      <c r="U7" s="5"/>
+      <c r="V7" s="5"/>
+      <c r="W7" s="5"/>
+      <c r="X7" s="5"/>
+      <c r="Y7" s="5"/>
+      <c r="Z7" s="5"/>
+      <c r="AA7" s="5"/>
+      <c r="AB7" s="5"/>
+      <c r="AC7" s="5"/>
+      <c r="AD7" s="5"/>
+      <c r="AE7" s="5"/>
+      <c r="AF7" s="5"/>
+      <c r="AG7" s="18"/>
+    </row>
+    <row r="8" spans="1:33" ht="15">
+      <c r="A8" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-      <c r="F7" s="1"/>
-      <c r="G7" s="1"/>
-      <c r="H7" s="1"/>
-      <c r="I7" s="1"/>
-      <c r="J7" s="1"/>
-      <c r="K7" s="1"/>
-      <c r="L7" s="1"/>
-      <c r="M7" s="1"/>
-      <c r="N7" s="1"/>
-      <c r="O7" s="1"/>
-      <c r="P7" s="1"/>
-      <c r="Q7" s="1"/>
-      <c r="R7" s="1"/>
-      <c r="S7" s="1"/>
-      <c r="T7" s="1"/>
-      <c r="U7" s="1"/>
-      <c r="V7" s="1"/>
-      <c r="W7" s="1"/>
-      <c r="X7" s="1"/>
-      <c r="Y7" s="1"/>
-      <c r="Z7" s="1"/>
-      <c r="AA7" s="1"/>
-      <c r="AB7" s="1"/>
-      <c r="AC7" s="1"/>
-      <c r="AD7" s="1"/>
-      <c r="AE7" s="1"/>
-      <c r="AF7" s="1"/>
-      <c r="AG7" s="16"/>
-    </row>
-    <row r="8" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A8" s="19" t="s">
+      <c r="B8" s="1"/>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+      <c r="F8" s="1"/>
+      <c r="G8" s="1"/>
+      <c r="H8" s="1"/>
+      <c r="I8" s="1"/>
+      <c r="J8" s="1"/>
+      <c r="K8" s="1"/>
+      <c r="L8" s="1"/>
+      <c r="M8" s="1"/>
+      <c r="N8" s="1"/>
+      <c r="O8" s="1"/>
+      <c r="P8" s="1"/>
+      <c r="Q8" s="1"/>
+      <c r="R8" s="1"/>
+      <c r="S8" s="1"/>
+      <c r="T8" s="1"/>
+      <c r="U8" s="1"/>
+      <c r="V8" s="1"/>
+      <c r="W8" s="1"/>
+      <c r="X8" s="1"/>
+      <c r="Y8" s="1"/>
+      <c r="Z8" s="1"/>
+      <c r="AA8" s="1"/>
+      <c r="AB8" s="1"/>
+      <c r="AC8" s="1"/>
+      <c r="AD8" s="1"/>
+      <c r="AE8" s="1"/>
+      <c r="AF8" s="1"/>
+      <c r="AG8" s="16"/>
+    </row>
+    <row r="9" spans="1:33" ht="15">
+      <c r="A9" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
-      <c r="H8" s="7"/>
-      <c r="I8" s="7"/>
-      <c r="J8" s="7"/>
-      <c r="K8" s="7"/>
-      <c r="L8" s="7"/>
-      <c r="M8" s="7"/>
-      <c r="N8" s="7"/>
-      <c r="O8" s="7"/>
-      <c r="P8" s="7"/>
-      <c r="Q8" s="7"/>
-      <c r="R8" s="7"/>
-      <c r="S8" s="7"/>
-      <c r="T8" s="7"/>
-      <c r="U8" s="7"/>
-      <c r="V8" s="7"/>
-      <c r="W8" s="7"/>
-      <c r="X8" s="7"/>
-      <c r="Y8" s="7"/>
-      <c r="Z8" s="7"/>
-      <c r="AA8" s="7"/>
-      <c r="AB8" s="7"/>
-      <c r="AC8" s="7"/>
-      <c r="AD8" s="7"/>
-      <c r="AE8" s="7"/>
-      <c r="AF8" s="7"/>
-      <c r="AG8" s="20"/>
-    </row>
-    <row r="9" spans="1:33" s="8" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="27"/>
-      <c r="B9" s="28"/>
-      <c r="C9" s="28"/>
-      <c r="D9" s="28"/>
-      <c r="E9" s="28"/>
-      <c r="F9" s="28"/>
-      <c r="G9" s="28"/>
-      <c r="H9" s="28"/>
-      <c r="I9" s="28"/>
-      <c r="J9" s="28"/>
-      <c r="K9" s="28"/>
-      <c r="L9" s="28"/>
-      <c r="M9" s="28"/>
-      <c r="N9" s="28"/>
-      <c r="O9" s="28"/>
-      <c r="P9" s="28"/>
-      <c r="Q9" s="28"/>
-      <c r="R9" s="28"/>
-      <c r="S9" s="28"/>
-      <c r="T9" s="28"/>
-      <c r="U9" s="28"/>
-      <c r="V9" s="28"/>
-      <c r="W9" s="28"/>
-      <c r="X9" s="28"/>
-      <c r="Y9" s="28"/>
-      <c r="Z9" s="28"/>
-      <c r="AA9" s="28"/>
-      <c r="AB9" s="28"/>
-      <c r="AC9" s="28"/>
-      <c r="AD9" s="28"/>
-      <c r="AE9" s="28"/>
-      <c r="AF9" s="28"/>
-      <c r="AG9" s="29"/>
-    </row>
-    <row r="10" spans="1:33" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="21" t="s">
+      <c r="B9" s="7"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="7"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="7"/>
+      <c r="G9" s="7"/>
+      <c r="H9" s="7"/>
+      <c r="I9" s="7"/>
+      <c r="J9" s="7"/>
+      <c r="K9" s="7"/>
+      <c r="L9" s="7"/>
+      <c r="M9" s="7"/>
+      <c r="N9" s="7"/>
+      <c r="O9" s="7"/>
+      <c r="P9" s="7"/>
+      <c r="Q9" s="7"/>
+      <c r="R9" s="7"/>
+      <c r="S9" s="7"/>
+      <c r="T9" s="7"/>
+      <c r="U9" s="7"/>
+      <c r="V9" s="7"/>
+      <c r="W9" s="7"/>
+      <c r="X9" s="7"/>
+      <c r="Y9" s="7"/>
+      <c r="Z9" s="7"/>
+      <c r="AA9" s="7"/>
+      <c r="AB9" s="7"/>
+      <c r="AC9" s="7"/>
+      <c r="AD9" s="7"/>
+      <c r="AE9" s="7"/>
+      <c r="AF9" s="7"/>
+      <c r="AG9" s="20"/>
+    </row>
+    <row r="10" spans="1:33" s="8" customFormat="1" ht="15" customHeight="1">
+      <c r="A10" s="27"/>
+      <c r="B10" s="28"/>
+      <c r="C10" s="28"/>
+      <c r="D10" s="28"/>
+      <c r="E10" s="28"/>
+      <c r="F10" s="28"/>
+      <c r="G10" s="28"/>
+      <c r="H10" s="28"/>
+      <c r="I10" s="28"/>
+      <c r="J10" s="28"/>
+      <c r="K10" s="28"/>
+      <c r="L10" s="28"/>
+      <c r="M10" s="28"/>
+      <c r="N10" s="28"/>
+      <c r="O10" s="28"/>
+      <c r="P10" s="28"/>
+      <c r="Q10" s="28"/>
+      <c r="R10" s="28"/>
+      <c r="S10" s="28"/>
+      <c r="T10" s="28"/>
+      <c r="U10" s="28"/>
+      <c r="V10" s="28"/>
+      <c r="W10" s="28"/>
+      <c r="X10" s="28"/>
+      <c r="Y10" s="28"/>
+      <c r="Z10" s="28"/>
+      <c r="AA10" s="28"/>
+      <c r="AB10" s="28"/>
+      <c r="AC10" s="28"/>
+      <c r="AD10" s="28"/>
+      <c r="AE10" s="28"/>
+      <c r="AF10" s="28"/>
+      <c r="AG10" s="29"/>
+    </row>
+    <row r="11" spans="1:33" s="3" customFormat="1" ht="15">
+      <c r="A11" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="B10" s="43" t="s">
+      <c r="B11" s="44" t="s">
         <v>35</v>
       </c>
-      <c r="C10" s="44"/>
-      <c r="D10" s="44"/>
-      <c r="E10" s="44"/>
-      <c r="F10" s="44"/>
-      <c r="G10" s="44"/>
-      <c r="H10" s="44"/>
-      <c r="I10" s="44"/>
-      <c r="J10" s="44"/>
-      <c r="K10" s="44"/>
-      <c r="L10" s="44"/>
-      <c r="M10" s="44"/>
-      <c r="N10" s="44"/>
-      <c r="O10" s="44"/>
-      <c r="P10" s="44"/>
-      <c r="Q10" s="44"/>
-      <c r="R10" s="44"/>
-      <c r="S10" s="44"/>
-      <c r="T10" s="44"/>
-      <c r="U10" s="44"/>
-      <c r="V10" s="30"/>
-      <c r="W10" s="30"/>
-      <c r="X10" s="30"/>
-      <c r="Y10" s="30"/>
-      <c r="Z10" s="30"/>
-      <c r="AA10" s="30"/>
-      <c r="AB10" s="30"/>
-      <c r="AC10" s="30"/>
-      <c r="AD10" s="30"/>
-      <c r="AE10" s="30"/>
-      <c r="AF10" s="30"/>
-      <c r="AG10" s="31"/>
-    </row>
-    <row r="11" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A11" s="11" t="s">
+      <c r="C11" s="45"/>
+      <c r="D11" s="45"/>
+      <c r="E11" s="45"/>
+      <c r="F11" s="45"/>
+      <c r="G11" s="45"/>
+      <c r="H11" s="45"/>
+      <c r="I11" s="45"/>
+      <c r="J11" s="45"/>
+      <c r="K11" s="45"/>
+      <c r="L11" s="45"/>
+      <c r="M11" s="45"/>
+      <c r="N11" s="45"/>
+      <c r="O11" s="45"/>
+      <c r="P11" s="45"/>
+      <c r="Q11" s="45"/>
+      <c r="R11" s="45"/>
+      <c r="S11" s="45"/>
+      <c r="T11" s="45"/>
+      <c r="U11" s="45"/>
+      <c r="V11" s="30"/>
+      <c r="W11" s="30"/>
+      <c r="X11" s="30"/>
+      <c r="Y11" s="30"/>
+      <c r="Z11" s="30"/>
+      <c r="AA11" s="30"/>
+      <c r="AB11" s="30"/>
+      <c r="AC11" s="30"/>
+      <c r="AD11" s="30"/>
+      <c r="AE11" s="30"/>
+      <c r="AF11" s="30"/>
+      <c r="AG11" s="31"/>
+    </row>
+    <row r="12" spans="1:33" ht="15">
+      <c r="A12" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="B11" s="4">
+      <c r="B12" s="4">
         <v>55</v>
       </c>
-      <c r="C11" s="4">
+      <c r="C12" s="4">
         <v>54</v>
       </c>
-      <c r="D11" s="4">
+      <c r="D12" s="4">
         <v>53</v>
       </c>
-      <c r="E11" s="4">
+      <c r="E12" s="4">
         <v>52</v>
       </c>
-      <c r="F11" s="4">
+      <c r="F12" s="4">
         <v>51</v>
       </c>
-      <c r="G11" s="4">
+      <c r="G12" s="4">
         <v>61</v>
       </c>
-      <c r="H11" s="4">
+      <c r="H12" s="4">
         <v>62</v>
       </c>
-      <c r="I11" s="4">
+      <c r="I12" s="4">
         <v>63</v>
       </c>
-      <c r="J11" s="4">
+      <c r="J12" s="4">
         <v>64</v>
       </c>
-      <c r="K11" s="4">
+      <c r="K12" s="4">
         <v>65</v>
       </c>
-      <c r="L11" s="4">
+      <c r="L12" s="4">
         <v>75</v>
       </c>
-      <c r="M11" s="4">
+      <c r="M12" s="4">
         <v>74</v>
       </c>
-      <c r="N11" s="4">
+      <c r="N12" s="4">
         <v>73</v>
       </c>
-      <c r="O11" s="4">
+      <c r="O12" s="4">
         <v>72</v>
       </c>
-      <c r="P11" s="4">
+      <c r="P12" s="4">
         <v>71</v>
       </c>
-      <c r="Q11" s="4">
+      <c r="Q12" s="4">
         <v>81</v>
       </c>
-      <c r="R11" s="4">
+      <c r="R12" s="4">
         <v>82</v>
       </c>
-      <c r="S11" s="4">
+      <c r="S12" s="4">
         <v>83</v>
       </c>
-      <c r="T11" s="4">
+      <c r="T12" s="4">
         <v>84</v>
       </c>
-      <c r="U11" s="4">
+      <c r="U12" s="4">
         <v>85</v>
       </c>
-      <c r="V11" s="32"/>
-      <c r="W11" s="32"/>
-      <c r="X11" s="32"/>
-      <c r="Y11" s="32"/>
-      <c r="Z11" s="32"/>
-      <c r="AA11" s="32"/>
-      <c r="AB11" s="32"/>
-      <c r="AC11" s="32"/>
-      <c r="AD11" s="32"/>
-      <c r="AE11" s="32"/>
-      <c r="AF11" s="32"/>
-      <c r="AG11" s="33"/>
-    </row>
-    <row r="12" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A12" s="13" t="s">
+      <c r="V12" s="32"/>
+      <c r="W12" s="32"/>
+      <c r="X12" s="32"/>
+      <c r="Y12" s="32"/>
+      <c r="Z12" s="32"/>
+      <c r="AA12" s="32"/>
+      <c r="AB12" s="32"/>
+      <c r="AC12" s="32"/>
+      <c r="AD12" s="32"/>
+      <c r="AE12" s="32"/>
+      <c r="AF12" s="32"/>
+      <c r="AG12" s="33"/>
+    </row>
+    <row r="13" spans="1:33" ht="15">
+      <c r="A13" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="B12" s="6"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
-      <c r="H12" s="6"/>
-      <c r="I12" s="6"/>
-      <c r="J12" s="6"/>
-      <c r="K12" s="6"/>
-      <c r="L12" s="6"/>
-      <c r="M12" s="6"/>
-      <c r="N12" s="6"/>
-      <c r="O12" s="6"/>
-      <c r="P12" s="6"/>
-      <c r="Q12" s="6"/>
-      <c r="R12" s="6"/>
-      <c r="S12" s="6"/>
-      <c r="T12" s="6"/>
-      <c r="U12" s="6"/>
-      <c r="V12" s="34"/>
-      <c r="W12" s="34"/>
-      <c r="X12" s="34"/>
-      <c r="Y12" s="34"/>
-      <c r="Z12" s="34"/>
-      <c r="AA12" s="34"/>
-      <c r="AB12" s="34"/>
-      <c r="AC12" s="34"/>
-      <c r="AD12" s="34"/>
-      <c r="AE12" s="34"/>
-      <c r="AF12" s="34"/>
-      <c r="AG12" s="35"/>
-    </row>
-    <row r="13" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A13" s="17" t="s">
-        <v>29</v>
-      </c>
-      <c r="B13" s="5"/>
-      <c r="C13" s="5"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-      <c r="F13" s="5"/>
-      <c r="G13" s="5"/>
-      <c r="H13" s="5"/>
-      <c r="I13" s="5"/>
-      <c r="J13" s="5"/>
-      <c r="K13" s="5"/>
-      <c r="L13" s="5"/>
-      <c r="M13" s="5"/>
-      <c r="N13" s="5"/>
-      <c r="O13" s="5"/>
-      <c r="P13" s="5"/>
-      <c r="Q13" s="5"/>
-      <c r="R13" s="5"/>
-      <c r="S13" s="5"/>
-      <c r="T13" s="5"/>
-      <c r="U13" s="5"/>
+      <c r="B13" s="6"/>
+      <c r="C13" s="6"/>
+      <c r="D13" s="6"/>
+      <c r="E13" s="6"/>
+      <c r="F13" s="6"/>
+      <c r="G13" s="6"/>
+      <c r="H13" s="6"/>
+      <c r="I13" s="6"/>
+      <c r="J13" s="6"/>
+      <c r="K13" s="6"/>
+      <c r="L13" s="6"/>
+      <c r="M13" s="6"/>
+      <c r="N13" s="6"/>
+      <c r="O13" s="6"/>
+      <c r="P13" s="6"/>
+      <c r="Q13" s="6"/>
+      <c r="R13" s="6"/>
+      <c r="S13" s="6"/>
+      <c r="T13" s="6"/>
+      <c r="U13" s="6"/>
       <c r="V13" s="34"/>
       <c r="W13" s="34"/>
       <c r="X13" s="34"/>
@@ -1775,30 +1783,30 @@
       <c r="AF13" s="34"/>
       <c r="AG13" s="35"/>
     </row>
-    <row r="14" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A14" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
-      <c r="F14" s="1"/>
-      <c r="G14" s="1"/>
-      <c r="H14" s="1"/>
-      <c r="I14" s="1"/>
-      <c r="J14" s="1"/>
-      <c r="K14" s="1"/>
-      <c r="L14" s="1"/>
-      <c r="M14" s="1"/>
-      <c r="N14" s="1"/>
-      <c r="O14" s="1"/>
-      <c r="P14" s="1"/>
-      <c r="Q14" s="1"/>
-      <c r="R14" s="1"/>
-      <c r="S14" s="1"/>
-      <c r="T14" s="1"/>
-      <c r="U14" s="1"/>
+    <row r="14" spans="1:33" ht="15">
+      <c r="A14" s="52" t="s">
+        <v>37</v>
+      </c>
+      <c r="B14" s="53"/>
+      <c r="C14" s="53"/>
+      <c r="D14" s="53"/>
+      <c r="E14" s="53"/>
+      <c r="F14" s="53"/>
+      <c r="G14" s="53"/>
+      <c r="H14" s="53"/>
+      <c r="I14" s="53"/>
+      <c r="J14" s="53"/>
+      <c r="K14" s="53"/>
+      <c r="L14" s="53"/>
+      <c r="M14" s="53"/>
+      <c r="N14" s="53"/>
+      <c r="O14" s="53"/>
+      <c r="P14" s="53"/>
+      <c r="Q14" s="53"/>
+      <c r="R14" s="53"/>
+      <c r="S14" s="53"/>
+      <c r="T14" s="53"/>
+      <c r="U14" s="53"/>
       <c r="V14" s="34"/>
       <c r="W14" s="34"/>
       <c r="X14" s="34"/>
@@ -1812,30 +1820,30 @@
       <c r="AF14" s="34"/>
       <c r="AG14" s="35"/>
     </row>
-    <row r="15" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A15" s="19" t="s">
-        <v>30</v>
-      </c>
-      <c r="B15" s="7"/>
-      <c r="C15" s="7"/>
-      <c r="D15" s="7"/>
-      <c r="E15" s="7"/>
-      <c r="F15" s="7"/>
-      <c r="G15" s="7"/>
-      <c r="H15" s="7"/>
-      <c r="I15" s="7"/>
-      <c r="J15" s="7"/>
-      <c r="K15" s="7"/>
-      <c r="L15" s="7"/>
-      <c r="M15" s="7"/>
-      <c r="N15" s="7"/>
-      <c r="O15" s="7"/>
-      <c r="P15" s="7"/>
-      <c r="Q15" s="7"/>
-      <c r="R15" s="7"/>
-      <c r="S15" s="7"/>
-      <c r="T15" s="7"/>
-      <c r="U15" s="7"/>
+    <row r="15" spans="1:33" ht="15">
+      <c r="A15" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" s="5"/>
+      <c r="C15" s="5"/>
+      <c r="D15" s="5"/>
+      <c r="E15" s="5"/>
+      <c r="F15" s="5"/>
+      <c r="G15" s="5"/>
+      <c r="H15" s="5"/>
+      <c r="I15" s="5"/>
+      <c r="J15" s="5"/>
+      <c r="K15" s="5"/>
+      <c r="L15" s="5"/>
+      <c r="M15" s="5"/>
+      <c r="N15" s="5"/>
+      <c r="O15" s="5"/>
+      <c r="P15" s="5"/>
+      <c r="Q15" s="5"/>
+      <c r="R15" s="5"/>
+      <c r="S15" s="5"/>
+      <c r="T15" s="5"/>
+      <c r="U15" s="5"/>
       <c r="V15" s="34"/>
       <c r="W15" s="34"/>
       <c r="X15" s="34"/>
@@ -1849,653 +1857,653 @@
       <c r="AF15" s="34"/>
       <c r="AG15" s="35"/>
     </row>
-    <row r="16" spans="1:33" s="8" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="38"/>
-      <c r="B16" s="39"/>
-      <c r="C16" s="39"/>
-      <c r="D16" s="39"/>
-      <c r="E16" s="39"/>
-      <c r="F16" s="39"/>
-      <c r="G16" s="39"/>
-      <c r="H16" s="39"/>
-      <c r="I16" s="39"/>
-      <c r="J16" s="39"/>
-      <c r="K16" s="39"/>
-      <c r="L16" s="39"/>
-      <c r="M16" s="39"/>
-      <c r="N16" s="39"/>
-      <c r="O16" s="39"/>
-      <c r="P16" s="39"/>
-      <c r="Q16" s="39"/>
-      <c r="R16" s="39"/>
-      <c r="S16" s="39"/>
-      <c r="T16" s="39"/>
-      <c r="U16" s="39"/>
-      <c r="V16" s="39"/>
-      <c r="W16" s="39"/>
-      <c r="X16" s="39"/>
-      <c r="Y16" s="39"/>
-      <c r="Z16" s="39"/>
-      <c r="AA16" s="39"/>
-      <c r="AB16" s="39"/>
-      <c r="AC16" s="39"/>
-      <c r="AD16" s="39"/>
-      <c r="AE16" s="39"/>
-      <c r="AF16" s="39"/>
-      <c r="AG16" s="40"/>
-    </row>
-    <row r="17" spans="1:33" s="24" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="18" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A18" s="9" t="s">
+    <row r="16" spans="1:33" ht="15">
+      <c r="A16" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="B16" s="1"/>
+      <c r="C16" s="1"/>
+      <c r="D16" s="1"/>
+      <c r="E16" s="1"/>
+      <c r="F16" s="1"/>
+      <c r="G16" s="1"/>
+      <c r="H16" s="1"/>
+      <c r="I16" s="1"/>
+      <c r="J16" s="1"/>
+      <c r="K16" s="1"/>
+      <c r="L16" s="1"/>
+      <c r="M16" s="1"/>
+      <c r="N16" s="1"/>
+      <c r="O16" s="1"/>
+      <c r="P16" s="1"/>
+      <c r="Q16" s="1"/>
+      <c r="R16" s="1"/>
+      <c r="S16" s="1"/>
+      <c r="T16" s="1"/>
+      <c r="U16" s="1"/>
+      <c r="V16" s="34"/>
+      <c r="W16" s="34"/>
+      <c r="X16" s="34"/>
+      <c r="Y16" s="34"/>
+      <c r="Z16" s="34"/>
+      <c r="AA16" s="34"/>
+      <c r="AB16" s="34"/>
+      <c r="AC16" s="34"/>
+      <c r="AD16" s="34"/>
+      <c r="AE16" s="34"/>
+      <c r="AF16" s="34"/>
+      <c r="AG16" s="35"/>
+    </row>
+    <row r="17" spans="1:33" ht="15">
+      <c r="A17" s="19" t="s">
+        <v>30</v>
+      </c>
+      <c r="B17" s="7"/>
+      <c r="C17" s="7"/>
+      <c r="D17" s="7"/>
+      <c r="E17" s="7"/>
+      <c r="F17" s="7"/>
+      <c r="G17" s="7"/>
+      <c r="H17" s="7"/>
+      <c r="I17" s="7"/>
+      <c r="J17" s="7"/>
+      <c r="K17" s="7"/>
+      <c r="L17" s="7"/>
+      <c r="M17" s="7"/>
+      <c r="N17" s="7"/>
+      <c r="O17" s="7"/>
+      <c r="P17" s="7"/>
+      <c r="Q17" s="7"/>
+      <c r="R17" s="7"/>
+      <c r="S17" s="7"/>
+      <c r="T17" s="7"/>
+      <c r="U17" s="7"/>
+      <c r="V17" s="34"/>
+      <c r="W17" s="34"/>
+      <c r="X17" s="34"/>
+      <c r="Y17" s="34"/>
+      <c r="Z17" s="34"/>
+      <c r="AA17" s="34"/>
+      <c r="AB17" s="34"/>
+      <c r="AC17" s="34"/>
+      <c r="AD17" s="34"/>
+      <c r="AE17" s="34"/>
+      <c r="AF17" s="34"/>
+      <c r="AG17" s="35"/>
+    </row>
+    <row r="18" spans="1:33" s="8" customFormat="1" ht="15" customHeight="1" thickBot="1">
+      <c r="A18" s="38"/>
+      <c r="B18" s="39"/>
+      <c r="C18" s="39"/>
+      <c r="D18" s="39"/>
+      <c r="E18" s="39"/>
+      <c r="F18" s="39"/>
+      <c r="G18" s="39"/>
+      <c r="H18" s="39"/>
+      <c r="I18" s="39"/>
+      <c r="J18" s="39"/>
+      <c r="K18" s="39"/>
+      <c r="L18" s="39"/>
+      <c r="M18" s="39"/>
+      <c r="N18" s="39"/>
+      <c r="O18" s="39"/>
+      <c r="P18" s="39"/>
+      <c r="Q18" s="39"/>
+      <c r="R18" s="39"/>
+      <c r="S18" s="39"/>
+      <c r="T18" s="39"/>
+      <c r="U18" s="39"/>
+      <c r="V18" s="39"/>
+      <c r="W18" s="39"/>
+      <c r="X18" s="39"/>
+      <c r="Y18" s="39"/>
+      <c r="Z18" s="39"/>
+      <c r="AA18" s="39"/>
+      <c r="AB18" s="39"/>
+      <c r="AC18" s="39"/>
+      <c r="AD18" s="39"/>
+      <c r="AE18" s="39"/>
+      <c r="AF18" s="39"/>
+      <c r="AG18" s="40"/>
+    </row>
+    <row r="19" spans="1:33" s="24" customFormat="1" ht="15" thickBot="1"/>
+    <row r="20" spans="1:33" ht="15">
+      <c r="A20" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="B18" s="36"/>
-      <c r="C18" s="36"/>
-      <c r="D18" s="36"/>
-      <c r="E18" s="36"/>
-      <c r="F18" s="36"/>
-      <c r="G18" s="36"/>
-      <c r="H18" s="36"/>
-      <c r="I18" s="36"/>
-      <c r="J18" s="36"/>
-      <c r="K18" s="36"/>
-      <c r="L18" s="36"/>
-      <c r="M18" s="36"/>
-      <c r="N18" s="36"/>
-      <c r="O18" s="36"/>
-      <c r="P18" s="36"/>
-      <c r="Q18" s="36"/>
-      <c r="R18" s="36"/>
-      <c r="S18" s="36"/>
-      <c r="T18" s="36"/>
-      <c r="U18" s="36"/>
-      <c r="V18" s="36"/>
-      <c r="W18" s="36"/>
-      <c r="X18" s="36"/>
-      <c r="Y18" s="36"/>
-      <c r="Z18" s="36"/>
-      <c r="AA18" s="36"/>
-      <c r="AB18" s="36"/>
-      <c r="AC18" s="36"/>
-      <c r="AD18" s="36"/>
-      <c r="AE18" s="36"/>
-      <c r="AF18" s="36"/>
-      <c r="AG18" s="37"/>
-    </row>
-    <row r="19" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A19" s="10" t="s">
+      <c r="B20" s="36"/>
+      <c r="C20" s="36"/>
+      <c r="D20" s="36"/>
+      <c r="E20" s="36"/>
+      <c r="F20" s="36"/>
+      <c r="G20" s="36"/>
+      <c r="H20" s="36"/>
+      <c r="I20" s="36"/>
+      <c r="J20" s="36"/>
+      <c r="K20" s="36"/>
+      <c r="L20" s="36"/>
+      <c r="M20" s="36"/>
+      <c r="N20" s="36"/>
+      <c r="O20" s="36"/>
+      <c r="P20" s="36"/>
+      <c r="Q20" s="36"/>
+      <c r="R20" s="36"/>
+      <c r="S20" s="36"/>
+      <c r="T20" s="36"/>
+      <c r="U20" s="36"/>
+      <c r="V20" s="36"/>
+      <c r="W20" s="36"/>
+      <c r="X20" s="36"/>
+      <c r="Y20" s="36"/>
+      <c r="Z20" s="36"/>
+      <c r="AA20" s="36"/>
+      <c r="AB20" s="36"/>
+      <c r="AC20" s="36"/>
+      <c r="AD20" s="36"/>
+      <c r="AE20" s="36"/>
+      <c r="AF20" s="36"/>
+      <c r="AG20" s="37"/>
+    </row>
+    <row r="21" spans="1:33">
+      <c r="A21" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="B19" s="48" t="s">
+      <c r="B21" s="49" t="s">
         <v>34</v>
       </c>
-      <c r="C19" s="49"/>
-      <c r="D19" s="49"/>
-      <c r="E19" s="49"/>
-      <c r="F19" s="49"/>
-      <c r="G19" s="49"/>
-      <c r="H19" s="49"/>
-      <c r="I19" s="49"/>
-      <c r="J19" s="49"/>
-      <c r="K19" s="49"/>
-      <c r="L19" s="49"/>
-      <c r="M19" s="49"/>
-      <c r="N19" s="49"/>
-      <c r="O19" s="49"/>
-      <c r="P19" s="49"/>
-      <c r="Q19" s="49"/>
-      <c r="R19" s="49"/>
-      <c r="S19" s="49"/>
-      <c r="T19" s="49"/>
-      <c r="U19" s="49"/>
-      <c r="V19" s="49"/>
-      <c r="W19" s="49"/>
-      <c r="X19" s="49"/>
-      <c r="Y19" s="49"/>
-      <c r="Z19" s="49"/>
-      <c r="AA19" s="49"/>
-      <c r="AB19" s="49"/>
-      <c r="AC19" s="49"/>
-      <c r="AD19" s="49"/>
-      <c r="AE19" s="49"/>
-      <c r="AF19" s="49"/>
-      <c r="AG19" s="50"/>
-    </row>
-    <row r="20" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A20" s="11" t="s">
+      <c r="C21" s="50"/>
+      <c r="D21" s="50"/>
+      <c r="E21" s="50"/>
+      <c r="F21" s="50"/>
+      <c r="G21" s="50"/>
+      <c r="H21" s="50"/>
+      <c r="I21" s="50"/>
+      <c r="J21" s="50"/>
+      <c r="K21" s="50"/>
+      <c r="L21" s="50"/>
+      <c r="M21" s="50"/>
+      <c r="N21" s="50"/>
+      <c r="O21" s="50"/>
+      <c r="P21" s="50"/>
+      <c r="Q21" s="50"/>
+      <c r="R21" s="50"/>
+      <c r="S21" s="50"/>
+      <c r="T21" s="50"/>
+      <c r="U21" s="50"/>
+      <c r="V21" s="50"/>
+      <c r="W21" s="50"/>
+      <c r="X21" s="50"/>
+      <c r="Y21" s="50"/>
+      <c r="Z21" s="50"/>
+      <c r="AA21" s="50"/>
+      <c r="AB21" s="50"/>
+      <c r="AC21" s="50"/>
+      <c r="AD21" s="50"/>
+      <c r="AE21" s="50"/>
+      <c r="AF21" s="50"/>
+      <c r="AG21" s="51"/>
+    </row>
+    <row r="22" spans="1:33" ht="15">
+      <c r="A22" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="B20" s="4">
+      <c r="B22" s="4">
         <v>1</v>
       </c>
-      <c r="C20" s="4">
+      <c r="C22" s="4">
         <v>2</v>
       </c>
-      <c r="D20" s="4">
+      <c r="D22" s="4">
         <v>3</v>
       </c>
-      <c r="E20" s="4">
+      <c r="E22" s="4">
         <v>4</v>
       </c>
-      <c r="F20" s="4">
+      <c r="F22" s="4">
         <v>5</v>
       </c>
-      <c r="G20" s="4">
+      <c r="G22" s="4">
         <v>6</v>
       </c>
-      <c r="H20" s="4">
+      <c r="H22" s="4">
         <v>7</v>
       </c>
-      <c r="I20" s="4">
+      <c r="I22" s="4">
         <v>8</v>
       </c>
-      <c r="J20" s="4">
+      <c r="J22" s="4">
         <v>9</v>
       </c>
-      <c r="K20" s="4">
+      <c r="K22" s="4">
         <v>10</v>
       </c>
-      <c r="L20" s="4">
+      <c r="L22" s="4">
         <v>11</v>
       </c>
-      <c r="M20" s="4">
+      <c r="M22" s="4">
         <v>12</v>
       </c>
-      <c r="N20" s="4">
+      <c r="N22" s="4">
         <v>13</v>
       </c>
-      <c r="O20" s="4">
+      <c r="O22" s="4">
         <v>14</v>
       </c>
-      <c r="P20" s="4">
+      <c r="P22" s="4">
         <v>15</v>
       </c>
-      <c r="Q20" s="4">
+      <c r="Q22" s="4">
         <v>16</v>
       </c>
-      <c r="R20" s="4">
+      <c r="R22" s="4">
         <v>17</v>
       </c>
-      <c r="S20" s="4">
+      <c r="S22" s="4">
         <v>18</v>
       </c>
-      <c r="T20" s="4">
+      <c r="T22" s="4">
         <v>19</v>
       </c>
-      <c r="U20" s="4">
+      <c r="U22" s="4">
         <v>20</v>
       </c>
-      <c r="V20" s="4">
+      <c r="V22" s="4">
         <v>21</v>
       </c>
-      <c r="W20" s="4">
+      <c r="W22" s="4">
         <v>22</v>
       </c>
-      <c r="X20" s="4">
+      <c r="X22" s="4">
         <v>23</v>
       </c>
-      <c r="Y20" s="4">
+      <c r="Y22" s="4">
         <v>24</v>
       </c>
-      <c r="Z20" s="4">
+      <c r="Z22" s="4">
         <v>25</v>
       </c>
-      <c r="AA20" s="4">
+      <c r="AA22" s="4">
         <v>26</v>
       </c>
-      <c r="AB20" s="4">
+      <c r="AB22" s="4">
         <v>27</v>
       </c>
-      <c r="AC20" s="4">
+      <c r="AC22" s="4">
         <v>28</v>
       </c>
-      <c r="AD20" s="4">
+      <c r="AD22" s="4">
         <v>29</v>
       </c>
-      <c r="AE20" s="4">
+      <c r="AE22" s="4">
         <v>30</v>
       </c>
-      <c r="AF20" s="4">
+      <c r="AF22" s="4">
         <v>31</v>
       </c>
-      <c r="AG20" s="4">
+      <c r="AG22" s="4">
         <v>32</v>
       </c>
     </row>
-    <row r="21" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A21" s="13" t="s">
+    <row r="23" spans="1:33" ht="15">
+      <c r="A23" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="B21" s="6"/>
-      <c r="C21" s="6"/>
-      <c r="D21" s="6"/>
-      <c r="E21" s="6"/>
-      <c r="F21" s="6"/>
-      <c r="G21" s="6"/>
-      <c r="H21" s="6"/>
-      <c r="I21" s="6"/>
-      <c r="J21" s="6"/>
-      <c r="K21" s="6"/>
-      <c r="L21" s="6"/>
-      <c r="M21" s="6"/>
-      <c r="N21" s="6"/>
-      <c r="O21" s="6"/>
-      <c r="P21" s="6"/>
-      <c r="Q21" s="6"/>
-      <c r="R21" s="6"/>
-      <c r="S21" s="6"/>
-      <c r="T21" s="6"/>
-      <c r="U21" s="6"/>
-      <c r="V21" s="6"/>
-      <c r="W21" s="6"/>
-      <c r="X21" s="6"/>
-      <c r="Y21" s="6"/>
-      <c r="Z21" s="6"/>
-      <c r="AA21" s="6"/>
-      <c r="AB21" s="6"/>
-      <c r="AC21" s="6"/>
-      <c r="AD21" s="6"/>
-      <c r="AE21" s="6"/>
-      <c r="AF21" s="6"/>
-      <c r="AG21" s="14"/>
-    </row>
-    <row r="22" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A22" s="17" t="s">
+      <c r="B23" s="6"/>
+      <c r="C23" s="6"/>
+      <c r="D23" s="6"/>
+      <c r="E23" s="6"/>
+      <c r="F23" s="6"/>
+      <c r="G23" s="6"/>
+      <c r="H23" s="6"/>
+      <c r="I23" s="6"/>
+      <c r="J23" s="6"/>
+      <c r="K23" s="6"/>
+      <c r="L23" s="6"/>
+      <c r="M23" s="6"/>
+      <c r="N23" s="6"/>
+      <c r="O23" s="6"/>
+      <c r="P23" s="6"/>
+      <c r="Q23" s="6"/>
+      <c r="R23" s="6"/>
+      <c r="S23" s="6"/>
+      <c r="T23" s="6"/>
+      <c r="U23" s="6"/>
+      <c r="V23" s="6"/>
+      <c r="W23" s="6"/>
+      <c r="X23" s="6"/>
+      <c r="Y23" s="6"/>
+      <c r="Z23" s="6"/>
+      <c r="AA23" s="6"/>
+      <c r="AB23" s="6"/>
+      <c r="AC23" s="6"/>
+      <c r="AD23" s="6"/>
+      <c r="AE23" s="6"/>
+      <c r="AF23" s="6"/>
+      <c r="AG23" s="14"/>
+    </row>
+    <row r="24" spans="1:33" ht="15">
+      <c r="A24" s="52" t="s">
+        <v>36</v>
+      </c>
+      <c r="B24" s="53"/>
+      <c r="C24" s="53"/>
+      <c r="D24" s="53"/>
+      <c r="E24" s="53"/>
+      <c r="F24" s="53"/>
+      <c r="G24" s="53"/>
+      <c r="H24" s="53"/>
+      <c r="I24" s="53"/>
+      <c r="J24" s="53"/>
+      <c r="K24" s="53"/>
+      <c r="L24" s="53"/>
+      <c r="M24" s="53"/>
+      <c r="N24" s="53"/>
+      <c r="O24" s="53"/>
+      <c r="P24" s="53"/>
+      <c r="Q24" s="53"/>
+      <c r="R24" s="53"/>
+      <c r="S24" s="53"/>
+      <c r="T24" s="53"/>
+      <c r="U24" s="53"/>
+      <c r="V24" s="53"/>
+      <c r="W24" s="53"/>
+      <c r="X24" s="53"/>
+      <c r="Y24" s="53"/>
+      <c r="Z24" s="53"/>
+      <c r="AA24" s="53"/>
+      <c r="AB24" s="53"/>
+      <c r="AC24" s="53"/>
+      <c r="AD24" s="53"/>
+      <c r="AE24" s="53"/>
+      <c r="AF24" s="53"/>
+      <c r="AG24" s="54"/>
+    </row>
+    <row r="25" spans="1:33" ht="15">
+      <c r="A25" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="B22" s="5"/>
-      <c r="C22" s="5"/>
-      <c r="D22" s="5"/>
-      <c r="E22" s="5"/>
-      <c r="F22" s="5"/>
-      <c r="G22" s="5"/>
-      <c r="H22" s="5"/>
-      <c r="I22" s="5"/>
-      <c r="J22" s="5"/>
-      <c r="K22" s="5"/>
-      <c r="L22" s="5"/>
-      <c r="M22" s="5"/>
-      <c r="N22" s="5"/>
-      <c r="O22" s="5"/>
-      <c r="P22" s="5"/>
-      <c r="Q22" s="5"/>
-      <c r="R22" s="5"/>
-      <c r="S22" s="5"/>
-      <c r="T22" s="5"/>
-      <c r="U22" s="5"/>
-      <c r="V22" s="5"/>
-      <c r="W22" s="5"/>
-      <c r="X22" s="5"/>
-      <c r="Y22" s="5"/>
-      <c r="Z22" s="5"/>
-      <c r="AA22" s="5"/>
-      <c r="AB22" s="5"/>
-      <c r="AC22" s="5"/>
-      <c r="AD22" s="5"/>
-      <c r="AE22" s="5"/>
-      <c r="AF22" s="5"/>
-      <c r="AG22" s="18"/>
-    </row>
-    <row r="23" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A23" s="15" t="s">
+      <c r="B25" s="5"/>
+      <c r="C25" s="5"/>
+      <c r="D25" s="5"/>
+      <c r="E25" s="5"/>
+      <c r="F25" s="5"/>
+      <c r="G25" s="5"/>
+      <c r="H25" s="5"/>
+      <c r="I25" s="5"/>
+      <c r="J25" s="5"/>
+      <c r="K25" s="5"/>
+      <c r="L25" s="5"/>
+      <c r="M25" s="5"/>
+      <c r="N25" s="5"/>
+      <c r="O25" s="5"/>
+      <c r="P25" s="5"/>
+      <c r="Q25" s="5"/>
+      <c r="R25" s="5"/>
+      <c r="S25" s="5"/>
+      <c r="T25" s="5"/>
+      <c r="U25" s="5"/>
+      <c r="V25" s="5"/>
+      <c r="W25" s="5"/>
+      <c r="X25" s="5"/>
+      <c r="Y25" s="5"/>
+      <c r="Z25" s="5"/>
+      <c r="AA25" s="5"/>
+      <c r="AB25" s="5"/>
+      <c r="AC25" s="5"/>
+      <c r="AD25" s="5"/>
+      <c r="AE25" s="5"/>
+      <c r="AF25" s="5"/>
+      <c r="AG25" s="18"/>
+    </row>
+    <row r="26" spans="1:33" ht="15">
+      <c r="A26" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B23" s="1"/>
-      <c r="C23" s="1"/>
-      <c r="D23" s="1"/>
-      <c r="E23" s="1"/>
-      <c r="F23" s="1"/>
-      <c r="G23" s="1"/>
-      <c r="H23" s="1"/>
-      <c r="I23" s="1"/>
-      <c r="J23" s="1"/>
-      <c r="K23" s="1"/>
-      <c r="L23" s="1"/>
-      <c r="M23" s="1"/>
-      <c r="N23" s="1"/>
-      <c r="O23" s="1"/>
-      <c r="P23" s="1"/>
-      <c r="Q23" s="1"/>
-      <c r="R23" s="1"/>
-      <c r="S23" s="1"/>
-      <c r="T23" s="1"/>
-      <c r="U23" s="1"/>
-      <c r="V23" s="1"/>
-      <c r="W23" s="1"/>
-      <c r="X23" s="1"/>
-      <c r="Y23" s="1"/>
-      <c r="Z23" s="1"/>
-      <c r="AA23" s="1"/>
-      <c r="AB23" s="1"/>
-      <c r="AC23" s="1"/>
-      <c r="AD23" s="1"/>
-      <c r="AE23" s="1"/>
-      <c r="AF23" s="1"/>
-      <c r="AG23" s="16"/>
-    </row>
-    <row r="24" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A24" s="19" t="s">
+      <c r="B26" s="1"/>
+      <c r="C26" s="1"/>
+      <c r="D26" s="1"/>
+      <c r="E26" s="1"/>
+      <c r="F26" s="1"/>
+      <c r="G26" s="1"/>
+      <c r="H26" s="1"/>
+      <c r="I26" s="1"/>
+      <c r="J26" s="1"/>
+      <c r="K26" s="1"/>
+      <c r="L26" s="1"/>
+      <c r="M26" s="1"/>
+      <c r="N26" s="1"/>
+      <c r="O26" s="1"/>
+      <c r="P26" s="1"/>
+      <c r="Q26" s="1"/>
+      <c r="R26" s="1"/>
+      <c r="S26" s="1"/>
+      <c r="T26" s="1"/>
+      <c r="U26" s="1"/>
+      <c r="V26" s="1"/>
+      <c r="W26" s="1"/>
+      <c r="X26" s="1"/>
+      <c r="Y26" s="1"/>
+      <c r="Z26" s="1"/>
+      <c r="AA26" s="1"/>
+      <c r="AB26" s="1"/>
+      <c r="AC26" s="1"/>
+      <c r="AD26" s="1"/>
+      <c r="AE26" s="1"/>
+      <c r="AF26" s="1"/>
+      <c r="AG26" s="16"/>
+    </row>
+    <row r="27" spans="1:33" ht="15">
+      <c r="A27" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="B24" s="7"/>
-      <c r="C24" s="7"/>
-      <c r="D24" s="7"/>
-      <c r="E24" s="7"/>
-      <c r="F24" s="7"/>
-      <c r="G24" s="7"/>
-      <c r="H24" s="7"/>
-      <c r="I24" s="7"/>
-      <c r="J24" s="7"/>
-      <c r="K24" s="7"/>
-      <c r="L24" s="7"/>
-      <c r="M24" s="7"/>
-      <c r="N24" s="7"/>
-      <c r="O24" s="7"/>
-      <c r="P24" s="7"/>
-      <c r="Q24" s="7"/>
-      <c r="R24" s="7"/>
-      <c r="S24" s="7"/>
-      <c r="T24" s="7"/>
-      <c r="U24" s="7"/>
-      <c r="V24" s="7"/>
-      <c r="W24" s="7"/>
-      <c r="X24" s="7"/>
-      <c r="Y24" s="7"/>
-      <c r="Z24" s="7"/>
-      <c r="AA24" s="7"/>
-      <c r="AB24" s="7"/>
-      <c r="AC24" s="7"/>
-      <c r="AD24" s="7"/>
-      <c r="AE24" s="7"/>
-      <c r="AF24" s="7"/>
-      <c r="AG24" s="20"/>
-    </row>
-    <row r="25" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A25" s="27"/>
-      <c r="B25" s="28"/>
-      <c r="C25" s="28"/>
-      <c r="D25" s="28"/>
-      <c r="E25" s="28"/>
-      <c r="F25" s="28"/>
-      <c r="G25" s="28"/>
-      <c r="H25" s="28"/>
-      <c r="I25" s="28"/>
-      <c r="J25" s="28"/>
-      <c r="K25" s="28"/>
-      <c r="L25" s="28"/>
-      <c r="M25" s="28"/>
-      <c r="N25" s="28"/>
-      <c r="O25" s="28"/>
-      <c r="P25" s="28"/>
-      <c r="Q25" s="28"/>
-      <c r="R25" s="28"/>
-      <c r="S25" s="28"/>
-      <c r="T25" s="28"/>
-      <c r="U25" s="28"/>
-      <c r="V25" s="28"/>
-      <c r="W25" s="28"/>
-      <c r="X25" s="28"/>
-      <c r="Y25" s="28"/>
-      <c r="Z25" s="28"/>
-      <c r="AA25" s="28"/>
-      <c r="AB25" s="28"/>
-      <c r="AC25" s="28"/>
-      <c r="AD25" s="28"/>
-      <c r="AE25" s="28"/>
-      <c r="AF25" s="28"/>
-      <c r="AG25" s="29"/>
-    </row>
-    <row r="26" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A26" s="21" t="s">
+      <c r="B27" s="7"/>
+      <c r="C27" s="7"/>
+      <c r="D27" s="7"/>
+      <c r="E27" s="7"/>
+      <c r="F27" s="7"/>
+      <c r="G27" s="7"/>
+      <c r="H27" s="7"/>
+      <c r="I27" s="7"/>
+      <c r="J27" s="7"/>
+      <c r="K27" s="7"/>
+      <c r="L27" s="7"/>
+      <c r="M27" s="7"/>
+      <c r="N27" s="7"/>
+      <c r="O27" s="7"/>
+      <c r="P27" s="7"/>
+      <c r="Q27" s="7"/>
+      <c r="R27" s="7"/>
+      <c r="S27" s="7"/>
+      <c r="T27" s="7"/>
+      <c r="U27" s="7"/>
+      <c r="V27" s="7"/>
+      <c r="W27" s="7"/>
+      <c r="X27" s="7"/>
+      <c r="Y27" s="7"/>
+      <c r="Z27" s="7"/>
+      <c r="AA27" s="7"/>
+      <c r="AB27" s="7"/>
+      <c r="AC27" s="7"/>
+      <c r="AD27" s="7"/>
+      <c r="AE27" s="7"/>
+      <c r="AF27" s="7"/>
+      <c r="AG27" s="20"/>
+    </row>
+    <row r="28" spans="1:33" ht="15">
+      <c r="A28" s="27"/>
+      <c r="B28" s="28"/>
+      <c r="C28" s="28"/>
+      <c r="D28" s="28"/>
+      <c r="E28" s="28"/>
+      <c r="F28" s="28"/>
+      <c r="G28" s="28"/>
+      <c r="H28" s="28"/>
+      <c r="I28" s="28"/>
+      <c r="J28" s="28"/>
+      <c r="K28" s="28"/>
+      <c r="L28" s="28"/>
+      <c r="M28" s="28"/>
+      <c r="N28" s="28"/>
+      <c r="O28" s="28"/>
+      <c r="P28" s="28"/>
+      <c r="Q28" s="28"/>
+      <c r="R28" s="28"/>
+      <c r="S28" s="28"/>
+      <c r="T28" s="28"/>
+      <c r="U28" s="28"/>
+      <c r="V28" s="28"/>
+      <c r="W28" s="28"/>
+      <c r="X28" s="28"/>
+      <c r="Y28" s="28"/>
+      <c r="Z28" s="28"/>
+      <c r="AA28" s="28"/>
+      <c r="AB28" s="28"/>
+      <c r="AC28" s="28"/>
+      <c r="AD28" s="28"/>
+      <c r="AE28" s="28"/>
+      <c r="AF28" s="28"/>
+      <c r="AG28" s="29"/>
+    </row>
+    <row r="29" spans="1:33" ht="15">
+      <c r="A29" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="B26" s="43" t="s">
+      <c r="B29" s="44" t="s">
         <v>35</v>
       </c>
-      <c r="C26" s="44"/>
-      <c r="D26" s="44"/>
-      <c r="E26" s="44"/>
-      <c r="F26" s="44"/>
-      <c r="G26" s="44"/>
-      <c r="H26" s="44"/>
-      <c r="I26" s="44"/>
-      <c r="J26" s="44"/>
-      <c r="K26" s="44"/>
-      <c r="L26" s="44"/>
-      <c r="M26" s="44"/>
-      <c r="N26" s="44"/>
-      <c r="O26" s="44"/>
-      <c r="P26" s="44"/>
-      <c r="Q26" s="44"/>
-      <c r="R26" s="44"/>
-      <c r="S26" s="44"/>
-      <c r="T26" s="44"/>
-      <c r="U26" s="44"/>
-      <c r="V26" s="30"/>
-      <c r="W26" s="30"/>
-      <c r="X26" s="30"/>
-      <c r="Y26" s="30"/>
-      <c r="Z26" s="30"/>
-      <c r="AA26" s="30"/>
-      <c r="AB26" s="30"/>
-      <c r="AC26" s="30"/>
-      <c r="AD26" s="30"/>
-      <c r="AE26" s="30"/>
-      <c r="AF26" s="30"/>
-      <c r="AG26" s="31"/>
-    </row>
-    <row r="27" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A27" s="11" t="s">
+      <c r="C29" s="45"/>
+      <c r="D29" s="45"/>
+      <c r="E29" s="45"/>
+      <c r="F29" s="45"/>
+      <c r="G29" s="45"/>
+      <c r="H29" s="45"/>
+      <c r="I29" s="45"/>
+      <c r="J29" s="45"/>
+      <c r="K29" s="45"/>
+      <c r="L29" s="45"/>
+      <c r="M29" s="45"/>
+      <c r="N29" s="45"/>
+      <c r="O29" s="45"/>
+      <c r="P29" s="45"/>
+      <c r="Q29" s="45"/>
+      <c r="R29" s="45"/>
+      <c r="S29" s="45"/>
+      <c r="T29" s="45"/>
+      <c r="U29" s="45"/>
+      <c r="V29" s="30"/>
+      <c r="W29" s="30"/>
+      <c r="X29" s="30"/>
+      <c r="Y29" s="30"/>
+      <c r="Z29" s="30"/>
+      <c r="AA29" s="30"/>
+      <c r="AB29" s="30"/>
+      <c r="AC29" s="30"/>
+      <c r="AD29" s="30"/>
+      <c r="AE29" s="30"/>
+      <c r="AF29" s="30"/>
+      <c r="AG29" s="31"/>
+    </row>
+    <row r="30" spans="1:33" ht="15">
+      <c r="A30" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="B27" s="4" t="s">
+      <c r="B30" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="C27" s="4" t="s">
+      <c r="C30" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D27" s="4" t="s">
+      <c r="D30" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="E27" s="4" t="s">
+      <c r="E30" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F27" s="4" t="s">
+      <c r="F30" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G27" s="4" t="s">
+      <c r="G30" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="H27" s="4" t="s">
+      <c r="H30" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="I27" s="4" t="s">
+      <c r="I30" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="J27" s="4" t="s">
+      <c r="J30" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="K27" s="4" t="s">
+      <c r="K30" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="L27" s="4" t="s">
+      <c r="L30" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="M27" s="4" t="s">
+      <c r="M30" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="N27" s="4" t="s">
+      <c r="N30" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="O27" s="4" t="s">
+      <c r="O30" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="P27" s="4" t="s">
+      <c r="P30" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="Q27" s="4" t="s">
+      <c r="Q30" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="R27" s="4" t="s">
+      <c r="R30" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="S27" s="4" t="s">
+      <c r="S30" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="T27" s="4" t="s">
+      <c r="T30" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="U27" s="4" t="s">
+      <c r="U30" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="V27" s="32"/>
-      <c r="W27" s="32"/>
-      <c r="X27" s="32"/>
-      <c r="Y27" s="32"/>
-      <c r="Z27" s="32"/>
-      <c r="AA27" s="32"/>
-      <c r="AB27" s="32"/>
-      <c r="AC27" s="32"/>
-      <c r="AD27" s="32"/>
-      <c r="AE27" s="32"/>
-      <c r="AF27" s="32"/>
-      <c r="AG27" s="33"/>
-    </row>
-    <row r="28" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A28" s="13" t="s">
+      <c r="V30" s="32"/>
+      <c r="W30" s="32"/>
+      <c r="X30" s="32"/>
+      <c r="Y30" s="32"/>
+      <c r="Z30" s="32"/>
+      <c r="AA30" s="32"/>
+      <c r="AB30" s="32"/>
+      <c r="AC30" s="32"/>
+      <c r="AD30" s="32"/>
+      <c r="AE30" s="32"/>
+      <c r="AF30" s="32"/>
+      <c r="AG30" s="33"/>
+    </row>
+    <row r="31" spans="1:33" ht="15">
+      <c r="A31" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="6"/>
-      <c r="C28" s="6"/>
-      <c r="D28" s="6"/>
-      <c r="E28" s="6"/>
-      <c r="F28" s="6"/>
-      <c r="G28" s="6"/>
-      <c r="H28" s="6"/>
-      <c r="I28" s="6"/>
-      <c r="J28" s="6"/>
-      <c r="K28" s="6"/>
-      <c r="L28" s="6"/>
-      <c r="M28" s="6"/>
-      <c r="N28" s="6"/>
-      <c r="O28" s="6"/>
-      <c r="P28" s="6"/>
-      <c r="Q28" s="6"/>
-      <c r="R28" s="6"/>
-      <c r="S28" s="6"/>
-      <c r="T28" s="6"/>
-      <c r="U28" s="6"/>
-      <c r="V28" s="34"/>
-      <c r="W28" s="34"/>
-      <c r="X28" s="34"/>
-      <c r="Y28" s="34"/>
-      <c r="Z28" s="34"/>
-      <c r="AA28" s="34"/>
-      <c r="AB28" s="34"/>
-      <c r="AC28" s="34"/>
-      <c r="AD28" s="34"/>
-      <c r="AE28" s="34"/>
-      <c r="AF28" s="34"/>
-      <c r="AG28" s="35"/>
-    </row>
-    <row r="29" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A29" s="17" t="s">
-        <v>29</v>
-      </c>
-      <c r="B29" s="5"/>
-      <c r="C29" s="5"/>
-      <c r="D29" s="5"/>
-      <c r="E29" s="5"/>
-      <c r="F29" s="5"/>
-      <c r="G29" s="5"/>
-      <c r="H29" s="5"/>
-      <c r="I29" s="5"/>
-      <c r="J29" s="5"/>
-      <c r="K29" s="5"/>
-      <c r="L29" s="5"/>
-      <c r="M29" s="5"/>
-      <c r="N29" s="5"/>
-      <c r="O29" s="5"/>
-      <c r="P29" s="5"/>
-      <c r="Q29" s="5"/>
-      <c r="R29" s="5"/>
-      <c r="S29" s="5"/>
-      <c r="T29" s="5"/>
-      <c r="U29" s="5"/>
-      <c r="V29" s="34"/>
-      <c r="W29" s="34"/>
-      <c r="X29" s="34"/>
-      <c r="Y29" s="34"/>
-      <c r="Z29" s="34"/>
-      <c r="AA29" s="34"/>
-      <c r="AB29" s="34"/>
-      <c r="AC29" s="34"/>
-      <c r="AD29" s="34"/>
-      <c r="AE29" s="34"/>
-      <c r="AF29" s="34"/>
-      <c r="AG29" s="35"/>
-    </row>
-    <row r="30" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A30" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="B30" s="1"/>
-      <c r="C30" s="1"/>
-      <c r="D30" s="1"/>
-      <c r="E30" s="1"/>
-      <c r="F30" s="1"/>
-      <c r="G30" s="1"/>
-      <c r="H30" s="1"/>
-      <c r="I30" s="1"/>
-      <c r="J30" s="1"/>
-      <c r="K30" s="1"/>
-      <c r="L30" s="1"/>
-      <c r="M30" s="1"/>
-      <c r="N30" s="1"/>
-      <c r="O30" s="1"/>
-      <c r="P30" s="1"/>
-      <c r="Q30" s="1"/>
-      <c r="R30" s="1"/>
-      <c r="S30" s="1"/>
-      <c r="T30" s="1"/>
-      <c r="U30" s="1"/>
-      <c r="V30" s="34"/>
-      <c r="W30" s="34"/>
-      <c r="X30" s="34"/>
-      <c r="Y30" s="34"/>
-      <c r="Z30" s="34"/>
-      <c r="AA30" s="34"/>
-      <c r="AB30" s="34"/>
-      <c r="AC30" s="34"/>
-      <c r="AD30" s="34"/>
-      <c r="AE30" s="34"/>
-      <c r="AF30" s="34"/>
-      <c r="AG30" s="35"/>
-    </row>
-    <row r="31" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A31" s="19" t="s">
-        <v>30</v>
-      </c>
-      <c r="B31" s="7"/>
-      <c r="C31" s="7"/>
-      <c r="D31" s="7"/>
-      <c r="E31" s="7"/>
-      <c r="F31" s="7"/>
-      <c r="G31" s="7"/>
-      <c r="H31" s="7"/>
-      <c r="I31" s="7"/>
-      <c r="J31" s="7"/>
-      <c r="K31" s="7"/>
-      <c r="L31" s="7"/>
-      <c r="M31" s="7"/>
-      <c r="N31" s="7"/>
-      <c r="O31" s="7"/>
-      <c r="P31" s="7"/>
-      <c r="Q31" s="7"/>
-      <c r="R31" s="7"/>
-      <c r="S31" s="7"/>
-      <c r="T31" s="7"/>
-      <c r="U31" s="7"/>
+      <c r="B31" s="6"/>
+      <c r="C31" s="6"/>
+      <c r="D31" s="6"/>
+      <c r="E31" s="6"/>
+      <c r="F31" s="6"/>
+      <c r="G31" s="6"/>
+      <c r="H31" s="6"/>
+      <c r="I31" s="6"/>
+      <c r="J31" s="6"/>
+      <c r="K31" s="6"/>
+      <c r="L31" s="6"/>
+      <c r="M31" s="6"/>
+      <c r="N31" s="6"/>
+      <c r="O31" s="6"/>
+      <c r="P31" s="6"/>
+      <c r="Q31" s="6"/>
+      <c r="R31" s="6"/>
+      <c r="S31" s="6"/>
+      <c r="T31" s="6"/>
+      <c r="U31" s="6"/>
       <c r="V31" s="34"/>
       <c r="W31" s="34"/>
       <c r="X31" s="34"/>
@@ -2509,91 +2517,242 @@
       <c r="AF31" s="34"/>
       <c r="AG31" s="35"/>
     </row>
-    <row r="32" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A32" s="27"/>
-      <c r="B32" s="28"/>
-      <c r="C32" s="28"/>
-      <c r="D32" s="28"/>
-      <c r="E32" s="28"/>
-      <c r="F32" s="28"/>
-      <c r="G32" s="28"/>
-      <c r="H32" s="28"/>
-      <c r="I32" s="28"/>
-      <c r="J32" s="28"/>
-      <c r="K32" s="28"/>
-      <c r="L32" s="28"/>
-      <c r="M32" s="28"/>
-      <c r="N32" s="28"/>
-      <c r="O32" s="28"/>
-      <c r="P32" s="28"/>
-      <c r="Q32" s="28"/>
-      <c r="R32" s="28"/>
-      <c r="S32" s="28"/>
-      <c r="T32" s="28"/>
-      <c r="U32" s="28"/>
-      <c r="V32" s="28"/>
-      <c r="W32" s="28"/>
-      <c r="X32" s="28"/>
-      <c r="Y32" s="28"/>
-      <c r="Z32" s="28"/>
-      <c r="AA32" s="28"/>
-      <c r="AB32" s="28"/>
-      <c r="AC32" s="28"/>
-      <c r="AD32" s="28"/>
-      <c r="AE32" s="28"/>
-      <c r="AF32" s="28"/>
-      <c r="AG32" s="29"/>
-    </row>
-    <row r="33" spans="1:33" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="22" t="s">
+    <row r="32" spans="1:33" ht="15">
+      <c r="A32" s="52" t="s">
+        <v>37</v>
+      </c>
+      <c r="B32" s="53"/>
+      <c r="C32" s="53"/>
+      <c r="D32" s="53"/>
+      <c r="E32" s="53"/>
+      <c r="F32" s="53"/>
+      <c r="G32" s="53"/>
+      <c r="H32" s="53"/>
+      <c r="I32" s="53"/>
+      <c r="J32" s="53"/>
+      <c r="K32" s="53"/>
+      <c r="L32" s="53"/>
+      <c r="M32" s="53"/>
+      <c r="N32" s="53"/>
+      <c r="O32" s="53"/>
+      <c r="P32" s="53"/>
+      <c r="Q32" s="53"/>
+      <c r="R32" s="53"/>
+      <c r="S32" s="53"/>
+      <c r="T32" s="53"/>
+      <c r="U32" s="53"/>
+      <c r="V32" s="34"/>
+      <c r="W32" s="34"/>
+      <c r="X32" s="34"/>
+      <c r="Y32" s="34"/>
+      <c r="Z32" s="34"/>
+      <c r="AA32" s="34"/>
+      <c r="AB32" s="34"/>
+      <c r="AC32" s="34"/>
+      <c r="AD32" s="34"/>
+      <c r="AE32" s="34"/>
+      <c r="AF32" s="34"/>
+      <c r="AG32" s="35"/>
+    </row>
+    <row r="33" spans="1:33" ht="15">
+      <c r="A33" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="B33" s="5"/>
+      <c r="C33" s="5"/>
+      <c r="D33" s="5"/>
+      <c r="E33" s="5"/>
+      <c r="F33" s="5"/>
+      <c r="G33" s="5"/>
+      <c r="H33" s="5"/>
+      <c r="I33" s="5"/>
+      <c r="J33" s="5"/>
+      <c r="K33" s="5"/>
+      <c r="L33" s="5"/>
+      <c r="M33" s="5"/>
+      <c r="N33" s="5"/>
+      <c r="O33" s="5"/>
+      <c r="P33" s="5"/>
+      <c r="Q33" s="5"/>
+      <c r="R33" s="5"/>
+      <c r="S33" s="5"/>
+      <c r="T33" s="5"/>
+      <c r="U33" s="5"/>
+      <c r="V33" s="34"/>
+      <c r="W33" s="34"/>
+      <c r="X33" s="34"/>
+      <c r="Y33" s="34"/>
+      <c r="Z33" s="34"/>
+      <c r="AA33" s="34"/>
+      <c r="AB33" s="34"/>
+      <c r="AC33" s="34"/>
+      <c r="AD33" s="34"/>
+      <c r="AE33" s="34"/>
+      <c r="AF33" s="34"/>
+      <c r="AG33" s="35"/>
+    </row>
+    <row r="34" spans="1:33" ht="15">
+      <c r="A34" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="B34" s="1"/>
+      <c r="C34" s="1"/>
+      <c r="D34" s="1"/>
+      <c r="E34" s="1"/>
+      <c r="F34" s="1"/>
+      <c r="G34" s="1"/>
+      <c r="H34" s="1"/>
+      <c r="I34" s="1"/>
+      <c r="J34" s="1"/>
+      <c r="K34" s="1"/>
+      <c r="L34" s="1"/>
+      <c r="M34" s="1"/>
+      <c r="N34" s="1"/>
+      <c r="O34" s="1"/>
+      <c r="P34" s="1"/>
+      <c r="Q34" s="1"/>
+      <c r="R34" s="1"/>
+      <c r="S34" s="1"/>
+      <c r="T34" s="1"/>
+      <c r="U34" s="1"/>
+      <c r="V34" s="34"/>
+      <c r="W34" s="34"/>
+      <c r="X34" s="34"/>
+      <c r="Y34" s="34"/>
+      <c r="Z34" s="34"/>
+      <c r="AA34" s="34"/>
+      <c r="AB34" s="34"/>
+      <c r="AC34" s="34"/>
+      <c r="AD34" s="34"/>
+      <c r="AE34" s="34"/>
+      <c r="AF34" s="34"/>
+      <c r="AG34" s="35"/>
+    </row>
+    <row r="35" spans="1:33" ht="15">
+      <c r="A35" s="19" t="s">
+        <v>30</v>
+      </c>
+      <c r="B35" s="7"/>
+      <c r="C35" s="7"/>
+      <c r="D35" s="7"/>
+      <c r="E35" s="7"/>
+      <c r="F35" s="7"/>
+      <c r="G35" s="7"/>
+      <c r="H35" s="7"/>
+      <c r="I35" s="7"/>
+      <c r="J35" s="7"/>
+      <c r="K35" s="7"/>
+      <c r="L35" s="7"/>
+      <c r="M35" s="7"/>
+      <c r="N35" s="7"/>
+      <c r="O35" s="7"/>
+      <c r="P35" s="7"/>
+      <c r="Q35" s="7"/>
+      <c r="R35" s="7"/>
+      <c r="S35" s="7"/>
+      <c r="T35" s="7"/>
+      <c r="U35" s="7"/>
+      <c r="V35" s="34"/>
+      <c r="W35" s="34"/>
+      <c r="X35" s="34"/>
+      <c r="Y35" s="34"/>
+      <c r="Z35" s="34"/>
+      <c r="AA35" s="34"/>
+      <c r="AB35" s="34"/>
+      <c r="AC35" s="34"/>
+      <c r="AD35" s="34"/>
+      <c r="AE35" s="34"/>
+      <c r="AF35" s="34"/>
+      <c r="AG35" s="35"/>
+    </row>
+    <row r="36" spans="1:33" ht="15">
+      <c r="A36" s="27"/>
+      <c r="B36" s="28"/>
+      <c r="C36" s="28"/>
+      <c r="D36" s="28"/>
+      <c r="E36" s="28"/>
+      <c r="F36" s="28"/>
+      <c r="G36" s="28"/>
+      <c r="H36" s="28"/>
+      <c r="I36" s="28"/>
+      <c r="J36" s="28"/>
+      <c r="K36" s="28"/>
+      <c r="L36" s="28"/>
+      <c r="M36" s="28"/>
+      <c r="N36" s="28"/>
+      <c r="O36" s="28"/>
+      <c r="P36" s="28"/>
+      <c r="Q36" s="28"/>
+      <c r="R36" s="28"/>
+      <c r="S36" s="28"/>
+      <c r="T36" s="28"/>
+      <c r="U36" s="28"/>
+      <c r="V36" s="28"/>
+      <c r="W36" s="28"/>
+      <c r="X36" s="28"/>
+      <c r="Y36" s="28"/>
+      <c r="Z36" s="28"/>
+      <c r="AA36" s="28"/>
+      <c r="AB36" s="28"/>
+      <c r="AC36" s="28"/>
+      <c r="AD36" s="28"/>
+      <c r="AE36" s="28"/>
+      <c r="AF36" s="28"/>
+      <c r="AG36" s="29"/>
+    </row>
+    <row r="37" spans="1:33" ht="15.75" thickBot="1">
+      <c r="A37" s="22" t="s">
         <v>33</v>
       </c>
-      <c r="B33" s="23"/>
-      <c r="C33" s="25"/>
-      <c r="D33" s="25"/>
-      <c r="E33" s="25"/>
-      <c r="F33" s="25"/>
-      <c r="G33" s="25"/>
-      <c r="H33" s="25"/>
-      <c r="I33" s="25"/>
-      <c r="J33" s="25"/>
-      <c r="K33" s="25"/>
-      <c r="L33" s="25"/>
-      <c r="M33" s="25"/>
-      <c r="N33" s="25"/>
-      <c r="O33" s="25"/>
-      <c r="P33" s="25"/>
-      <c r="Q33" s="25"/>
-      <c r="R33" s="25"/>
-      <c r="S33" s="25"/>
-      <c r="T33" s="25"/>
-      <c r="U33" s="25"/>
-      <c r="V33" s="25"/>
-      <c r="W33" s="25"/>
-      <c r="X33" s="25"/>
-      <c r="Y33" s="25"/>
-      <c r="Z33" s="25"/>
-      <c r="AA33" s="25"/>
-      <c r="AB33" s="25"/>
-      <c r="AC33" s="25"/>
-      <c r="AD33" s="25"/>
-      <c r="AE33" s="25"/>
-      <c r="AF33" s="25"/>
-      <c r="AG33" s="26"/>
-    </row>
-    <row r="34" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="N34" s="41"/>
-    </row>
-    <row r="40" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="C40" s="51"/>
+      <c r="B37" s="23"/>
+      <c r="C37" s="25"/>
+      <c r="D37" s="25"/>
+      <c r="E37" s="25"/>
+      <c r="F37" s="25"/>
+      <c r="G37" s="25"/>
+      <c r="H37" s="25"/>
+      <c r="I37" s="25"/>
+      <c r="J37" s="25"/>
+      <c r="K37" s="25"/>
+      <c r="L37" s="25"/>
+      <c r="M37" s="25"/>
+      <c r="N37" s="25"/>
+      <c r="O37" s="25"/>
+      <c r="P37" s="25"/>
+      <c r="Q37" s="25"/>
+      <c r="R37" s="25"/>
+      <c r="S37" s="25"/>
+      <c r="T37" s="25"/>
+      <c r="U37" s="25"/>
+      <c r="V37" s="25"/>
+      <c r="W37" s="25"/>
+      <c r="X37" s="25"/>
+      <c r="Y37" s="25"/>
+      <c r="Z37" s="25"/>
+      <c r="AA37" s="25"/>
+      <c r="AB37" s="25"/>
+      <c r="AC37" s="25"/>
+      <c r="AD37" s="25"/>
+      <c r="AE37" s="25"/>
+      <c r="AF37" s="25"/>
+      <c r="AG37" s="26"/>
+    </row>
+    <row r="38" spans="1:33">
+      <c r="N38" s="41"/>
+    </row>
+    <row r="44" spans="1:33">
+      <c r="C44" s="42"/>
+    </row>
+    <row r="46" spans="1:33">
+      <c r="G46" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A1:XFD1"/>
-    <mergeCell ref="B10:U10"/>
+    <mergeCell ref="B11:U11"/>
     <mergeCell ref="B3:AG3"/>
-    <mergeCell ref="B19:AG19"/>
-    <mergeCell ref="B26:U26"/>
+    <mergeCell ref="B21:AG21"/>
+    <mergeCell ref="B29:U29"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
feat: adiciona suporte ao modelo de 4 componentes (C/O) no processamento, formulários e canvas (#29)
</commit_message>
<xml_diff>
--- a/app/assets/planilhas/teethgram_en.xlsx
+++ b/app/assets/planilhas/teethgram_en.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\almei\dev\teethGram\app\assets\planilhas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{071AEE10-5C9E-46EF-807F-451296B52ACC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{AFFBEBE6-A6BC-498C-A820-BBF450B005CB}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,12 +36,12 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Acer</author>
   </authors>
   <commentList>
-    <comment ref="A5" authorId="0" shapeId="0" xr:uid="{644B7FCF-627E-4E62-A53E-F918F34EE001}">
+    <comment ref="A5" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -56,7 +55,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A6" authorId="0" shapeId="0" xr:uid="{2E440F82-1ED1-4C0A-8C89-CAC623CBBD31}">
+    <comment ref="A7" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -70,7 +69,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A7" authorId="0" shapeId="0" xr:uid="{A4DD2828-35E0-4A5F-9196-F4E1CED96808}">
+    <comment ref="A8" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -84,7 +83,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A8" authorId="0" shapeId="0" xr:uid="{E48B4EB0-D078-4A8C-A169-0ACA2332C515}">
+    <comment ref="A9" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -97,7 +96,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A12" authorId="0" shapeId="0" xr:uid="{4B1F7472-8288-4D18-AEBA-DFFCDEA8A3E2}">
+    <comment ref="A13" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -111,7 +110,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A13" authorId="0" shapeId="0" xr:uid="{5C01E885-706E-4DD4-8899-0996FA7C1E83}">
+    <comment ref="A15" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -125,7 +124,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A14" authorId="0" shapeId="0" xr:uid="{7354F24A-D9B6-400C-9B5C-7188D1761EE6}">
+    <comment ref="A16" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -139,7 +138,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A15" authorId="0" shapeId="0" xr:uid="{E1DBFD74-70CF-4967-8538-81E0FB5B8008}">
+    <comment ref="A17" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -152,7 +151,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A21" authorId="0" shapeId="0" xr:uid="{530DA091-E276-46FF-837E-F2FF425C6DF7}">
+    <comment ref="A23" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -166,7 +165,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A22" authorId="0" shapeId="0" xr:uid="{8D07286F-8727-4357-9417-A22B0C5C0E9E}">
+    <comment ref="A25" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -180,7 +179,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A23" authorId="0" shapeId="0" xr:uid="{AEDD797E-6029-49AB-B684-18BCF2D7ABA1}">
+    <comment ref="A26" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -194,7 +193,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A24" authorId="0" shapeId="0" xr:uid="{0BDDB6FB-1367-41B0-9ECD-1612D5B326D3}">
+    <comment ref="A27" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -207,7 +206,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A28" authorId="0" shapeId="0" xr:uid="{E586BBD3-A76F-47AB-9B09-03CA944C390E}">
+    <comment ref="A31" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -221,7 +220,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A29" authorId="0" shapeId="0" xr:uid="{EAE70C67-A158-42EA-81E3-7ED4E2D2B0F6}">
+    <comment ref="A33" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -235,7 +234,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A30" authorId="0" shapeId="0" xr:uid="{65F162A7-3776-48D5-AF6F-F6BBAD7337E5}">
+    <comment ref="A34" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -249,7 +248,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A31" authorId="0" shapeId="0" xr:uid="{838042A5-64E2-424B-8E3B-22D465E70084}">
+    <comment ref="A35" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -267,7 +266,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="38">
   <si>
     <t>A</t>
   </si>
@@ -375,13 +374,19 @@
   </si>
   <si>
     <t>Fill in the total number of participants affected per dental unit for each component (d, m, f) or for the total (dmft).</t>
+  </si>
+  <si>
+    <t>Decayed/Filled (D/F)</t>
+  </si>
+  <si>
+    <t>decayed/filled (d/f)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -788,7 +793,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -851,6 +856,7 @@
     <xf numFmtId="0" fontId="1" fillId="14" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="14" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -878,7 +884,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1217,15 +1225,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91CAF953-5A63-4D25-9285-6A1D6422454A}">
-  <dimension ref="A1:AG40"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:AG46"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="20.28515625" customWidth="1"/>
+    <col min="1" max="1" width="20.25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" s="42" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="1:33" s="2" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:33" s="43" customFormat="1" ht="15" customHeight="1" thickBot="1"/>
+    <row r="2" spans="1:33" s="2" customFormat="1" ht="15" customHeight="1" thickBot="1">
       <c r="A2" s="9" t="s">
         <v>20</v>
       </c>
@@ -1262,46 +1270,46 @@
       <c r="AF2" s="36"/>
       <c r="AG2" s="37"/>
     </row>
-    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:33">
       <c r="A3" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="45" t="s">
+      <c r="B3" s="46" t="s">
         <v>34</v>
       </c>
-      <c r="C3" s="46"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="46"/>
-      <c r="F3" s="46"/>
-      <c r="G3" s="46"/>
-      <c r="H3" s="46"/>
-      <c r="I3" s="46"/>
-      <c r="J3" s="46"/>
-      <c r="K3" s="46"/>
-      <c r="L3" s="46"/>
-      <c r="M3" s="46"/>
-      <c r="N3" s="46"/>
-      <c r="O3" s="46"/>
-      <c r="P3" s="46"/>
-      <c r="Q3" s="46"/>
-      <c r="R3" s="46"/>
-      <c r="S3" s="46"/>
-      <c r="T3" s="46"/>
-      <c r="U3" s="46"/>
-      <c r="V3" s="46"/>
-      <c r="W3" s="46"/>
-      <c r="X3" s="46"/>
-      <c r="Y3" s="46"/>
-      <c r="Z3" s="46"/>
-      <c r="AA3" s="46"/>
-      <c r="AB3" s="46"/>
-      <c r="AC3" s="46"/>
-      <c r="AD3" s="46"/>
-      <c r="AE3" s="46"/>
-      <c r="AF3" s="46"/>
-      <c r="AG3" s="47"/>
-    </row>
-    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="C3" s="47"/>
+      <c r="D3" s="47"/>
+      <c r="E3" s="47"/>
+      <c r="F3" s="47"/>
+      <c r="G3" s="47"/>
+      <c r="H3" s="47"/>
+      <c r="I3" s="47"/>
+      <c r="J3" s="47"/>
+      <c r="K3" s="47"/>
+      <c r="L3" s="47"/>
+      <c r="M3" s="47"/>
+      <c r="N3" s="47"/>
+      <c r="O3" s="47"/>
+      <c r="P3" s="47"/>
+      <c r="Q3" s="47"/>
+      <c r="R3" s="47"/>
+      <c r="S3" s="47"/>
+      <c r="T3" s="47"/>
+      <c r="U3" s="47"/>
+      <c r="V3" s="47"/>
+      <c r="W3" s="47"/>
+      <c r="X3" s="47"/>
+      <c r="Y3" s="47"/>
+      <c r="Z3" s="47"/>
+      <c r="AA3" s="47"/>
+      <c r="AB3" s="47"/>
+      <c r="AC3" s="47"/>
+      <c r="AD3" s="47"/>
+      <c r="AE3" s="47"/>
+      <c r="AF3" s="47"/>
+      <c r="AG3" s="48"/>
+    </row>
+    <row r="4" spans="1:33" ht="15">
       <c r="A4" s="11" t="s">
         <v>22</v>
       </c>
@@ -1402,7 +1410,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:33" ht="15">
       <c r="A5" s="13" t="s">
         <v>23</v>
       </c>
@@ -1439,329 +1447,329 @@
       <c r="AF5" s="6"/>
       <c r="AG5" s="14"/>
     </row>
-    <row r="6" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A6" s="17" t="s">
+    <row r="6" spans="1:33" ht="15">
+      <c r="A6" s="52" t="s">
+        <v>36</v>
+      </c>
+      <c r="B6" s="53"/>
+      <c r="C6" s="53"/>
+      <c r="D6" s="53"/>
+      <c r="E6" s="53"/>
+      <c r="F6" s="53"/>
+      <c r="G6" s="53"/>
+      <c r="H6" s="53"/>
+      <c r="I6" s="53"/>
+      <c r="J6" s="53"/>
+      <c r="K6" s="53"/>
+      <c r="L6" s="53"/>
+      <c r="M6" s="53"/>
+      <c r="N6" s="53"/>
+      <c r="O6" s="53"/>
+      <c r="P6" s="53"/>
+      <c r="Q6" s="53"/>
+      <c r="R6" s="53"/>
+      <c r="S6" s="53"/>
+      <c r="T6" s="53"/>
+      <c r="U6" s="53"/>
+      <c r="V6" s="53"/>
+      <c r="W6" s="53"/>
+      <c r="X6" s="53"/>
+      <c r="Y6" s="53"/>
+      <c r="Z6" s="53"/>
+      <c r="AA6" s="53"/>
+      <c r="AB6" s="53"/>
+      <c r="AC6" s="53"/>
+      <c r="AD6" s="53"/>
+      <c r="AE6" s="53"/>
+      <c r="AF6" s="53"/>
+      <c r="AG6" s="54"/>
+    </row>
+    <row r="7" spans="1:33" ht="15">
+      <c r="A7" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5"/>
-      <c r="H6" s="5"/>
-      <c r="I6" s="5"/>
-      <c r="J6" s="5"/>
-      <c r="K6" s="5"/>
-      <c r="L6" s="5"/>
-      <c r="M6" s="5"/>
-      <c r="N6" s="5"/>
-      <c r="O6" s="5"/>
-      <c r="P6" s="5"/>
-      <c r="Q6" s="5"/>
-      <c r="R6" s="5"/>
-      <c r="S6" s="5"/>
-      <c r="T6" s="5"/>
-      <c r="U6" s="5"/>
-      <c r="V6" s="5"/>
-      <c r="W6" s="5"/>
-      <c r="X6" s="5"/>
-      <c r="Y6" s="5"/>
-      <c r="Z6" s="5"/>
-      <c r="AA6" s="5"/>
-      <c r="AB6" s="5"/>
-      <c r="AC6" s="5"/>
-      <c r="AD6" s="5"/>
-      <c r="AE6" s="5"/>
-      <c r="AF6" s="5"/>
-      <c r="AG6" s="18"/>
-    </row>
-    <row r="7" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A7" s="15" t="s">
+      <c r="B7" s="5"/>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5"/>
+      <c r="F7" s="5"/>
+      <c r="G7" s="5"/>
+      <c r="H7" s="5"/>
+      <c r="I7" s="5"/>
+      <c r="J7" s="5"/>
+      <c r="K7" s="5"/>
+      <c r="L7" s="5"/>
+      <c r="M7" s="5"/>
+      <c r="N7" s="5"/>
+      <c r="O7" s="5"/>
+      <c r="P7" s="5"/>
+      <c r="Q7" s="5"/>
+      <c r="R7" s="5"/>
+      <c r="S7" s="5"/>
+      <c r="T7" s="5"/>
+      <c r="U7" s="5"/>
+      <c r="V7" s="5"/>
+      <c r="W7" s="5"/>
+      <c r="X7" s="5"/>
+      <c r="Y7" s="5"/>
+      <c r="Z7" s="5"/>
+      <c r="AA7" s="5"/>
+      <c r="AB7" s="5"/>
+      <c r="AC7" s="5"/>
+      <c r="AD7" s="5"/>
+      <c r="AE7" s="5"/>
+      <c r="AF7" s="5"/>
+      <c r="AG7" s="18"/>
+    </row>
+    <row r="8" spans="1:33" ht="15">
+      <c r="A8" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-      <c r="F7" s="1"/>
-      <c r="G7" s="1"/>
-      <c r="H7" s="1"/>
-      <c r="I7" s="1"/>
-      <c r="J7" s="1"/>
-      <c r="K7" s="1"/>
-      <c r="L7" s="1"/>
-      <c r="M7" s="1"/>
-      <c r="N7" s="1"/>
-      <c r="O7" s="1"/>
-      <c r="P7" s="1"/>
-      <c r="Q7" s="1"/>
-      <c r="R7" s="1"/>
-      <c r="S7" s="1"/>
-      <c r="T7" s="1"/>
-      <c r="U7" s="1"/>
-      <c r="V7" s="1"/>
-      <c r="W7" s="1"/>
-      <c r="X7" s="1"/>
-      <c r="Y7" s="1"/>
-      <c r="Z7" s="1"/>
-      <c r="AA7" s="1"/>
-      <c r="AB7" s="1"/>
-      <c r="AC7" s="1"/>
-      <c r="AD7" s="1"/>
-      <c r="AE7" s="1"/>
-      <c r="AF7" s="1"/>
-      <c r="AG7" s="16"/>
-    </row>
-    <row r="8" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A8" s="19" t="s">
+      <c r="B8" s="1"/>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+      <c r="F8" s="1"/>
+      <c r="G8" s="1"/>
+      <c r="H8" s="1"/>
+      <c r="I8" s="1"/>
+      <c r="J8" s="1"/>
+      <c r="K8" s="1"/>
+      <c r="L8" s="1"/>
+      <c r="M8" s="1"/>
+      <c r="N8" s="1"/>
+      <c r="O8" s="1"/>
+      <c r="P8" s="1"/>
+      <c r="Q8" s="1"/>
+      <c r="R8" s="1"/>
+      <c r="S8" s="1"/>
+      <c r="T8" s="1"/>
+      <c r="U8" s="1"/>
+      <c r="V8" s="1"/>
+      <c r="W8" s="1"/>
+      <c r="X8" s="1"/>
+      <c r="Y8" s="1"/>
+      <c r="Z8" s="1"/>
+      <c r="AA8" s="1"/>
+      <c r="AB8" s="1"/>
+      <c r="AC8" s="1"/>
+      <c r="AD8" s="1"/>
+      <c r="AE8" s="1"/>
+      <c r="AF8" s="1"/>
+      <c r="AG8" s="16"/>
+    </row>
+    <row r="9" spans="1:33" ht="15">
+      <c r="A9" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
-      <c r="H8" s="7"/>
-      <c r="I8" s="7"/>
-      <c r="J8" s="7"/>
-      <c r="K8" s="7"/>
-      <c r="L8" s="7"/>
-      <c r="M8" s="7"/>
-      <c r="N8" s="7"/>
-      <c r="O8" s="7"/>
-      <c r="P8" s="7"/>
-      <c r="Q8" s="7"/>
-      <c r="R8" s="7"/>
-      <c r="S8" s="7"/>
-      <c r="T8" s="7"/>
-      <c r="U8" s="7"/>
-      <c r="V8" s="7"/>
-      <c r="W8" s="7"/>
-      <c r="X8" s="7"/>
-      <c r="Y8" s="7"/>
-      <c r="Z8" s="7"/>
-      <c r="AA8" s="7"/>
-      <c r="AB8" s="7"/>
-      <c r="AC8" s="7"/>
-      <c r="AD8" s="7"/>
-      <c r="AE8" s="7"/>
-      <c r="AF8" s="7"/>
-      <c r="AG8" s="20"/>
-    </row>
-    <row r="9" spans="1:33" s="8" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="27"/>
-      <c r="B9" s="28"/>
-      <c r="C9" s="28"/>
-      <c r="D9" s="28"/>
-      <c r="E9" s="28"/>
-      <c r="F9" s="28"/>
-      <c r="G9" s="28"/>
-      <c r="H9" s="28"/>
-      <c r="I9" s="28"/>
-      <c r="J9" s="28"/>
-      <c r="K9" s="28"/>
-      <c r="L9" s="28"/>
-      <c r="M9" s="28"/>
-      <c r="N9" s="28"/>
-      <c r="O9" s="28"/>
-      <c r="P9" s="28"/>
-      <c r="Q9" s="28"/>
-      <c r="R9" s="28"/>
-      <c r="S9" s="28"/>
-      <c r="T9" s="28"/>
-      <c r="U9" s="28"/>
-      <c r="V9" s="28"/>
-      <c r="W9" s="28"/>
-      <c r="X9" s="28"/>
-      <c r="Y9" s="28"/>
-      <c r="Z9" s="28"/>
-      <c r="AA9" s="28"/>
-      <c r="AB9" s="28"/>
-      <c r="AC9" s="28"/>
-      <c r="AD9" s="28"/>
-      <c r="AE9" s="28"/>
-      <c r="AF9" s="28"/>
-      <c r="AG9" s="29"/>
-    </row>
-    <row r="10" spans="1:33" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="21" t="s">
+      <c r="B9" s="7"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="7"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="7"/>
+      <c r="G9" s="7"/>
+      <c r="H9" s="7"/>
+      <c r="I9" s="7"/>
+      <c r="J9" s="7"/>
+      <c r="K9" s="7"/>
+      <c r="L9" s="7"/>
+      <c r="M9" s="7"/>
+      <c r="N9" s="7"/>
+      <c r="O9" s="7"/>
+      <c r="P9" s="7"/>
+      <c r="Q9" s="7"/>
+      <c r="R9" s="7"/>
+      <c r="S9" s="7"/>
+      <c r="T9" s="7"/>
+      <c r="U9" s="7"/>
+      <c r="V9" s="7"/>
+      <c r="W9" s="7"/>
+      <c r="X9" s="7"/>
+      <c r="Y9" s="7"/>
+      <c r="Z9" s="7"/>
+      <c r="AA9" s="7"/>
+      <c r="AB9" s="7"/>
+      <c r="AC9" s="7"/>
+      <c r="AD9" s="7"/>
+      <c r="AE9" s="7"/>
+      <c r="AF9" s="7"/>
+      <c r="AG9" s="20"/>
+    </row>
+    <row r="10" spans="1:33" s="8" customFormat="1" ht="15" customHeight="1">
+      <c r="A10" s="27"/>
+      <c r="B10" s="28"/>
+      <c r="C10" s="28"/>
+      <c r="D10" s="28"/>
+      <c r="E10" s="28"/>
+      <c r="F10" s="28"/>
+      <c r="G10" s="28"/>
+      <c r="H10" s="28"/>
+      <c r="I10" s="28"/>
+      <c r="J10" s="28"/>
+      <c r="K10" s="28"/>
+      <c r="L10" s="28"/>
+      <c r="M10" s="28"/>
+      <c r="N10" s="28"/>
+      <c r="O10" s="28"/>
+      <c r="P10" s="28"/>
+      <c r="Q10" s="28"/>
+      <c r="R10" s="28"/>
+      <c r="S10" s="28"/>
+      <c r="T10" s="28"/>
+      <c r="U10" s="28"/>
+      <c r="V10" s="28"/>
+      <c r="W10" s="28"/>
+      <c r="X10" s="28"/>
+      <c r="Y10" s="28"/>
+      <c r="Z10" s="28"/>
+      <c r="AA10" s="28"/>
+      <c r="AB10" s="28"/>
+      <c r="AC10" s="28"/>
+      <c r="AD10" s="28"/>
+      <c r="AE10" s="28"/>
+      <c r="AF10" s="28"/>
+      <c r="AG10" s="29"/>
+    </row>
+    <row r="11" spans="1:33" s="3" customFormat="1" ht="15">
+      <c r="A11" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="B10" s="43" t="s">
+      <c r="B11" s="44" t="s">
         <v>35</v>
       </c>
-      <c r="C10" s="44"/>
-      <c r="D10" s="44"/>
-      <c r="E10" s="44"/>
-      <c r="F10" s="44"/>
-      <c r="G10" s="44"/>
-      <c r="H10" s="44"/>
-      <c r="I10" s="44"/>
-      <c r="J10" s="44"/>
-      <c r="K10" s="44"/>
-      <c r="L10" s="44"/>
-      <c r="M10" s="44"/>
-      <c r="N10" s="44"/>
-      <c r="O10" s="44"/>
-      <c r="P10" s="44"/>
-      <c r="Q10" s="44"/>
-      <c r="R10" s="44"/>
-      <c r="S10" s="44"/>
-      <c r="T10" s="44"/>
-      <c r="U10" s="44"/>
-      <c r="V10" s="30"/>
-      <c r="W10" s="30"/>
-      <c r="X10" s="30"/>
-      <c r="Y10" s="30"/>
-      <c r="Z10" s="30"/>
-      <c r="AA10" s="30"/>
-      <c r="AB10" s="30"/>
-      <c r="AC10" s="30"/>
-      <c r="AD10" s="30"/>
-      <c r="AE10" s="30"/>
-      <c r="AF10" s="30"/>
-      <c r="AG10" s="31"/>
-    </row>
-    <row r="11" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A11" s="11" t="s">
+      <c r="C11" s="45"/>
+      <c r="D11" s="45"/>
+      <c r="E11" s="45"/>
+      <c r="F11" s="45"/>
+      <c r="G11" s="45"/>
+      <c r="H11" s="45"/>
+      <c r="I11" s="45"/>
+      <c r="J11" s="45"/>
+      <c r="K11" s="45"/>
+      <c r="L11" s="45"/>
+      <c r="M11" s="45"/>
+      <c r="N11" s="45"/>
+      <c r="O11" s="45"/>
+      <c r="P11" s="45"/>
+      <c r="Q11" s="45"/>
+      <c r="R11" s="45"/>
+      <c r="S11" s="45"/>
+      <c r="T11" s="45"/>
+      <c r="U11" s="45"/>
+      <c r="V11" s="30"/>
+      <c r="W11" s="30"/>
+      <c r="X11" s="30"/>
+      <c r="Y11" s="30"/>
+      <c r="Z11" s="30"/>
+      <c r="AA11" s="30"/>
+      <c r="AB11" s="30"/>
+      <c r="AC11" s="30"/>
+      <c r="AD11" s="30"/>
+      <c r="AE11" s="30"/>
+      <c r="AF11" s="30"/>
+      <c r="AG11" s="31"/>
+    </row>
+    <row r="12" spans="1:33" ht="15">
+      <c r="A12" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="B11" s="4">
+      <c r="B12" s="4">
         <v>55</v>
       </c>
-      <c r="C11" s="4">
+      <c r="C12" s="4">
         <v>54</v>
       </c>
-      <c r="D11" s="4">
+      <c r="D12" s="4">
         <v>53</v>
       </c>
-      <c r="E11" s="4">
+      <c r="E12" s="4">
         <v>52</v>
       </c>
-      <c r="F11" s="4">
+      <c r="F12" s="4">
         <v>51</v>
       </c>
-      <c r="G11" s="4">
+      <c r="G12" s="4">
         <v>61</v>
       </c>
-      <c r="H11" s="4">
+      <c r="H12" s="4">
         <v>62</v>
       </c>
-      <c r="I11" s="4">
+      <c r="I12" s="4">
         <v>63</v>
       </c>
-      <c r="J11" s="4">
+      <c r="J12" s="4">
         <v>64</v>
       </c>
-      <c r="K11" s="4">
+      <c r="K12" s="4">
         <v>65</v>
       </c>
-      <c r="L11" s="4">
+      <c r="L12" s="4">
         <v>75</v>
       </c>
-      <c r="M11" s="4">
+      <c r="M12" s="4">
         <v>74</v>
       </c>
-      <c r="N11" s="4">
+      <c r="N12" s="4">
         <v>73</v>
       </c>
-      <c r="O11" s="4">
+      <c r="O12" s="4">
         <v>72</v>
       </c>
-      <c r="P11" s="4">
+      <c r="P12" s="4">
         <v>71</v>
       </c>
-      <c r="Q11" s="4">
+      <c r="Q12" s="4">
         <v>81</v>
       </c>
-      <c r="R11" s="4">
+      <c r="R12" s="4">
         <v>82</v>
       </c>
-      <c r="S11" s="4">
+      <c r="S12" s="4">
         <v>83</v>
       </c>
-      <c r="T11" s="4">
+      <c r="T12" s="4">
         <v>84</v>
       </c>
-      <c r="U11" s="4">
+      <c r="U12" s="4">
         <v>85</v>
       </c>
-      <c r="V11" s="32"/>
-      <c r="W11" s="32"/>
-      <c r="X11" s="32"/>
-      <c r="Y11" s="32"/>
-      <c r="Z11" s="32"/>
-      <c r="AA11" s="32"/>
-      <c r="AB11" s="32"/>
-      <c r="AC11" s="32"/>
-      <c r="AD11" s="32"/>
-      <c r="AE11" s="32"/>
-      <c r="AF11" s="32"/>
-      <c r="AG11" s="33"/>
-    </row>
-    <row r="12" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A12" s="13" t="s">
+      <c r="V12" s="32"/>
+      <c r="W12" s="32"/>
+      <c r="X12" s="32"/>
+      <c r="Y12" s="32"/>
+      <c r="Z12" s="32"/>
+      <c r="AA12" s="32"/>
+      <c r="AB12" s="32"/>
+      <c r="AC12" s="32"/>
+      <c r="AD12" s="32"/>
+      <c r="AE12" s="32"/>
+      <c r="AF12" s="32"/>
+      <c r="AG12" s="33"/>
+    </row>
+    <row r="13" spans="1:33" ht="15">
+      <c r="A13" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="B12" s="6"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
-      <c r="H12" s="6"/>
-      <c r="I12" s="6"/>
-      <c r="J12" s="6"/>
-      <c r="K12" s="6"/>
-      <c r="L12" s="6"/>
-      <c r="M12" s="6"/>
-      <c r="N12" s="6"/>
-      <c r="O12" s="6"/>
-      <c r="P12" s="6"/>
-      <c r="Q12" s="6"/>
-      <c r="R12" s="6"/>
-      <c r="S12" s="6"/>
-      <c r="T12" s="6"/>
-      <c r="U12" s="6"/>
-      <c r="V12" s="34"/>
-      <c r="W12" s="34"/>
-      <c r="X12" s="34"/>
-      <c r="Y12" s="34"/>
-      <c r="Z12" s="34"/>
-      <c r="AA12" s="34"/>
-      <c r="AB12" s="34"/>
-      <c r="AC12" s="34"/>
-      <c r="AD12" s="34"/>
-      <c r="AE12" s="34"/>
-      <c r="AF12" s="34"/>
-      <c r="AG12" s="35"/>
-    </row>
-    <row r="13" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A13" s="17" t="s">
-        <v>29</v>
-      </c>
-      <c r="B13" s="5"/>
-      <c r="C13" s="5"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-      <c r="F13" s="5"/>
-      <c r="G13" s="5"/>
-      <c r="H13" s="5"/>
-      <c r="I13" s="5"/>
-      <c r="J13" s="5"/>
-      <c r="K13" s="5"/>
-      <c r="L13" s="5"/>
-      <c r="M13" s="5"/>
-      <c r="N13" s="5"/>
-      <c r="O13" s="5"/>
-      <c r="P13" s="5"/>
-      <c r="Q13" s="5"/>
-      <c r="R13" s="5"/>
-      <c r="S13" s="5"/>
-      <c r="T13" s="5"/>
-      <c r="U13" s="5"/>
+      <c r="B13" s="6"/>
+      <c r="C13" s="6"/>
+      <c r="D13" s="6"/>
+      <c r="E13" s="6"/>
+      <c r="F13" s="6"/>
+      <c r="G13" s="6"/>
+      <c r="H13" s="6"/>
+      <c r="I13" s="6"/>
+      <c r="J13" s="6"/>
+      <c r="K13" s="6"/>
+      <c r="L13" s="6"/>
+      <c r="M13" s="6"/>
+      <c r="N13" s="6"/>
+      <c r="O13" s="6"/>
+      <c r="P13" s="6"/>
+      <c r="Q13" s="6"/>
+      <c r="R13" s="6"/>
+      <c r="S13" s="6"/>
+      <c r="T13" s="6"/>
+      <c r="U13" s="6"/>
       <c r="V13" s="34"/>
       <c r="W13" s="34"/>
       <c r="X13" s="34"/>
@@ -1775,30 +1783,30 @@
       <c r="AF13" s="34"/>
       <c r="AG13" s="35"/>
     </row>
-    <row r="14" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A14" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
-      <c r="F14" s="1"/>
-      <c r="G14" s="1"/>
-      <c r="H14" s="1"/>
-      <c r="I14" s="1"/>
-      <c r="J14" s="1"/>
-      <c r="K14" s="1"/>
-      <c r="L14" s="1"/>
-      <c r="M14" s="1"/>
-      <c r="N14" s="1"/>
-      <c r="O14" s="1"/>
-      <c r="P14" s="1"/>
-      <c r="Q14" s="1"/>
-      <c r="R14" s="1"/>
-      <c r="S14" s="1"/>
-      <c r="T14" s="1"/>
-      <c r="U14" s="1"/>
+    <row r="14" spans="1:33" ht="15">
+      <c r="A14" s="52" t="s">
+        <v>37</v>
+      </c>
+      <c r="B14" s="53"/>
+      <c r="C14" s="53"/>
+      <c r="D14" s="53"/>
+      <c r="E14" s="53"/>
+      <c r="F14" s="53"/>
+      <c r="G14" s="53"/>
+      <c r="H14" s="53"/>
+      <c r="I14" s="53"/>
+      <c r="J14" s="53"/>
+      <c r="K14" s="53"/>
+      <c r="L14" s="53"/>
+      <c r="M14" s="53"/>
+      <c r="N14" s="53"/>
+      <c r="O14" s="53"/>
+      <c r="P14" s="53"/>
+      <c r="Q14" s="53"/>
+      <c r="R14" s="53"/>
+      <c r="S14" s="53"/>
+      <c r="T14" s="53"/>
+      <c r="U14" s="53"/>
       <c r="V14" s="34"/>
       <c r="W14" s="34"/>
       <c r="X14" s="34"/>
@@ -1812,30 +1820,30 @@
       <c r="AF14" s="34"/>
       <c r="AG14" s="35"/>
     </row>
-    <row r="15" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A15" s="19" t="s">
-        <v>30</v>
-      </c>
-      <c r="B15" s="7"/>
-      <c r="C15" s="7"/>
-      <c r="D15" s="7"/>
-      <c r="E15" s="7"/>
-      <c r="F15" s="7"/>
-      <c r="G15" s="7"/>
-      <c r="H15" s="7"/>
-      <c r="I15" s="7"/>
-      <c r="J15" s="7"/>
-      <c r="K15" s="7"/>
-      <c r="L15" s="7"/>
-      <c r="M15" s="7"/>
-      <c r="N15" s="7"/>
-      <c r="O15" s="7"/>
-      <c r="P15" s="7"/>
-      <c r="Q15" s="7"/>
-      <c r="R15" s="7"/>
-      <c r="S15" s="7"/>
-      <c r="T15" s="7"/>
-      <c r="U15" s="7"/>
+    <row r="15" spans="1:33" ht="15">
+      <c r="A15" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" s="5"/>
+      <c r="C15" s="5"/>
+      <c r="D15" s="5"/>
+      <c r="E15" s="5"/>
+      <c r="F15" s="5"/>
+      <c r="G15" s="5"/>
+      <c r="H15" s="5"/>
+      <c r="I15" s="5"/>
+      <c r="J15" s="5"/>
+      <c r="K15" s="5"/>
+      <c r="L15" s="5"/>
+      <c r="M15" s="5"/>
+      <c r="N15" s="5"/>
+      <c r="O15" s="5"/>
+      <c r="P15" s="5"/>
+      <c r="Q15" s="5"/>
+      <c r="R15" s="5"/>
+      <c r="S15" s="5"/>
+      <c r="T15" s="5"/>
+      <c r="U15" s="5"/>
       <c r="V15" s="34"/>
       <c r="W15" s="34"/>
       <c r="X15" s="34"/>
@@ -1849,653 +1857,653 @@
       <c r="AF15" s="34"/>
       <c r="AG15" s="35"/>
     </row>
-    <row r="16" spans="1:33" s="8" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="38"/>
-      <c r="B16" s="39"/>
-      <c r="C16" s="39"/>
-      <c r="D16" s="39"/>
-      <c r="E16" s="39"/>
-      <c r="F16" s="39"/>
-      <c r="G16" s="39"/>
-      <c r="H16" s="39"/>
-      <c r="I16" s="39"/>
-      <c r="J16" s="39"/>
-      <c r="K16" s="39"/>
-      <c r="L16" s="39"/>
-      <c r="M16" s="39"/>
-      <c r="N16" s="39"/>
-      <c r="O16" s="39"/>
-      <c r="P16" s="39"/>
-      <c r="Q16" s="39"/>
-      <c r="R16" s="39"/>
-      <c r="S16" s="39"/>
-      <c r="T16" s="39"/>
-      <c r="U16" s="39"/>
-      <c r="V16" s="39"/>
-      <c r="W16" s="39"/>
-      <c r="X16" s="39"/>
-      <c r="Y16" s="39"/>
-      <c r="Z16" s="39"/>
-      <c r="AA16" s="39"/>
-      <c r="AB16" s="39"/>
-      <c r="AC16" s="39"/>
-      <c r="AD16" s="39"/>
-      <c r="AE16" s="39"/>
-      <c r="AF16" s="39"/>
-      <c r="AG16" s="40"/>
-    </row>
-    <row r="17" spans="1:33" s="24" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="18" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A18" s="9" t="s">
+    <row r="16" spans="1:33" ht="15">
+      <c r="A16" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="B16" s="1"/>
+      <c r="C16" s="1"/>
+      <c r="D16" s="1"/>
+      <c r="E16" s="1"/>
+      <c r="F16" s="1"/>
+      <c r="G16" s="1"/>
+      <c r="H16" s="1"/>
+      <c r="I16" s="1"/>
+      <c r="J16" s="1"/>
+      <c r="K16" s="1"/>
+      <c r="L16" s="1"/>
+      <c r="M16" s="1"/>
+      <c r="N16" s="1"/>
+      <c r="O16" s="1"/>
+      <c r="P16" s="1"/>
+      <c r="Q16" s="1"/>
+      <c r="R16" s="1"/>
+      <c r="S16" s="1"/>
+      <c r="T16" s="1"/>
+      <c r="U16" s="1"/>
+      <c r="V16" s="34"/>
+      <c r="W16" s="34"/>
+      <c r="X16" s="34"/>
+      <c r="Y16" s="34"/>
+      <c r="Z16" s="34"/>
+      <c r="AA16" s="34"/>
+      <c r="AB16" s="34"/>
+      <c r="AC16" s="34"/>
+      <c r="AD16" s="34"/>
+      <c r="AE16" s="34"/>
+      <c r="AF16" s="34"/>
+      <c r="AG16" s="35"/>
+    </row>
+    <row r="17" spans="1:33" ht="15">
+      <c r="A17" s="19" t="s">
+        <v>30</v>
+      </c>
+      <c r="B17" s="7"/>
+      <c r="C17" s="7"/>
+      <c r="D17" s="7"/>
+      <c r="E17" s="7"/>
+      <c r="F17" s="7"/>
+      <c r="G17" s="7"/>
+      <c r="H17" s="7"/>
+      <c r="I17" s="7"/>
+      <c r="J17" s="7"/>
+      <c r="K17" s="7"/>
+      <c r="L17" s="7"/>
+      <c r="M17" s="7"/>
+      <c r="N17" s="7"/>
+      <c r="O17" s="7"/>
+      <c r="P17" s="7"/>
+      <c r="Q17" s="7"/>
+      <c r="R17" s="7"/>
+      <c r="S17" s="7"/>
+      <c r="T17" s="7"/>
+      <c r="U17" s="7"/>
+      <c r="V17" s="34"/>
+      <c r="W17" s="34"/>
+      <c r="X17" s="34"/>
+      <c r="Y17" s="34"/>
+      <c r="Z17" s="34"/>
+      <c r="AA17" s="34"/>
+      <c r="AB17" s="34"/>
+      <c r="AC17" s="34"/>
+      <c r="AD17" s="34"/>
+      <c r="AE17" s="34"/>
+      <c r="AF17" s="34"/>
+      <c r="AG17" s="35"/>
+    </row>
+    <row r="18" spans="1:33" s="8" customFormat="1" ht="15" customHeight="1" thickBot="1">
+      <c r="A18" s="38"/>
+      <c r="B18" s="39"/>
+      <c r="C18" s="39"/>
+      <c r="D18" s="39"/>
+      <c r="E18" s="39"/>
+      <c r="F18" s="39"/>
+      <c r="G18" s="39"/>
+      <c r="H18" s="39"/>
+      <c r="I18" s="39"/>
+      <c r="J18" s="39"/>
+      <c r="K18" s="39"/>
+      <c r="L18" s="39"/>
+      <c r="M18" s="39"/>
+      <c r="N18" s="39"/>
+      <c r="O18" s="39"/>
+      <c r="P18" s="39"/>
+      <c r="Q18" s="39"/>
+      <c r="R18" s="39"/>
+      <c r="S18" s="39"/>
+      <c r="T18" s="39"/>
+      <c r="U18" s="39"/>
+      <c r="V18" s="39"/>
+      <c r="W18" s="39"/>
+      <c r="X18" s="39"/>
+      <c r="Y18" s="39"/>
+      <c r="Z18" s="39"/>
+      <c r="AA18" s="39"/>
+      <c r="AB18" s="39"/>
+      <c r="AC18" s="39"/>
+      <c r="AD18" s="39"/>
+      <c r="AE18" s="39"/>
+      <c r="AF18" s="39"/>
+      <c r="AG18" s="40"/>
+    </row>
+    <row r="19" spans="1:33" s="24" customFormat="1" ht="15" thickBot="1"/>
+    <row r="20" spans="1:33" ht="15">
+      <c r="A20" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="B18" s="36"/>
-      <c r="C18" s="36"/>
-      <c r="D18" s="36"/>
-      <c r="E18" s="36"/>
-      <c r="F18" s="36"/>
-      <c r="G18" s="36"/>
-      <c r="H18" s="36"/>
-      <c r="I18" s="36"/>
-      <c r="J18" s="36"/>
-      <c r="K18" s="36"/>
-      <c r="L18" s="36"/>
-      <c r="M18" s="36"/>
-      <c r="N18" s="36"/>
-      <c r="O18" s="36"/>
-      <c r="P18" s="36"/>
-      <c r="Q18" s="36"/>
-      <c r="R18" s="36"/>
-      <c r="S18" s="36"/>
-      <c r="T18" s="36"/>
-      <c r="U18" s="36"/>
-      <c r="V18" s="36"/>
-      <c r="W18" s="36"/>
-      <c r="X18" s="36"/>
-      <c r="Y18" s="36"/>
-      <c r="Z18" s="36"/>
-      <c r="AA18" s="36"/>
-      <c r="AB18" s="36"/>
-      <c r="AC18" s="36"/>
-      <c r="AD18" s="36"/>
-      <c r="AE18" s="36"/>
-      <c r="AF18" s="36"/>
-      <c r="AG18" s="37"/>
-    </row>
-    <row r="19" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A19" s="10" t="s">
+      <c r="B20" s="36"/>
+      <c r="C20" s="36"/>
+      <c r="D20" s="36"/>
+      <c r="E20" s="36"/>
+      <c r="F20" s="36"/>
+      <c r="G20" s="36"/>
+      <c r="H20" s="36"/>
+      <c r="I20" s="36"/>
+      <c r="J20" s="36"/>
+      <c r="K20" s="36"/>
+      <c r="L20" s="36"/>
+      <c r="M20" s="36"/>
+      <c r="N20" s="36"/>
+      <c r="O20" s="36"/>
+      <c r="P20" s="36"/>
+      <c r="Q20" s="36"/>
+      <c r="R20" s="36"/>
+      <c r="S20" s="36"/>
+      <c r="T20" s="36"/>
+      <c r="U20" s="36"/>
+      <c r="V20" s="36"/>
+      <c r="W20" s="36"/>
+      <c r="X20" s="36"/>
+      <c r="Y20" s="36"/>
+      <c r="Z20" s="36"/>
+      <c r="AA20" s="36"/>
+      <c r="AB20" s="36"/>
+      <c r="AC20" s="36"/>
+      <c r="AD20" s="36"/>
+      <c r="AE20" s="36"/>
+      <c r="AF20" s="36"/>
+      <c r="AG20" s="37"/>
+    </row>
+    <row r="21" spans="1:33">
+      <c r="A21" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="B19" s="48" t="s">
+      <c r="B21" s="49" t="s">
         <v>34</v>
       </c>
-      <c r="C19" s="49"/>
-      <c r="D19" s="49"/>
-      <c r="E19" s="49"/>
-      <c r="F19" s="49"/>
-      <c r="G19" s="49"/>
-      <c r="H19" s="49"/>
-      <c r="I19" s="49"/>
-      <c r="J19" s="49"/>
-      <c r="K19" s="49"/>
-      <c r="L19" s="49"/>
-      <c r="M19" s="49"/>
-      <c r="N19" s="49"/>
-      <c r="O19" s="49"/>
-      <c r="P19" s="49"/>
-      <c r="Q19" s="49"/>
-      <c r="R19" s="49"/>
-      <c r="S19" s="49"/>
-      <c r="T19" s="49"/>
-      <c r="U19" s="49"/>
-      <c r="V19" s="49"/>
-      <c r="W19" s="49"/>
-      <c r="X19" s="49"/>
-      <c r="Y19" s="49"/>
-      <c r="Z19" s="49"/>
-      <c r="AA19" s="49"/>
-      <c r="AB19" s="49"/>
-      <c r="AC19" s="49"/>
-      <c r="AD19" s="49"/>
-      <c r="AE19" s="49"/>
-      <c r="AF19" s="49"/>
-      <c r="AG19" s="50"/>
-    </row>
-    <row r="20" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A20" s="11" t="s">
+      <c r="C21" s="50"/>
+      <c r="D21" s="50"/>
+      <c r="E21" s="50"/>
+      <c r="F21" s="50"/>
+      <c r="G21" s="50"/>
+      <c r="H21" s="50"/>
+      <c r="I21" s="50"/>
+      <c r="J21" s="50"/>
+      <c r="K21" s="50"/>
+      <c r="L21" s="50"/>
+      <c r="M21" s="50"/>
+      <c r="N21" s="50"/>
+      <c r="O21" s="50"/>
+      <c r="P21" s="50"/>
+      <c r="Q21" s="50"/>
+      <c r="R21" s="50"/>
+      <c r="S21" s="50"/>
+      <c r="T21" s="50"/>
+      <c r="U21" s="50"/>
+      <c r="V21" s="50"/>
+      <c r="W21" s="50"/>
+      <c r="X21" s="50"/>
+      <c r="Y21" s="50"/>
+      <c r="Z21" s="50"/>
+      <c r="AA21" s="50"/>
+      <c r="AB21" s="50"/>
+      <c r="AC21" s="50"/>
+      <c r="AD21" s="50"/>
+      <c r="AE21" s="50"/>
+      <c r="AF21" s="50"/>
+      <c r="AG21" s="51"/>
+    </row>
+    <row r="22" spans="1:33" ht="15">
+      <c r="A22" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="B20" s="4">
+      <c r="B22" s="4">
         <v>1</v>
       </c>
-      <c r="C20" s="4">
+      <c r="C22" s="4">
         <v>2</v>
       </c>
-      <c r="D20" s="4">
+      <c r="D22" s="4">
         <v>3</v>
       </c>
-      <c r="E20" s="4">
+      <c r="E22" s="4">
         <v>4</v>
       </c>
-      <c r="F20" s="4">
+      <c r="F22" s="4">
         <v>5</v>
       </c>
-      <c r="G20" s="4">
+      <c r="G22" s="4">
         <v>6</v>
       </c>
-      <c r="H20" s="4">
+      <c r="H22" s="4">
         <v>7</v>
       </c>
-      <c r="I20" s="4">
+      <c r="I22" s="4">
         <v>8</v>
       </c>
-      <c r="J20" s="4">
+      <c r="J22" s="4">
         <v>9</v>
       </c>
-      <c r="K20" s="4">
+      <c r="K22" s="4">
         <v>10</v>
       </c>
-      <c r="L20" s="4">
+      <c r="L22" s="4">
         <v>11</v>
       </c>
-      <c r="M20" s="4">
+      <c r="M22" s="4">
         <v>12</v>
       </c>
-      <c r="N20" s="4">
+      <c r="N22" s="4">
         <v>13</v>
       </c>
-      <c r="O20" s="4">
+      <c r="O22" s="4">
         <v>14</v>
       </c>
-      <c r="P20" s="4">
+      <c r="P22" s="4">
         <v>15</v>
       </c>
-      <c r="Q20" s="4">
+      <c r="Q22" s="4">
         <v>16</v>
       </c>
-      <c r="R20" s="4">
+      <c r="R22" s="4">
         <v>17</v>
       </c>
-      <c r="S20" s="4">
+      <c r="S22" s="4">
         <v>18</v>
       </c>
-      <c r="T20" s="4">
+      <c r="T22" s="4">
         <v>19</v>
       </c>
-      <c r="U20" s="4">
+      <c r="U22" s="4">
         <v>20</v>
       </c>
-      <c r="V20" s="4">
+      <c r="V22" s="4">
         <v>21</v>
       </c>
-      <c r="W20" s="4">
+      <c r="W22" s="4">
         <v>22</v>
       </c>
-      <c r="X20" s="4">
+      <c r="X22" s="4">
         <v>23</v>
       </c>
-      <c r="Y20" s="4">
+      <c r="Y22" s="4">
         <v>24</v>
       </c>
-      <c r="Z20" s="4">
+      <c r="Z22" s="4">
         <v>25</v>
       </c>
-      <c r="AA20" s="4">
+      <c r="AA22" s="4">
         <v>26</v>
       </c>
-      <c r="AB20" s="4">
+      <c r="AB22" s="4">
         <v>27</v>
       </c>
-      <c r="AC20" s="4">
+      <c r="AC22" s="4">
         <v>28</v>
       </c>
-      <c r="AD20" s="4">
+      <c r="AD22" s="4">
         <v>29</v>
       </c>
-      <c r="AE20" s="4">
+      <c r="AE22" s="4">
         <v>30</v>
       </c>
-      <c r="AF20" s="4">
+      <c r="AF22" s="4">
         <v>31</v>
       </c>
-      <c r="AG20" s="4">
+      <c r="AG22" s="4">
         <v>32</v>
       </c>
     </row>
-    <row r="21" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A21" s="13" t="s">
+    <row r="23" spans="1:33" ht="15">
+      <c r="A23" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="B21" s="6"/>
-      <c r="C21" s="6"/>
-      <c r="D21" s="6"/>
-      <c r="E21" s="6"/>
-      <c r="F21" s="6"/>
-      <c r="G21" s="6"/>
-      <c r="H21" s="6"/>
-      <c r="I21" s="6"/>
-      <c r="J21" s="6"/>
-      <c r="K21" s="6"/>
-      <c r="L21" s="6"/>
-      <c r="M21" s="6"/>
-      <c r="N21" s="6"/>
-      <c r="O21" s="6"/>
-      <c r="P21" s="6"/>
-      <c r="Q21" s="6"/>
-      <c r="R21" s="6"/>
-      <c r="S21" s="6"/>
-      <c r="T21" s="6"/>
-      <c r="U21" s="6"/>
-      <c r="V21" s="6"/>
-      <c r="W21" s="6"/>
-      <c r="X21" s="6"/>
-      <c r="Y21" s="6"/>
-      <c r="Z21" s="6"/>
-      <c r="AA21" s="6"/>
-      <c r="AB21" s="6"/>
-      <c r="AC21" s="6"/>
-      <c r="AD21" s="6"/>
-      <c r="AE21" s="6"/>
-      <c r="AF21" s="6"/>
-      <c r="AG21" s="14"/>
-    </row>
-    <row r="22" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A22" s="17" t="s">
+      <c r="B23" s="6"/>
+      <c r="C23" s="6"/>
+      <c r="D23" s="6"/>
+      <c r="E23" s="6"/>
+      <c r="F23" s="6"/>
+      <c r="G23" s="6"/>
+      <c r="H23" s="6"/>
+      <c r="I23" s="6"/>
+      <c r="J23" s="6"/>
+      <c r="K23" s="6"/>
+      <c r="L23" s="6"/>
+      <c r="M23" s="6"/>
+      <c r="N23" s="6"/>
+      <c r="O23" s="6"/>
+      <c r="P23" s="6"/>
+      <c r="Q23" s="6"/>
+      <c r="R23" s="6"/>
+      <c r="S23" s="6"/>
+      <c r="T23" s="6"/>
+      <c r="U23" s="6"/>
+      <c r="V23" s="6"/>
+      <c r="W23" s="6"/>
+      <c r="X23" s="6"/>
+      <c r="Y23" s="6"/>
+      <c r="Z23" s="6"/>
+      <c r="AA23" s="6"/>
+      <c r="AB23" s="6"/>
+      <c r="AC23" s="6"/>
+      <c r="AD23" s="6"/>
+      <c r="AE23" s="6"/>
+      <c r="AF23" s="6"/>
+      <c r="AG23" s="14"/>
+    </row>
+    <row r="24" spans="1:33" ht="15">
+      <c r="A24" s="52" t="s">
+        <v>36</v>
+      </c>
+      <c r="B24" s="53"/>
+      <c r="C24" s="53"/>
+      <c r="D24" s="53"/>
+      <c r="E24" s="53"/>
+      <c r="F24" s="53"/>
+      <c r="G24" s="53"/>
+      <c r="H24" s="53"/>
+      <c r="I24" s="53"/>
+      <c r="J24" s="53"/>
+      <c r="K24" s="53"/>
+      <c r="L24" s="53"/>
+      <c r="M24" s="53"/>
+      <c r="N24" s="53"/>
+      <c r="O24" s="53"/>
+      <c r="P24" s="53"/>
+      <c r="Q24" s="53"/>
+      <c r="R24" s="53"/>
+      <c r="S24" s="53"/>
+      <c r="T24" s="53"/>
+      <c r="U24" s="53"/>
+      <c r="V24" s="53"/>
+      <c r="W24" s="53"/>
+      <c r="X24" s="53"/>
+      <c r="Y24" s="53"/>
+      <c r="Z24" s="53"/>
+      <c r="AA24" s="53"/>
+      <c r="AB24" s="53"/>
+      <c r="AC24" s="53"/>
+      <c r="AD24" s="53"/>
+      <c r="AE24" s="53"/>
+      <c r="AF24" s="53"/>
+      <c r="AG24" s="54"/>
+    </row>
+    <row r="25" spans="1:33" ht="15">
+      <c r="A25" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="B22" s="5"/>
-      <c r="C22" s="5"/>
-      <c r="D22" s="5"/>
-      <c r="E22" s="5"/>
-      <c r="F22" s="5"/>
-      <c r="G22" s="5"/>
-      <c r="H22" s="5"/>
-      <c r="I22" s="5"/>
-      <c r="J22" s="5"/>
-      <c r="K22" s="5"/>
-      <c r="L22" s="5"/>
-      <c r="M22" s="5"/>
-      <c r="N22" s="5"/>
-      <c r="O22" s="5"/>
-      <c r="P22" s="5"/>
-      <c r="Q22" s="5"/>
-      <c r="R22" s="5"/>
-      <c r="S22" s="5"/>
-      <c r="T22" s="5"/>
-      <c r="U22" s="5"/>
-      <c r="V22" s="5"/>
-      <c r="W22" s="5"/>
-      <c r="X22" s="5"/>
-      <c r="Y22" s="5"/>
-      <c r="Z22" s="5"/>
-      <c r="AA22" s="5"/>
-      <c r="AB22" s="5"/>
-      <c r="AC22" s="5"/>
-      <c r="AD22" s="5"/>
-      <c r="AE22" s="5"/>
-      <c r="AF22" s="5"/>
-      <c r="AG22" s="18"/>
-    </row>
-    <row r="23" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A23" s="15" t="s">
+      <c r="B25" s="5"/>
+      <c r="C25" s="5"/>
+      <c r="D25" s="5"/>
+      <c r="E25" s="5"/>
+      <c r="F25" s="5"/>
+      <c r="G25" s="5"/>
+      <c r="H25" s="5"/>
+      <c r="I25" s="5"/>
+      <c r="J25" s="5"/>
+      <c r="K25" s="5"/>
+      <c r="L25" s="5"/>
+      <c r="M25" s="5"/>
+      <c r="N25" s="5"/>
+      <c r="O25" s="5"/>
+      <c r="P25" s="5"/>
+      <c r="Q25" s="5"/>
+      <c r="R25" s="5"/>
+      <c r="S25" s="5"/>
+      <c r="T25" s="5"/>
+      <c r="U25" s="5"/>
+      <c r="V25" s="5"/>
+      <c r="W25" s="5"/>
+      <c r="X25" s="5"/>
+      <c r="Y25" s="5"/>
+      <c r="Z25" s="5"/>
+      <c r="AA25" s="5"/>
+      <c r="AB25" s="5"/>
+      <c r="AC25" s="5"/>
+      <c r="AD25" s="5"/>
+      <c r="AE25" s="5"/>
+      <c r="AF25" s="5"/>
+      <c r="AG25" s="18"/>
+    </row>
+    <row r="26" spans="1:33" ht="15">
+      <c r="A26" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B23" s="1"/>
-      <c r="C23" s="1"/>
-      <c r="D23" s="1"/>
-      <c r="E23" s="1"/>
-      <c r="F23" s="1"/>
-      <c r="G23" s="1"/>
-      <c r="H23" s="1"/>
-      <c r="I23" s="1"/>
-      <c r="J23" s="1"/>
-      <c r="K23" s="1"/>
-      <c r="L23" s="1"/>
-      <c r="M23" s="1"/>
-      <c r="N23" s="1"/>
-      <c r="O23" s="1"/>
-      <c r="P23" s="1"/>
-      <c r="Q23" s="1"/>
-      <c r="R23" s="1"/>
-      <c r="S23" s="1"/>
-      <c r="T23" s="1"/>
-      <c r="U23" s="1"/>
-      <c r="V23" s="1"/>
-      <c r="W23" s="1"/>
-      <c r="X23" s="1"/>
-      <c r="Y23" s="1"/>
-      <c r="Z23" s="1"/>
-      <c r="AA23" s="1"/>
-      <c r="AB23" s="1"/>
-      <c r="AC23" s="1"/>
-      <c r="AD23" s="1"/>
-      <c r="AE23" s="1"/>
-      <c r="AF23" s="1"/>
-      <c r="AG23" s="16"/>
-    </row>
-    <row r="24" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A24" s="19" t="s">
+      <c r="B26" s="1"/>
+      <c r="C26" s="1"/>
+      <c r="D26" s="1"/>
+      <c r="E26" s="1"/>
+      <c r="F26" s="1"/>
+      <c r="G26" s="1"/>
+      <c r="H26" s="1"/>
+      <c r="I26" s="1"/>
+      <c r="J26" s="1"/>
+      <c r="K26" s="1"/>
+      <c r="L26" s="1"/>
+      <c r="M26" s="1"/>
+      <c r="N26" s="1"/>
+      <c r="O26" s="1"/>
+      <c r="P26" s="1"/>
+      <c r="Q26" s="1"/>
+      <c r="R26" s="1"/>
+      <c r="S26" s="1"/>
+      <c r="T26" s="1"/>
+      <c r="U26" s="1"/>
+      <c r="V26" s="1"/>
+      <c r="W26" s="1"/>
+      <c r="X26" s="1"/>
+      <c r="Y26" s="1"/>
+      <c r="Z26" s="1"/>
+      <c r="AA26" s="1"/>
+      <c r="AB26" s="1"/>
+      <c r="AC26" s="1"/>
+      <c r="AD26" s="1"/>
+      <c r="AE26" s="1"/>
+      <c r="AF26" s="1"/>
+      <c r="AG26" s="16"/>
+    </row>
+    <row r="27" spans="1:33" ht="15">
+      <c r="A27" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="B24" s="7"/>
-      <c r="C24" s="7"/>
-      <c r="D24" s="7"/>
-      <c r="E24" s="7"/>
-      <c r="F24" s="7"/>
-      <c r="G24" s="7"/>
-      <c r="H24" s="7"/>
-      <c r="I24" s="7"/>
-      <c r="J24" s="7"/>
-      <c r="K24" s="7"/>
-      <c r="L24" s="7"/>
-      <c r="M24" s="7"/>
-      <c r="N24" s="7"/>
-      <c r="O24" s="7"/>
-      <c r="P24" s="7"/>
-      <c r="Q24" s="7"/>
-      <c r="R24" s="7"/>
-      <c r="S24" s="7"/>
-      <c r="T24" s="7"/>
-      <c r="U24" s="7"/>
-      <c r="V24" s="7"/>
-      <c r="W24" s="7"/>
-      <c r="X24" s="7"/>
-      <c r="Y24" s="7"/>
-      <c r="Z24" s="7"/>
-      <c r="AA24" s="7"/>
-      <c r="AB24" s="7"/>
-      <c r="AC24" s="7"/>
-      <c r="AD24" s="7"/>
-      <c r="AE24" s="7"/>
-      <c r="AF24" s="7"/>
-      <c r="AG24" s="20"/>
-    </row>
-    <row r="25" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A25" s="27"/>
-      <c r="B25" s="28"/>
-      <c r="C25" s="28"/>
-      <c r="D25" s="28"/>
-      <c r="E25" s="28"/>
-      <c r="F25" s="28"/>
-      <c r="G25" s="28"/>
-      <c r="H25" s="28"/>
-      <c r="I25" s="28"/>
-      <c r="J25" s="28"/>
-      <c r="K25" s="28"/>
-      <c r="L25" s="28"/>
-      <c r="M25" s="28"/>
-      <c r="N25" s="28"/>
-      <c r="O25" s="28"/>
-      <c r="P25" s="28"/>
-      <c r="Q25" s="28"/>
-      <c r="R25" s="28"/>
-      <c r="S25" s="28"/>
-      <c r="T25" s="28"/>
-      <c r="U25" s="28"/>
-      <c r="V25" s="28"/>
-      <c r="W25" s="28"/>
-      <c r="X25" s="28"/>
-      <c r="Y25" s="28"/>
-      <c r="Z25" s="28"/>
-      <c r="AA25" s="28"/>
-      <c r="AB25" s="28"/>
-      <c r="AC25" s="28"/>
-      <c r="AD25" s="28"/>
-      <c r="AE25" s="28"/>
-      <c r="AF25" s="28"/>
-      <c r="AG25" s="29"/>
-    </row>
-    <row r="26" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A26" s="21" t="s">
+      <c r="B27" s="7"/>
+      <c r="C27" s="7"/>
+      <c r="D27" s="7"/>
+      <c r="E27" s="7"/>
+      <c r="F27" s="7"/>
+      <c r="G27" s="7"/>
+      <c r="H27" s="7"/>
+      <c r="I27" s="7"/>
+      <c r="J27" s="7"/>
+      <c r="K27" s="7"/>
+      <c r="L27" s="7"/>
+      <c r="M27" s="7"/>
+      <c r="N27" s="7"/>
+      <c r="O27" s="7"/>
+      <c r="P27" s="7"/>
+      <c r="Q27" s="7"/>
+      <c r="R27" s="7"/>
+      <c r="S27" s="7"/>
+      <c r="T27" s="7"/>
+      <c r="U27" s="7"/>
+      <c r="V27" s="7"/>
+      <c r="W27" s="7"/>
+      <c r="X27" s="7"/>
+      <c r="Y27" s="7"/>
+      <c r="Z27" s="7"/>
+      <c r="AA27" s="7"/>
+      <c r="AB27" s="7"/>
+      <c r="AC27" s="7"/>
+      <c r="AD27" s="7"/>
+      <c r="AE27" s="7"/>
+      <c r="AF27" s="7"/>
+      <c r="AG27" s="20"/>
+    </row>
+    <row r="28" spans="1:33" ht="15">
+      <c r="A28" s="27"/>
+      <c r="B28" s="28"/>
+      <c r="C28" s="28"/>
+      <c r="D28" s="28"/>
+      <c r="E28" s="28"/>
+      <c r="F28" s="28"/>
+      <c r="G28" s="28"/>
+      <c r="H28" s="28"/>
+      <c r="I28" s="28"/>
+      <c r="J28" s="28"/>
+      <c r="K28" s="28"/>
+      <c r="L28" s="28"/>
+      <c r="M28" s="28"/>
+      <c r="N28" s="28"/>
+      <c r="O28" s="28"/>
+      <c r="P28" s="28"/>
+      <c r="Q28" s="28"/>
+      <c r="R28" s="28"/>
+      <c r="S28" s="28"/>
+      <c r="T28" s="28"/>
+      <c r="U28" s="28"/>
+      <c r="V28" s="28"/>
+      <c r="W28" s="28"/>
+      <c r="X28" s="28"/>
+      <c r="Y28" s="28"/>
+      <c r="Z28" s="28"/>
+      <c r="AA28" s="28"/>
+      <c r="AB28" s="28"/>
+      <c r="AC28" s="28"/>
+      <c r="AD28" s="28"/>
+      <c r="AE28" s="28"/>
+      <c r="AF28" s="28"/>
+      <c r="AG28" s="29"/>
+    </row>
+    <row r="29" spans="1:33" ht="15">
+      <c r="A29" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="B26" s="43" t="s">
+      <c r="B29" s="44" t="s">
         <v>35</v>
       </c>
-      <c r="C26" s="44"/>
-      <c r="D26" s="44"/>
-      <c r="E26" s="44"/>
-      <c r="F26" s="44"/>
-      <c r="G26" s="44"/>
-      <c r="H26" s="44"/>
-      <c r="I26" s="44"/>
-      <c r="J26" s="44"/>
-      <c r="K26" s="44"/>
-      <c r="L26" s="44"/>
-      <c r="M26" s="44"/>
-      <c r="N26" s="44"/>
-      <c r="O26" s="44"/>
-      <c r="P26" s="44"/>
-      <c r="Q26" s="44"/>
-      <c r="R26" s="44"/>
-      <c r="S26" s="44"/>
-      <c r="T26" s="44"/>
-      <c r="U26" s="44"/>
-      <c r="V26" s="30"/>
-      <c r="W26" s="30"/>
-      <c r="X26" s="30"/>
-      <c r="Y26" s="30"/>
-      <c r="Z26" s="30"/>
-      <c r="AA26" s="30"/>
-      <c r="AB26" s="30"/>
-      <c r="AC26" s="30"/>
-      <c r="AD26" s="30"/>
-      <c r="AE26" s="30"/>
-      <c r="AF26" s="30"/>
-      <c r="AG26" s="31"/>
-    </row>
-    <row r="27" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A27" s="11" t="s">
+      <c r="C29" s="45"/>
+      <c r="D29" s="45"/>
+      <c r="E29" s="45"/>
+      <c r="F29" s="45"/>
+      <c r="G29" s="45"/>
+      <c r="H29" s="45"/>
+      <c r="I29" s="45"/>
+      <c r="J29" s="45"/>
+      <c r="K29" s="45"/>
+      <c r="L29" s="45"/>
+      <c r="M29" s="45"/>
+      <c r="N29" s="45"/>
+      <c r="O29" s="45"/>
+      <c r="P29" s="45"/>
+      <c r="Q29" s="45"/>
+      <c r="R29" s="45"/>
+      <c r="S29" s="45"/>
+      <c r="T29" s="45"/>
+      <c r="U29" s="45"/>
+      <c r="V29" s="30"/>
+      <c r="W29" s="30"/>
+      <c r="X29" s="30"/>
+      <c r="Y29" s="30"/>
+      <c r="Z29" s="30"/>
+      <c r="AA29" s="30"/>
+      <c r="AB29" s="30"/>
+      <c r="AC29" s="30"/>
+      <c r="AD29" s="30"/>
+      <c r="AE29" s="30"/>
+      <c r="AF29" s="30"/>
+      <c r="AG29" s="31"/>
+    </row>
+    <row r="30" spans="1:33" ht="15">
+      <c r="A30" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="B27" s="4" t="s">
+      <c r="B30" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="C27" s="4" t="s">
+      <c r="C30" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D27" s="4" t="s">
+      <c r="D30" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="E27" s="4" t="s">
+      <c r="E30" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F27" s="4" t="s">
+      <c r="F30" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G27" s="4" t="s">
+      <c r="G30" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="H27" s="4" t="s">
+      <c r="H30" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="I27" s="4" t="s">
+      <c r="I30" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="J27" s="4" t="s">
+      <c r="J30" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="K27" s="4" t="s">
+      <c r="K30" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="L27" s="4" t="s">
+      <c r="L30" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="M27" s="4" t="s">
+      <c r="M30" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="N27" s="4" t="s">
+      <c r="N30" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="O27" s="4" t="s">
+      <c r="O30" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="P27" s="4" t="s">
+      <c r="P30" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="Q27" s="4" t="s">
+      <c r="Q30" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="R27" s="4" t="s">
+      <c r="R30" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="S27" s="4" t="s">
+      <c r="S30" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="T27" s="4" t="s">
+      <c r="T30" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="U27" s="4" t="s">
+      <c r="U30" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="V27" s="32"/>
-      <c r="W27" s="32"/>
-      <c r="X27" s="32"/>
-      <c r="Y27" s="32"/>
-      <c r="Z27" s="32"/>
-      <c r="AA27" s="32"/>
-      <c r="AB27" s="32"/>
-      <c r="AC27" s="32"/>
-      <c r="AD27" s="32"/>
-      <c r="AE27" s="32"/>
-      <c r="AF27" s="32"/>
-      <c r="AG27" s="33"/>
-    </row>
-    <row r="28" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A28" s="13" t="s">
+      <c r="V30" s="32"/>
+      <c r="W30" s="32"/>
+      <c r="X30" s="32"/>
+      <c r="Y30" s="32"/>
+      <c r="Z30" s="32"/>
+      <c r="AA30" s="32"/>
+      <c r="AB30" s="32"/>
+      <c r="AC30" s="32"/>
+      <c r="AD30" s="32"/>
+      <c r="AE30" s="32"/>
+      <c r="AF30" s="32"/>
+      <c r="AG30" s="33"/>
+    </row>
+    <row r="31" spans="1:33" ht="15">
+      <c r="A31" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="6"/>
-      <c r="C28" s="6"/>
-      <c r="D28" s="6"/>
-      <c r="E28" s="6"/>
-      <c r="F28" s="6"/>
-      <c r="G28" s="6"/>
-      <c r="H28" s="6"/>
-      <c r="I28" s="6"/>
-      <c r="J28" s="6"/>
-      <c r="K28" s="6"/>
-      <c r="L28" s="6"/>
-      <c r="M28" s="6"/>
-      <c r="N28" s="6"/>
-      <c r="O28" s="6"/>
-      <c r="P28" s="6"/>
-      <c r="Q28" s="6"/>
-      <c r="R28" s="6"/>
-      <c r="S28" s="6"/>
-      <c r="T28" s="6"/>
-      <c r="U28" s="6"/>
-      <c r="V28" s="34"/>
-      <c r="W28" s="34"/>
-      <c r="X28" s="34"/>
-      <c r="Y28" s="34"/>
-      <c r="Z28" s="34"/>
-      <c r="AA28" s="34"/>
-      <c r="AB28" s="34"/>
-      <c r="AC28" s="34"/>
-      <c r="AD28" s="34"/>
-      <c r="AE28" s="34"/>
-      <c r="AF28" s="34"/>
-      <c r="AG28" s="35"/>
-    </row>
-    <row r="29" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A29" s="17" t="s">
-        <v>29</v>
-      </c>
-      <c r="B29" s="5"/>
-      <c r="C29" s="5"/>
-      <c r="D29" s="5"/>
-      <c r="E29" s="5"/>
-      <c r="F29" s="5"/>
-      <c r="G29" s="5"/>
-      <c r="H29" s="5"/>
-      <c r="I29" s="5"/>
-      <c r="J29" s="5"/>
-      <c r="K29" s="5"/>
-      <c r="L29" s="5"/>
-      <c r="M29" s="5"/>
-      <c r="N29" s="5"/>
-      <c r="O29" s="5"/>
-      <c r="P29" s="5"/>
-      <c r="Q29" s="5"/>
-      <c r="R29" s="5"/>
-      <c r="S29" s="5"/>
-      <c r="T29" s="5"/>
-      <c r="U29" s="5"/>
-      <c r="V29" s="34"/>
-      <c r="W29" s="34"/>
-      <c r="X29" s="34"/>
-      <c r="Y29" s="34"/>
-      <c r="Z29" s="34"/>
-      <c r="AA29" s="34"/>
-      <c r="AB29" s="34"/>
-      <c r="AC29" s="34"/>
-      <c r="AD29" s="34"/>
-      <c r="AE29" s="34"/>
-      <c r="AF29" s="34"/>
-      <c r="AG29" s="35"/>
-    </row>
-    <row r="30" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A30" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="B30" s="1"/>
-      <c r="C30" s="1"/>
-      <c r="D30" s="1"/>
-      <c r="E30" s="1"/>
-      <c r="F30" s="1"/>
-      <c r="G30" s="1"/>
-      <c r="H30" s="1"/>
-      <c r="I30" s="1"/>
-      <c r="J30" s="1"/>
-      <c r="K30" s="1"/>
-      <c r="L30" s="1"/>
-      <c r="M30" s="1"/>
-      <c r="N30" s="1"/>
-      <c r="O30" s="1"/>
-      <c r="P30" s="1"/>
-      <c r="Q30" s="1"/>
-      <c r="R30" s="1"/>
-      <c r="S30" s="1"/>
-      <c r="T30" s="1"/>
-      <c r="U30" s="1"/>
-      <c r="V30" s="34"/>
-      <c r="W30" s="34"/>
-      <c r="X30" s="34"/>
-      <c r="Y30" s="34"/>
-      <c r="Z30" s="34"/>
-      <c r="AA30" s="34"/>
-      <c r="AB30" s="34"/>
-      <c r="AC30" s="34"/>
-      <c r="AD30" s="34"/>
-      <c r="AE30" s="34"/>
-      <c r="AF30" s="34"/>
-      <c r="AG30" s="35"/>
-    </row>
-    <row r="31" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A31" s="19" t="s">
-        <v>30</v>
-      </c>
-      <c r="B31" s="7"/>
-      <c r="C31" s="7"/>
-      <c r="D31" s="7"/>
-      <c r="E31" s="7"/>
-      <c r="F31" s="7"/>
-      <c r="G31" s="7"/>
-      <c r="H31" s="7"/>
-      <c r="I31" s="7"/>
-      <c r="J31" s="7"/>
-      <c r="K31" s="7"/>
-      <c r="L31" s="7"/>
-      <c r="M31" s="7"/>
-      <c r="N31" s="7"/>
-      <c r="O31" s="7"/>
-      <c r="P31" s="7"/>
-      <c r="Q31" s="7"/>
-      <c r="R31" s="7"/>
-      <c r="S31" s="7"/>
-      <c r="T31" s="7"/>
-      <c r="U31" s="7"/>
+      <c r="B31" s="6"/>
+      <c r="C31" s="6"/>
+      <c r="D31" s="6"/>
+      <c r="E31" s="6"/>
+      <c r="F31" s="6"/>
+      <c r="G31" s="6"/>
+      <c r="H31" s="6"/>
+      <c r="I31" s="6"/>
+      <c r="J31" s="6"/>
+      <c r="K31" s="6"/>
+      <c r="L31" s="6"/>
+      <c r="M31" s="6"/>
+      <c r="N31" s="6"/>
+      <c r="O31" s="6"/>
+      <c r="P31" s="6"/>
+      <c r="Q31" s="6"/>
+      <c r="R31" s="6"/>
+      <c r="S31" s="6"/>
+      <c r="T31" s="6"/>
+      <c r="U31" s="6"/>
       <c r="V31" s="34"/>
       <c r="W31" s="34"/>
       <c r="X31" s="34"/>
@@ -2509,91 +2517,242 @@
       <c r="AF31" s="34"/>
       <c r="AG31" s="35"/>
     </row>
-    <row r="32" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A32" s="27"/>
-      <c r="B32" s="28"/>
-      <c r="C32" s="28"/>
-      <c r="D32" s="28"/>
-      <c r="E32" s="28"/>
-      <c r="F32" s="28"/>
-      <c r="G32" s="28"/>
-      <c r="H32" s="28"/>
-      <c r="I32" s="28"/>
-      <c r="J32" s="28"/>
-      <c r="K32" s="28"/>
-      <c r="L32" s="28"/>
-      <c r="M32" s="28"/>
-      <c r="N32" s="28"/>
-      <c r="O32" s="28"/>
-      <c r="P32" s="28"/>
-      <c r="Q32" s="28"/>
-      <c r="R32" s="28"/>
-      <c r="S32" s="28"/>
-      <c r="T32" s="28"/>
-      <c r="U32" s="28"/>
-      <c r="V32" s="28"/>
-      <c r="W32" s="28"/>
-      <c r="X32" s="28"/>
-      <c r="Y32" s="28"/>
-      <c r="Z32" s="28"/>
-      <c r="AA32" s="28"/>
-      <c r="AB32" s="28"/>
-      <c r="AC32" s="28"/>
-      <c r="AD32" s="28"/>
-      <c r="AE32" s="28"/>
-      <c r="AF32" s="28"/>
-      <c r="AG32" s="29"/>
-    </row>
-    <row r="33" spans="1:33" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="22" t="s">
+    <row r="32" spans="1:33" ht="15">
+      <c r="A32" s="52" t="s">
+        <v>37</v>
+      </c>
+      <c r="B32" s="53"/>
+      <c r="C32" s="53"/>
+      <c r="D32" s="53"/>
+      <c r="E32" s="53"/>
+      <c r="F32" s="53"/>
+      <c r="G32" s="53"/>
+      <c r="H32" s="53"/>
+      <c r="I32" s="53"/>
+      <c r="J32" s="53"/>
+      <c r="K32" s="53"/>
+      <c r="L32" s="53"/>
+      <c r="M32" s="53"/>
+      <c r="N32" s="53"/>
+      <c r="O32" s="53"/>
+      <c r="P32" s="53"/>
+      <c r="Q32" s="53"/>
+      <c r="R32" s="53"/>
+      <c r="S32" s="53"/>
+      <c r="T32" s="53"/>
+      <c r="U32" s="53"/>
+      <c r="V32" s="34"/>
+      <c r="W32" s="34"/>
+      <c r="X32" s="34"/>
+      <c r="Y32" s="34"/>
+      <c r="Z32" s="34"/>
+      <c r="AA32" s="34"/>
+      <c r="AB32" s="34"/>
+      <c r="AC32" s="34"/>
+      <c r="AD32" s="34"/>
+      <c r="AE32" s="34"/>
+      <c r="AF32" s="34"/>
+      <c r="AG32" s="35"/>
+    </row>
+    <row r="33" spans="1:33" ht="15">
+      <c r="A33" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="B33" s="5"/>
+      <c r="C33" s="5"/>
+      <c r="D33" s="5"/>
+      <c r="E33" s="5"/>
+      <c r="F33" s="5"/>
+      <c r="G33" s="5"/>
+      <c r="H33" s="5"/>
+      <c r="I33" s="5"/>
+      <c r="J33" s="5"/>
+      <c r="K33" s="5"/>
+      <c r="L33" s="5"/>
+      <c r="M33" s="5"/>
+      <c r="N33" s="5"/>
+      <c r="O33" s="5"/>
+      <c r="P33" s="5"/>
+      <c r="Q33" s="5"/>
+      <c r="R33" s="5"/>
+      <c r="S33" s="5"/>
+      <c r="T33" s="5"/>
+      <c r="U33" s="5"/>
+      <c r="V33" s="34"/>
+      <c r="W33" s="34"/>
+      <c r="X33" s="34"/>
+      <c r="Y33" s="34"/>
+      <c r="Z33" s="34"/>
+      <c r="AA33" s="34"/>
+      <c r="AB33" s="34"/>
+      <c r="AC33" s="34"/>
+      <c r="AD33" s="34"/>
+      <c r="AE33" s="34"/>
+      <c r="AF33" s="34"/>
+      <c r="AG33" s="35"/>
+    </row>
+    <row r="34" spans="1:33" ht="15">
+      <c r="A34" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="B34" s="1"/>
+      <c r="C34" s="1"/>
+      <c r="D34" s="1"/>
+      <c r="E34" s="1"/>
+      <c r="F34" s="1"/>
+      <c r="G34" s="1"/>
+      <c r="H34" s="1"/>
+      <c r="I34" s="1"/>
+      <c r="J34" s="1"/>
+      <c r="K34" s="1"/>
+      <c r="L34" s="1"/>
+      <c r="M34" s="1"/>
+      <c r="N34" s="1"/>
+      <c r="O34" s="1"/>
+      <c r="P34" s="1"/>
+      <c r="Q34" s="1"/>
+      <c r="R34" s="1"/>
+      <c r="S34" s="1"/>
+      <c r="T34" s="1"/>
+      <c r="U34" s="1"/>
+      <c r="V34" s="34"/>
+      <c r="W34" s="34"/>
+      <c r="X34" s="34"/>
+      <c r="Y34" s="34"/>
+      <c r="Z34" s="34"/>
+      <c r="AA34" s="34"/>
+      <c r="AB34" s="34"/>
+      <c r="AC34" s="34"/>
+      <c r="AD34" s="34"/>
+      <c r="AE34" s="34"/>
+      <c r="AF34" s="34"/>
+      <c r="AG34" s="35"/>
+    </row>
+    <row r="35" spans="1:33" ht="15">
+      <c r="A35" s="19" t="s">
+        <v>30</v>
+      </c>
+      <c r="B35" s="7"/>
+      <c r="C35" s="7"/>
+      <c r="D35" s="7"/>
+      <c r="E35" s="7"/>
+      <c r="F35" s="7"/>
+      <c r="G35" s="7"/>
+      <c r="H35" s="7"/>
+      <c r="I35" s="7"/>
+      <c r="J35" s="7"/>
+      <c r="K35" s="7"/>
+      <c r="L35" s="7"/>
+      <c r="M35" s="7"/>
+      <c r="N35" s="7"/>
+      <c r="O35" s="7"/>
+      <c r="P35" s="7"/>
+      <c r="Q35" s="7"/>
+      <c r="R35" s="7"/>
+      <c r="S35" s="7"/>
+      <c r="T35" s="7"/>
+      <c r="U35" s="7"/>
+      <c r="V35" s="34"/>
+      <c r="W35" s="34"/>
+      <c r="X35" s="34"/>
+      <c r="Y35" s="34"/>
+      <c r="Z35" s="34"/>
+      <c r="AA35" s="34"/>
+      <c r="AB35" s="34"/>
+      <c r="AC35" s="34"/>
+      <c r="AD35" s="34"/>
+      <c r="AE35" s="34"/>
+      <c r="AF35" s="34"/>
+      <c r="AG35" s="35"/>
+    </row>
+    <row r="36" spans="1:33" ht="15">
+      <c r="A36" s="27"/>
+      <c r="B36" s="28"/>
+      <c r="C36" s="28"/>
+      <c r="D36" s="28"/>
+      <c r="E36" s="28"/>
+      <c r="F36" s="28"/>
+      <c r="G36" s="28"/>
+      <c r="H36" s="28"/>
+      <c r="I36" s="28"/>
+      <c r="J36" s="28"/>
+      <c r="K36" s="28"/>
+      <c r="L36" s="28"/>
+      <c r="M36" s="28"/>
+      <c r="N36" s="28"/>
+      <c r="O36" s="28"/>
+      <c r="P36" s="28"/>
+      <c r="Q36" s="28"/>
+      <c r="R36" s="28"/>
+      <c r="S36" s="28"/>
+      <c r="T36" s="28"/>
+      <c r="U36" s="28"/>
+      <c r="V36" s="28"/>
+      <c r="W36" s="28"/>
+      <c r="X36" s="28"/>
+      <c r="Y36" s="28"/>
+      <c r="Z36" s="28"/>
+      <c r="AA36" s="28"/>
+      <c r="AB36" s="28"/>
+      <c r="AC36" s="28"/>
+      <c r="AD36" s="28"/>
+      <c r="AE36" s="28"/>
+      <c r="AF36" s="28"/>
+      <c r="AG36" s="29"/>
+    </row>
+    <row r="37" spans="1:33" ht="15.75" thickBot="1">
+      <c r="A37" s="22" t="s">
         <v>33</v>
       </c>
-      <c r="B33" s="23"/>
-      <c r="C33" s="25"/>
-      <c r="D33" s="25"/>
-      <c r="E33" s="25"/>
-      <c r="F33" s="25"/>
-      <c r="G33" s="25"/>
-      <c r="H33" s="25"/>
-      <c r="I33" s="25"/>
-      <c r="J33" s="25"/>
-      <c r="K33" s="25"/>
-      <c r="L33" s="25"/>
-      <c r="M33" s="25"/>
-      <c r="N33" s="25"/>
-      <c r="O33" s="25"/>
-      <c r="P33" s="25"/>
-      <c r="Q33" s="25"/>
-      <c r="R33" s="25"/>
-      <c r="S33" s="25"/>
-      <c r="T33" s="25"/>
-      <c r="U33" s="25"/>
-      <c r="V33" s="25"/>
-      <c r="W33" s="25"/>
-      <c r="X33" s="25"/>
-      <c r="Y33" s="25"/>
-      <c r="Z33" s="25"/>
-      <c r="AA33" s="25"/>
-      <c r="AB33" s="25"/>
-      <c r="AC33" s="25"/>
-      <c r="AD33" s="25"/>
-      <c r="AE33" s="25"/>
-      <c r="AF33" s="25"/>
-      <c r="AG33" s="26"/>
-    </row>
-    <row r="34" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="N34" s="41"/>
-    </row>
-    <row r="40" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="C40" s="51"/>
+      <c r="B37" s="23"/>
+      <c r="C37" s="25"/>
+      <c r="D37" s="25"/>
+      <c r="E37" s="25"/>
+      <c r="F37" s="25"/>
+      <c r="G37" s="25"/>
+      <c r="H37" s="25"/>
+      <c r="I37" s="25"/>
+      <c r="J37" s="25"/>
+      <c r="K37" s="25"/>
+      <c r="L37" s="25"/>
+      <c r="M37" s="25"/>
+      <c r="N37" s="25"/>
+      <c r="O37" s="25"/>
+      <c r="P37" s="25"/>
+      <c r="Q37" s="25"/>
+      <c r="R37" s="25"/>
+      <c r="S37" s="25"/>
+      <c r="T37" s="25"/>
+      <c r="U37" s="25"/>
+      <c r="V37" s="25"/>
+      <c r="W37" s="25"/>
+      <c r="X37" s="25"/>
+      <c r="Y37" s="25"/>
+      <c r="Z37" s="25"/>
+      <c r="AA37" s="25"/>
+      <c r="AB37" s="25"/>
+      <c r="AC37" s="25"/>
+      <c r="AD37" s="25"/>
+      <c r="AE37" s="25"/>
+      <c r="AF37" s="25"/>
+      <c r="AG37" s="26"/>
+    </row>
+    <row r="38" spans="1:33">
+      <c r="N38" s="41"/>
+    </row>
+    <row r="44" spans="1:33">
+      <c r="C44" s="42"/>
+    </row>
+    <row r="46" spans="1:33">
+      <c r="G46" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A1:XFD1"/>
-    <mergeCell ref="B10:U10"/>
+    <mergeCell ref="B11:U11"/>
     <mergeCell ref="B3:AG3"/>
-    <mergeCell ref="B19:AG19"/>
-    <mergeCell ref="B26:U26"/>
+    <mergeCell ref="B21:AG21"/>
+    <mergeCell ref="B29:U29"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>